<commit_message>
Add Christmas morning drinks and mince pies; NYE BBQ replaces fish and chips
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="136">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -227,6 +227,12 @@
     <t xml:space="preserve">Sunday lunch</t>
   </si>
   <si>
+    <t xml:space="preserve">Christmas morning: drinks only, with free mince pies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Year's Eve BBQ instead of fish &amp; chips. Please book.</t>
+  </si>
+  <si>
     <t xml:space="preserve">EXAMPLE (hidden): Christmas Eve hours. Copy this row, change it and set Status to Live.</t>
   </si>
   <si>
@@ -420,6 +426,9 @@
   </si>
   <si>
     <t xml:space="preserve">The 5-5-5 menu: Friday 9 and Saturday 10 October. Please reserve, we get busy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas morning: we're open for drinks, with free mince pies.</t>
   </si>
   <si>
     <t xml:space="preserve">New Year's Eve BBQ: smoked brisket, creamy mac and cheese, burgers and sausages with caramelised onions. Call to book.</t>
@@ -1399,16 +1408,16 @@
         <v>Regular</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6" t="n">
-        <v>0.5</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.625</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
@@ -1418,58 +1427,84 @@
         <v>67</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>46380</v>
+        <v>46381</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>46380</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>46357</v>
-      </c>
+        <v>46381</v>
+      </c>
+      <c r="L9" s="7"/>
       <c r="M9" s="5" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="N9" s="8" t="str">
         <f aca="true">IF(A9&amp;B9&amp;C9&amp;H9&amp;I9="","",IF(M9="Hidden","Hidden",IF(AND(J9&lt;&gt;"",J9&gt;TODAY()),"Scheduled",IF(AND(K9&lt;&gt;"",K9&lt;TODAY()),"Expired",IF(OR(J9&lt;&gt;"",K9&lt;&gt;""),"Special, in effect","Regular")))))</f>
-        <v>Hidden</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
+        <v>Scheduled</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
+      <c r="C10" s="6" t="n">
+        <v>0.708333333333333</v>
+      </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
+      <c r="I10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>46387</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>46387</v>
+      </c>
       <c r="L10" s="7"/>
-      <c r="M10" s="5"/>
+      <c r="M10" s="5" t="s">
+        <v>56</v>
+      </c>
       <c r="N10" s="8" t="str">
         <f aca="true">IF(A10&amp;B10&amp;C10&amp;H10&amp;I10="","",IF(M10="Hidden","Hidden",IF(AND(J10&lt;&gt;"",J10&gt;TODAY()),"Scheduled",IF(AND(K10&lt;&gt;"",K10&lt;TODAY()),"Expired",IF(OR(J10&lt;&gt;"",K10&lt;&gt;""),"Special, in effect","Regular")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
+        <v>Scheduled</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="B11" s="5"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="C11" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.625</v>
+      </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="5"/>
+      <c r="I11" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>46380</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>46380</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>46357</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="N11" s="8" t="str">
         <f aca="true">IF(A11&amp;B11&amp;C11&amp;H11&amp;I11="","",IF(M11="Hidden","Hidden",IF(AND(J11&lt;&gt;"",J11&gt;TODAY()),"Scheduled",IF(AND(K11&lt;&gt;"",K11&lt;TODAY()),"Expired",IF(OR(J11&lt;&gt;"",K11&lt;&gt;""),"Special, in effect","Regular")))))</f>
-        <v/>
+        <v>Hidden</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5122,31 +5157,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>40</v>
@@ -5161,23 +5196,25 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D2" s="9" t="n">
         <v>9.95</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>55</v>
       </c>
       <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
+      <c r="I2" s="7" t="n">
+        <v>46386</v>
+      </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
         <v>56</v>
@@ -5187,57 +5224,59 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D3" s="9"/>
+      <c r="D3" s="9" t="n">
+        <v>9.95</v>
+      </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>46387</v>
-      </c>
+        <v>46388</v>
+      </c>
+      <c r="I3" s="7"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
         <v>56</v>
       </c>
       <c r="L3" s="8" t="str">
         <f aca="true">IF(B3&amp;C3="","",IF(K3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(AND(I3&lt;&gt;"",I3&lt;TODAY()),"Expired","Showing"))))</f>
-        <v>Showing</v>
+        <v>Scheduled</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>14.95</v>
-      </c>
+      <c r="D4" s="9"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
+        <v>82</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>46387</v>
+      </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
         <v>56</v>
@@ -5247,9 +5286,9 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>86</v>
@@ -5258,11 +5297,11 @@
         <v>87</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>13.95</v>
+        <v>14.95</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="7"/>
@@ -5278,7 +5317,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>88</v>
@@ -5291,7 +5330,7 @@
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="7"/>
@@ -5307,7 +5346,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>90</v>
@@ -5320,7 +5359,7 @@
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="7"/>
@@ -5336,18 +5375,20 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="5"/>
+      <c r="C8" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="D8" s="9" t="n">
-        <v>11.95</v>
+        <v>13.95</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="7"/>
@@ -5363,22 +5404,18 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>95</v>
-      </c>
+      <c r="C9" s="5"/>
       <c r="D9" s="9" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>96</v>
-      </c>
+        <v>11.95</v>
+      </c>
+      <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="7"/>
@@ -5392,24 +5429,24 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="9" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="F10" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="7"/>
@@ -5423,18 +5460,24 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="5"/>
       <c r="C11" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="9" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>
@@ -5450,18 +5493,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B12" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="9" t="n">
-        <v>13.95</v>
-      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="9"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
@@ -5477,18 +5518,18 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="9" t="n">
-        <v>14.95</v>
+        <v>13.95</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="7"/>
@@ -5504,18 +5545,18 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="9" t="n">
-        <v>14.5</v>
+        <v>14.95</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="7"/>
@@ -5531,18 +5572,18 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="9" t="n">
-        <v>15.95</v>
+        <v>14.5</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="7"/>
@@ -5558,20 +5599,18 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" s="5" t="s">
         <v>106</v>
       </c>
+      <c r="C16" s="5"/>
       <c r="D16" s="9" t="n">
-        <v>16.95</v>
+        <v>15.95</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="7"/>
@@ -5587,18 +5626,20 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="5"/>
       <c r="D17" s="9" t="n">
-        <v>5.95</v>
+        <v>16.95</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="7"/>
@@ -5614,10 +5655,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9" t="n">
@@ -5625,7 +5666,7 @@
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="7"/>
@@ -5641,10 +5682,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9" t="n">
@@ -5652,7 +5693,7 @@
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="7"/>
@@ -5668,16 +5709,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C20" s="5"/>
-      <c r="D20" s="9"/>
+      <c r="D20" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="7"/>
@@ -5702,7 +5745,7 @@
       <c r="D21" s="9"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
@@ -5721,13 +5764,13 @@
         <v>66</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="9"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
@@ -5746,15 +5789,13 @@
         <v>66</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="9"/>
-      <c r="E23" s="5" t="s">
-        <v>96</v>
-      </c>
+      <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
@@ -5769,20 +5810,30 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
+      <c r="A24" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>117</v>
+      </c>
       <c r="C24" s="5"/>
       <c r="D24" s="9"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
+      <c r="E24" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>114</v>
+      </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
       <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
+      <c r="K24" s="5" t="s">
+        <v>56</v>
+      </c>
       <c r="L24" s="8" t="str">
         <f aca="true">IF(B24&amp;C24="","",IF(K24="Hidden","Hidden",IF(AND(H24&lt;&gt;"",H24&gt;TODAY()),"Scheduled",IF(AND(I24&lt;&gt;"",I24&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8837,25 +8888,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>40</v>
@@ -8869,13 +8920,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="5"/>
@@ -8892,13 +8943,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="5"/>
@@ -8915,13 +8966,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="5"/>
@@ -8938,10 +8989,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="9"/>
@@ -8959,10 +9010,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="9"/>
@@ -8980,10 +9031,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -11942,13 +11993,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>52</v>
@@ -11959,7 +12010,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46304</v>
@@ -11975,15 +12026,15 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>46387</v>
+        <v>46381</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>56</v>
@@ -11993,14 +12044,22 @@
         <v>Scheduled</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="5"/>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>56</v>
+      </c>
       <c r="E4" s="8" t="str">
         <f aca="true">IF(A4="","",IF(D4="Hidden","Hidden",IF(AND(B4&lt;&gt;"",B4&gt;TODAY()),"Scheduled",IF(AND(C4&lt;&gt;"",C4&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Scheduled</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add What's on events (new Events tab) and Walks & rides section
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Menu" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Drinks" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Offers" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Events" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="152">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Anything you add on the Hours, Menu, Drinks and Offers tabs appears on the website on the dates you choose. Nothing needs changing in the website itself.</t>
+    <t xml:space="preserve">Anything you add on the Hours, Menu, Drinks, Offers and Events tabs appears on the website on the dates you choose. Nothing needs changing in the website itself.</t>
   </si>
   <si>
     <t xml:space="preserve">How it works</t>
@@ -116,6 +117,12 @@
     <t xml:space="preserve">Offers is the red banner at the top of the website. Put the whole message in Text. If several offers are live, they all show.</t>
   </si>
   <si>
+    <t xml:space="preserve">Events tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events are the 'What's on' list on the website (BBQs, family fun days, quiz nights...). Give each one a Date (and an End date if it runs over several days). It appears from its Show from date and disappears by itself after the event. Put Yes in Family friendly to give it a family tag.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Note: the 'Showing today?' column looks at dates and Status only. It does not take the Days column into account.</t>
   </si>
   <si>
@@ -131,13 +138,13 @@
     <t xml:space="preserve">1. Upload this file to Google Drive and open it with Google Sheets (File &gt; Import if needed).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. For each tab (Hours, Menu, Drinks, Offers): File &gt; Share &gt; Publish to web &gt; pick that tab &gt; choose 'Comma-separated values (.csv)' &gt; Publish. Copy the link.</t>
+    <t xml:space="preserve">2. For each tab (Hours, Menu, Drinks, Offers, Events): File &gt; Share &gt; Publish to web &gt; pick that tab &gt; choose 'Comma-separated values (.csv)' &gt; Publish. Copy the link.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Paste the four links into config.js on the website (in GitHub), then save. After that, anything you change in the sheet appears on the website within about five minutes.</t>
+    <t xml:space="preserve">3. Paste the five links into config.js on the website (in GitHub), then save. After that, anything you change in the sheet appears on the website within about five minutes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Until then, the website reads the same content from the data folder on GitHub (hours.csv, menu.csv, drinks.csv, offers.csv).</t>
+    <t xml:space="preserve">Until then, the website reads the same content from the data folder on GitHub (hours.csv, menu.csv, drinks.csv, offers.csv, events.csv).</t>
   </si>
   <si>
     <t xml:space="preserve">What's on the sheet now</t>
@@ -432,6 +439,48 @@
   </si>
   <si>
     <t xml:space="preserve">New Year's Eve BBQ: smoked brisket, creamy mac and cheese, burgers and sausages with caramelised onions. Call to book.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Family friendly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE: Summer BBQ in the garden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From 2pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE (hidden): copy this row, change it and set Status to Live. Say what is on the BBQ menu here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking advised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE: Family fun day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 to 5pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE (hidden): bouncy castle in the garden for the little ones. Add ages, prices and anything else families need to know.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Just turn up</t>
   </si>
 </sst>
 </file>
@@ -894,7 +943,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A47"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -1063,62 +1112,72 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2"/>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
-        <v>31</v>
+      <c r="A37" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="A38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2"/>
+      <c r="A39" s="3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>33</v>
+      <c r="A40" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2"/>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
+      <c r="A46" s="2" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1153,51 +1212,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="6"/>
@@ -1206,14 +1265,14 @@
       <c r="F2" s="6"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
       <c r="M2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N2" s="8" t="str">
         <f aca="true">IF(A2&amp;B2&amp;C2&amp;H2&amp;I2="","",IF(M2="Hidden","Hidden",IF(AND(J2&lt;&gt;"",J2&gt;TODAY()),"Scheduled",IF(AND(K2&lt;&gt;"",K2&lt;TODAY()),"Expired",IF(OR(J2&lt;&gt;"",K2&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1222,7 +1281,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="6" t="n">
@@ -1236,13 +1295,13 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
       <c r="M3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N3" s="8" t="str">
         <f aca="true">IF(A3&amp;B3&amp;C3&amp;H3&amp;I3="","",IF(M3="Hidden","Hidden",IF(AND(J3&lt;&gt;"",J3&gt;TODAY()),"Scheduled",IF(AND(K3&lt;&gt;"",K3&lt;TODAY()),"Expired",IF(OR(J3&lt;&gt;"",K3&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1251,7 +1310,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="6" t="n">
@@ -1265,17 +1324,17 @@
         <v>0.833333333333333</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
       <c r="M4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N4" s="8" t="str">
         <f aca="true">IF(A4&amp;B4&amp;C4&amp;H4&amp;I4="","",IF(M4="Hidden","Hidden",IF(AND(J4&lt;&gt;"",J4&gt;TODAY()),"Scheduled",IF(AND(K4&lt;&gt;"",K4&lt;TODAY()),"Expired",IF(OR(J4&lt;&gt;"",K4&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1284,7 +1343,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="n">
@@ -1298,7 +1357,7 @@
         <v>0.833333333333333</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -1306,7 +1365,7 @@
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
       <c r="M5" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N5" s="8" t="str">
         <f aca="true">IF(A5&amp;B5&amp;C5&amp;H5&amp;I5="","",IF(M5="Hidden","Hidden",IF(AND(J5&lt;&gt;"",J5&gt;TODAY()),"Scheduled",IF(AND(K5&lt;&gt;"",K5&lt;TODAY()),"Expired",IF(OR(J5&lt;&gt;"",K5&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1315,7 +1374,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="6" t="n">
@@ -1331,7 +1390,7 @@
         <v>0.833333333333333</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -1339,7 +1398,7 @@
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
       <c r="M6" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N6" s="8" t="str">
         <f aca="true">IF(A6&amp;B6&amp;C6&amp;H6&amp;I6="","",IF(M6="Hidden","Hidden",IF(AND(J6&lt;&gt;"",J6&gt;TODAY()),"Scheduled",IF(AND(K6&lt;&gt;"",K6&lt;TODAY()),"Expired",IF(OR(J6&lt;&gt;"",K6&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1348,7 +1407,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="6" t="n">
@@ -1366,7 +1425,7 @@
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
       <c r="M7" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N7" s="8" t="str">
         <f aca="true">IF(A7&amp;B7&amp;C7&amp;H7&amp;I7="","",IF(M7="Hidden","Hidden",IF(AND(J7&lt;&gt;"",J7&gt;TODAY()),"Scheduled",IF(AND(K7&lt;&gt;"",K7&lt;TODAY()),"Expired",IF(OR(J7&lt;&gt;"",K7&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1375,10 +1434,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>0.5</v>
@@ -1393,7 +1452,7 @@
         <v>0.708333333333333</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -1401,7 +1460,7 @@
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
       <c r="M8" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N8" s="8" t="str">
         <f aca="true">IF(A8&amp;B8&amp;C8&amp;H8&amp;I8="","",IF(M8="Hidden","Hidden",IF(AND(J8&lt;&gt;"",J8&gt;TODAY()),"Scheduled",IF(AND(K8&lt;&gt;"",K8&lt;TODAY()),"Expired",IF(OR(J8&lt;&gt;"",K8&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1410,7 +1469,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6" t="n">
@@ -1424,7 +1483,7 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>46381</v>
@@ -1434,7 +1493,7 @@
       </c>
       <c r="L9" s="7"/>
       <c r="M9" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N9" s="8" t="str">
         <f aca="true">IF(A9&amp;B9&amp;C9&amp;H9&amp;I9="","",IF(M9="Hidden","Hidden",IF(AND(J9&lt;&gt;"",J9&gt;TODAY()),"Scheduled",IF(AND(K9&lt;&gt;"",K9&lt;TODAY()),"Expired",IF(OR(J9&lt;&gt;"",K9&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1443,7 +1502,7 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6" t="n">
@@ -1455,7 +1514,7 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>46387</v>
@@ -1465,7 +1524,7 @@
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N10" s="8" t="str">
         <f aca="true">IF(A10&amp;B10&amp;C10&amp;H10&amp;I10="","",IF(M10="Hidden","Hidden",IF(AND(J10&lt;&gt;"",J10&gt;TODAY()),"Scheduled",IF(AND(K10&lt;&gt;"",K10&lt;TODAY()),"Expired",IF(OR(J10&lt;&gt;"",K10&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -1474,7 +1533,7 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6" t="n">
@@ -1488,7 +1547,7 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>46380</v>
@@ -1500,7 +1559,7 @@
         <v>46357</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N11" s="8" t="str">
         <f aca="true">IF(A11&amp;B11&amp;C11&amp;H11&amp;I11="","",IF(M11="Hidden","Hidden",IF(AND(J11&lt;&gt;"",J11&gt;TODAY()),"Scheduled",IF(AND(K11&lt;&gt;"",K11&lt;TODAY()),"Expired",IF(OR(J11&lt;&gt;"",K11&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -5111,20 +5170,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:L200" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H200" type="list">
+      <formula1>"Yes"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M2:M200" type="list">
       <formula1>"Live,Hidden"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:L200" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B200" type="list">
       <formula1>"1st,2nd,3rd,4th,Last"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H200" type="list">
-      <formula1>"Yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5157,59 +5216,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D2" s="9" t="n">
         <v>9.95</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="7" t="n">
@@ -5217,7 +5276,7 @@
       </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L2" s="8" t="str">
         <f aca="true">IF(B2&amp;C2="","",IF(K2="Hidden","Hidden",IF(AND(H2&lt;&gt;"",H2&gt;TODAY()),"Scheduled",IF(AND(I2&lt;&gt;"",I2&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5227,20 +5286,20 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>9.95</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>46388</v>
@@ -5248,7 +5307,7 @@
       <c r="I3" s="7"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L3" s="8" t="str">
         <f aca="true">IF(B3&amp;C3="","",IF(K3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(AND(I3&lt;&gt;"",I3&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5258,18 +5317,18 @@
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46304</v>
@@ -5279,7 +5338,7 @@
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L4" s="8" t="str">
         <f aca="true">IF(B4&amp;C4="","",IF(K4="Hidden","Hidden",IF(AND(H4&lt;&gt;"",H4&gt;TODAY()),"Scheduled",IF(AND(I4&lt;&gt;"",I4&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5288,27 +5347,27 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>14.95</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L5" s="8" t="str">
         <f aca="true">IF(B5&amp;C5="","",IF(K5="Hidden","Hidden",IF(AND(H5&lt;&gt;"",H5&gt;TODAY()),"Scheduled",IF(AND(I5&lt;&gt;"",I5&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5317,27 +5376,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>13.95</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L6" s="8" t="str">
         <f aca="true">IF(B6&amp;C6="","",IF(K6="Hidden","Hidden",IF(AND(H6&lt;&gt;"",H6&gt;TODAY()),"Scheduled",IF(AND(I6&lt;&gt;"",I6&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5346,27 +5405,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>13.95</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L7" s="8" t="str">
         <f aca="true">IF(B7&amp;C7="","",IF(K7="Hidden","Hidden",IF(AND(H7&lt;&gt;"",H7&gt;TODAY()),"Scheduled",IF(AND(I7&lt;&gt;"",I7&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5375,27 +5434,27 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>13.95</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L8" s="8" t="str">
         <f aca="true">IF(B8&amp;C8="","",IF(K8="Hidden","Hidden",IF(AND(H8&lt;&gt;"",H8&gt;TODAY()),"Scheduled",IF(AND(I8&lt;&gt;"",I8&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5404,10 +5463,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="9" t="n">
@@ -5415,14 +5474,14 @@
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L9" s="8" t="str">
         <f aca="true">IF(B9&amp;C9="","",IF(K9="Hidden","Hidden",IF(AND(H9&lt;&gt;"",H9&gt;TODAY()),"Scheduled",IF(AND(I9&lt;&gt;"",I9&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5431,29 +5490,29 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>10.95</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L10" s="8" t="str">
         <f aca="true">IF(B10&amp;C10="","",IF(K10="Hidden","Hidden",IF(AND(H10&lt;&gt;"",H10&gt;TODAY()),"Scheduled",IF(AND(I10&lt;&gt;"",I10&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5462,29 +5521,29 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>13.95</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L11" s="8" t="str">
         <f aca="true">IF(B11&amp;C11="","",IF(K11="Hidden","Hidden",IF(AND(H11&lt;&gt;"",H11&gt;TODAY()),"Scheduled",IF(AND(I11&lt;&gt;"",I11&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5493,23 +5552,23 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L12" s="8" t="str">
         <f aca="true">IF(B12&amp;C12="","",IF(K12="Hidden","Hidden",IF(AND(H12&lt;&gt;"",H12&gt;TODAY()),"Scheduled",IF(AND(I12&lt;&gt;"",I12&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5518,10 +5577,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="9" t="n">
@@ -5529,14 +5588,14 @@
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L13" s="8" t="str">
         <f aca="true">IF(B13&amp;C13="","",IF(K13="Hidden","Hidden",IF(AND(H13&lt;&gt;"",H13&gt;TODAY()),"Scheduled",IF(AND(I13&lt;&gt;"",I13&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5545,10 +5604,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="9" t="n">
@@ -5556,14 +5615,14 @@
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L14" s="8" t="str">
         <f aca="true">IF(B14&amp;C14="","",IF(K14="Hidden","Hidden",IF(AND(H14&lt;&gt;"",H14&gt;TODAY()),"Scheduled",IF(AND(I14&lt;&gt;"",I14&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5572,10 +5631,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="9" t="n">
@@ -5583,14 +5642,14 @@
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L15" s="8" t="str">
         <f aca="true">IF(B15&amp;C15="","",IF(K15="Hidden","Hidden",IF(AND(H15&lt;&gt;"",H15&gt;TODAY()),"Scheduled",IF(AND(I15&lt;&gt;"",I15&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5599,10 +5658,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="9" t="n">
@@ -5610,14 +5669,14 @@
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="5"/>
       <c r="K16" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L16" s="8" t="str">
         <f aca="true">IF(B16&amp;C16="","",IF(K16="Hidden","Hidden",IF(AND(H16&lt;&gt;"",H16&gt;TODAY()),"Scheduled",IF(AND(I16&lt;&gt;"",I16&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5626,27 +5685,27 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>16.95</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="5"/>
       <c r="K17" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L17" s="8" t="str">
         <f aca="true">IF(B17&amp;C17="","",IF(K17="Hidden","Hidden",IF(AND(H17&lt;&gt;"",H17&gt;TODAY()),"Scheduled",IF(AND(I17&lt;&gt;"",I17&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5655,10 +5714,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9" t="n">
@@ -5666,14 +5725,14 @@
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="5"/>
       <c r="K18" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L18" s="8" t="str">
         <f aca="true">IF(B18&amp;C18="","",IF(K18="Hidden","Hidden",IF(AND(H18&lt;&gt;"",H18&gt;TODAY()),"Scheduled",IF(AND(I18&lt;&gt;"",I18&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5682,10 +5741,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9" t="n">
@@ -5693,14 +5752,14 @@
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L19" s="8" t="str">
         <f aca="true">IF(B19&amp;C19="","",IF(K19="Hidden","Hidden",IF(AND(H19&lt;&gt;"",H19&gt;TODAY()),"Scheduled",IF(AND(I19&lt;&gt;"",I19&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5709,10 +5768,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="9" t="n">
@@ -5720,14 +5779,14 @@
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
       <c r="J20" s="5"/>
       <c r="K20" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L20" s="8" t="str">
         <f aca="true">IF(B20&amp;C20="","",IF(K20="Hidden","Hidden",IF(AND(H20&lt;&gt;"",H20&gt;TODAY()),"Scheduled",IF(AND(I20&lt;&gt;"",I20&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5736,23 +5795,23 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="9"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L21" s="8" t="str">
         <f aca="true">IF(B21&amp;C21="","",IF(K21="Hidden","Hidden",IF(AND(H21&lt;&gt;"",H21&gt;TODAY()),"Scheduled",IF(AND(I21&lt;&gt;"",I21&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5761,23 +5820,23 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="9"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L22" s="8" t="str">
         <f aca="true">IF(B22&amp;C22="","",IF(K22="Hidden","Hidden",IF(AND(H22&lt;&gt;"",H22&gt;TODAY()),"Scheduled",IF(AND(I22&lt;&gt;"",I22&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5786,23 +5845,23 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="9"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L23" s="8" t="str">
         <f aca="true">IF(B23&amp;C23="","",IF(K23="Hidden","Hidden",IF(AND(H23&lt;&gt;"",H23&gt;TODAY()),"Scheduled",IF(AND(I23&lt;&gt;"",I23&lt;TODAY()),"Expired","Showing"))))</f>
@@ -5811,25 +5870,25 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="9"/>
       <c r="E24" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L24" s="8" t="str">
         <f aca="true">IF(B24&amp;C24="","",IF(K24="Hidden","Hidden",IF(AND(H24&lt;&gt;"",H24&gt;TODAY()),"Scheduled",IF(AND(I24&lt;&gt;"",I24&lt;TODAY()),"Expired","Showing"))))</f>
@@ -8841,20 +8900,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K200" type="list">
+      <formula1>"Live,Sold out,Hidden"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I200" type="date">
       <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F200" type="list">
+      <formula1>"Board,Sunday"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G200" type="list">
       <formula1>"Yes"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K200" type="list">
-      <formula1>"Live,Sold out,Hidden"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F200" type="list">
-      <formula1>"Board,Sunday"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -8888,45 +8947,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="5"/>
@@ -8934,7 +8993,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J2" s="8" t="str">
         <f aca="true">IF(B2&amp;C2="","",IF(I2="Hidden","Hidden",IF(AND(F2&lt;&gt;"",F2&gt;TODAY()),"Scheduled",IF(AND(G2&lt;&gt;"",G2&lt;TODAY()),"Expired","Showing"))))</f>
@@ -8943,13 +9002,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="5"/>
@@ -8957,7 +9016,7 @@
       <c r="G3" s="7"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J3" s="8" t="str">
         <f aca="true">IF(B3&amp;C3="","",IF(I3="Hidden","Hidden",IF(AND(F3&lt;&gt;"",F3&gt;TODAY()),"Scheduled",IF(AND(G3&lt;&gt;"",G3&lt;TODAY()),"Expired","Showing"))))</f>
@@ -8966,13 +9025,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="5"/>
@@ -8980,7 +9039,7 @@
       <c r="G4" s="7"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J4" s="8" t="str">
         <f aca="true">IF(B4&amp;C4="","",IF(I4="Hidden","Hidden",IF(AND(F4&lt;&gt;"",F4&gt;TODAY()),"Scheduled",IF(AND(G4&lt;&gt;"",G4&lt;TODAY()),"Expired","Showing"))))</f>
@@ -8989,10 +9048,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="9"/>
@@ -9001,7 +9060,7 @@
       <c r="G5" s="7"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J5" s="8" t="str">
         <f aca="true">IF(B5&amp;C5="","",IF(I5="Hidden","Hidden",IF(AND(F5&lt;&gt;"",F5&gt;TODAY()),"Scheduled",IF(AND(G5&lt;&gt;"",G5&lt;TODAY()),"Expired","Showing"))))</f>
@@ -9010,10 +9069,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="9"/>
@@ -9022,7 +9081,7 @@
       <c r="G6" s="7"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J6" s="8" t="str">
         <f aca="true">IF(B6&amp;C6="","",IF(I6="Hidden","Hidden",IF(AND(F6&lt;&gt;"",F6&gt;TODAY()),"Scheduled",IF(AND(G6&lt;&gt;"",G6&lt;TODAY()),"Expired","Showing"))))</f>
@@ -9031,10 +9090,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -9043,7 +9102,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J7" s="8" t="str">
         <f aca="true">IF(B7&amp;C7="","",IF(I7="Hidden","Hidden",IF(AND(F7&lt;&gt;"",F7&gt;TODAY()),"Scheduled",IF(AND(G7&lt;&gt;"",G7&lt;TODAY()),"Expired","Showing"))))</f>
@@ -11993,24 +12052,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46304</v>
@@ -12019,7 +12078,7 @@
         <v>46305</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E2" s="8" t="str">
         <f aca="true">IF(A2="","",IF(D2="Hidden","Hidden",IF(AND(B2&lt;&gt;"",B2&gt;TODAY()),"Scheduled",IF(AND(C2&lt;&gt;"",C2&lt;TODAY()),"Expired","Showing"))))</f>
@@ -12028,7 +12087,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -12037,7 +12096,7 @@
         <v>46381</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E3" s="8" t="str">
         <f aca="true">IF(A3="","",IF(D3="Hidden","Hidden",IF(AND(B3&lt;&gt;"",B3&gt;TODAY()),"Scheduled",IF(AND(C3&lt;&gt;"",C3&lt;TODAY()),"Expired","Showing"))))</f>
@@ -12046,7 +12105,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46357</v>
@@ -12055,7 +12114,7 @@
         <v>46387</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E4" s="8" t="str">
         <f aca="true">IF(A4="","",IF(D4="Hidden","Hidden",IF(AND(B4&lt;&gt;"",B4&gt;TODAY()),"Scheduled",IF(AND(C4&lt;&gt;"",C4&lt;TODAY()),"Expired","Showing"))))</f>
@@ -14052,4 +14111,3106 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J200"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>46564</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>46508</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="8" t="str">
+        <f aca="true">IF(A2="","",IF(I2="Hidden","Hidden",IF(AND(H2&lt;&gt;"",H2&gt;TODAY()),"Scheduled",IF(IF(C2&lt;&gt;"",C2,B2)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v>Hidden</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>46592</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>46553</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J3" s="8" t="str">
+        <f aca="true">IF(A3="","",IF(I3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(IF(C3&lt;&gt;"",C3,B3)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v>Hidden</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="8" t="str">
+        <f aca="true">IF(A4="","",IF(I4="Hidden","Hidden",IF(AND(H4&lt;&gt;"",H4&gt;TODAY()),"Scheduled",IF(IF(C4&lt;&gt;"",C4,B4)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="8" t="str">
+        <f aca="true">IF(A5="","",IF(I5="Hidden","Hidden",IF(AND(H5&lt;&gt;"",H5&gt;TODAY()),"Scheduled",IF(IF(C5&lt;&gt;"",C5,B5)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="8" t="str">
+        <f aca="true">IF(A6="","",IF(I6="Hidden","Hidden",IF(AND(H6&lt;&gt;"",H6&gt;TODAY()),"Scheduled",IF(IF(C6&lt;&gt;"",C6,B6)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="8" t="str">
+        <f aca="true">IF(A7="","",IF(I7="Hidden","Hidden",IF(AND(H7&lt;&gt;"",H7&gt;TODAY()),"Scheduled",IF(IF(C7&lt;&gt;"",C7,B7)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="8" t="str">
+        <f aca="true">IF(A8="","",IF(I8="Hidden","Hidden",IF(AND(H8&lt;&gt;"",H8&gt;TODAY()),"Scheduled",IF(IF(C8&lt;&gt;"",C8,B8)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="8" t="str">
+        <f aca="true">IF(A9="","",IF(I9="Hidden","Hidden",IF(AND(H9&lt;&gt;"",H9&gt;TODAY()),"Scheduled",IF(IF(C9&lt;&gt;"",C9,B9)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="8" t="str">
+        <f aca="true">IF(A10="","",IF(I10="Hidden","Hidden",IF(AND(H10&lt;&gt;"",H10&gt;TODAY()),"Scheduled",IF(IF(C10&lt;&gt;"",C10,B10)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="8" t="str">
+        <f aca="true">IF(A11="","",IF(I11="Hidden","Hidden",IF(AND(H11&lt;&gt;"",H11&gt;TODAY()),"Scheduled",IF(IF(C11&lt;&gt;"",C11,B11)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="8" t="str">
+        <f aca="true">IF(A12="","",IF(I12="Hidden","Hidden",IF(AND(H12&lt;&gt;"",H12&gt;TODAY()),"Scheduled",IF(IF(C12&lt;&gt;"",C12,B12)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="8" t="str">
+        <f aca="true">IF(A13="","",IF(I13="Hidden","Hidden",IF(AND(H13&lt;&gt;"",H13&gt;TODAY()),"Scheduled",IF(IF(C13&lt;&gt;"",C13,B13)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="8" t="str">
+        <f aca="true">IF(A14="","",IF(I14="Hidden","Hidden",IF(AND(H14&lt;&gt;"",H14&gt;TODAY()),"Scheduled",IF(IF(C14&lt;&gt;"",C14,B14)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="8" t="str">
+        <f aca="true">IF(A15="","",IF(I15="Hidden","Hidden",IF(AND(H15&lt;&gt;"",H15&gt;TODAY()),"Scheduled",IF(IF(C15&lt;&gt;"",C15,B15)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="8" t="str">
+        <f aca="true">IF(A16="","",IF(I16="Hidden","Hidden",IF(AND(H16&lt;&gt;"",H16&gt;TODAY()),"Scheduled",IF(IF(C16&lt;&gt;"",C16,B16)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="8" t="str">
+        <f aca="true">IF(A17="","",IF(I17="Hidden","Hidden",IF(AND(H17&lt;&gt;"",H17&gt;TODAY()),"Scheduled",IF(IF(C17&lt;&gt;"",C17,B17)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="8" t="str">
+        <f aca="true">IF(A18="","",IF(I18="Hidden","Hidden",IF(AND(H18&lt;&gt;"",H18&gt;TODAY()),"Scheduled",IF(IF(C18&lt;&gt;"",C18,B18)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="8" t="str">
+        <f aca="true">IF(A19="","",IF(I19="Hidden","Hidden",IF(AND(H19&lt;&gt;"",H19&gt;TODAY()),"Scheduled",IF(IF(C19&lt;&gt;"",C19,B19)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="8" t="str">
+        <f aca="true">IF(A20="","",IF(I20="Hidden","Hidden",IF(AND(H20&lt;&gt;"",H20&gt;TODAY()),"Scheduled",IF(IF(C20&lt;&gt;"",C20,B20)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="8" t="str">
+        <f aca="true">IF(A21="","",IF(I21="Hidden","Hidden",IF(AND(H21&lt;&gt;"",H21&gt;TODAY()),"Scheduled",IF(IF(C21&lt;&gt;"",C21,B21)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="8" t="str">
+        <f aca="true">IF(A22="","",IF(I22="Hidden","Hidden",IF(AND(H22&lt;&gt;"",H22&gt;TODAY()),"Scheduled",IF(IF(C22&lt;&gt;"",C22,B22)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="8" t="str">
+        <f aca="true">IF(A23="","",IF(I23="Hidden","Hidden",IF(AND(H23&lt;&gt;"",H23&gt;TODAY()),"Scheduled",IF(IF(C23&lt;&gt;"",C23,B23)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="8" t="str">
+        <f aca="true">IF(A24="","",IF(I24="Hidden","Hidden",IF(AND(H24&lt;&gt;"",H24&gt;TODAY()),"Scheduled",IF(IF(C24&lt;&gt;"",C24,B24)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="8" t="str">
+        <f aca="true">IF(A25="","",IF(I25="Hidden","Hidden",IF(AND(H25&lt;&gt;"",H25&gt;TODAY()),"Scheduled",IF(IF(C25&lt;&gt;"",C25,B25)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="8" t="str">
+        <f aca="true">IF(A26="","",IF(I26="Hidden","Hidden",IF(AND(H26&lt;&gt;"",H26&gt;TODAY()),"Scheduled",IF(IF(C26&lt;&gt;"",C26,B26)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="8" t="str">
+        <f aca="true">IF(A27="","",IF(I27="Hidden","Hidden",IF(AND(H27&lt;&gt;"",H27&gt;TODAY()),"Scheduled",IF(IF(C27&lt;&gt;"",C27,B27)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="8" t="str">
+        <f aca="true">IF(A28="","",IF(I28="Hidden","Hidden",IF(AND(H28&lt;&gt;"",H28&gt;TODAY()),"Scheduled",IF(IF(C28&lt;&gt;"",C28,B28)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="8" t="str">
+        <f aca="true">IF(A29="","",IF(I29="Hidden","Hidden",IF(AND(H29&lt;&gt;"",H29&gt;TODAY()),"Scheduled",IF(IF(C29&lt;&gt;"",C29,B29)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="8" t="str">
+        <f aca="true">IF(A30="","",IF(I30="Hidden","Hidden",IF(AND(H30&lt;&gt;"",H30&gt;TODAY()),"Scheduled",IF(IF(C30&lt;&gt;"",C30,B30)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="8" t="str">
+        <f aca="true">IF(A31="","",IF(I31="Hidden","Hidden",IF(AND(H31&lt;&gt;"",H31&gt;TODAY()),"Scheduled",IF(IF(C31&lt;&gt;"",C31,B31)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="8" t="str">
+        <f aca="true">IF(A32="","",IF(I32="Hidden","Hidden",IF(AND(H32&lt;&gt;"",H32&gt;TODAY()),"Scheduled",IF(IF(C32&lt;&gt;"",C32,B32)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="8" t="str">
+        <f aca="true">IF(A33="","",IF(I33="Hidden","Hidden",IF(AND(H33&lt;&gt;"",H33&gt;TODAY()),"Scheduled",IF(IF(C33&lt;&gt;"",C33,B33)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="8" t="str">
+        <f aca="true">IF(A34="","",IF(I34="Hidden","Hidden",IF(AND(H34&lt;&gt;"",H34&gt;TODAY()),"Scheduled",IF(IF(C34&lt;&gt;"",C34,B34)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="8" t="str">
+        <f aca="true">IF(A35="","",IF(I35="Hidden","Hidden",IF(AND(H35&lt;&gt;"",H35&gt;TODAY()),"Scheduled",IF(IF(C35&lt;&gt;"",C35,B35)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="8" t="str">
+        <f aca="true">IF(A36="","",IF(I36="Hidden","Hidden",IF(AND(H36&lt;&gt;"",H36&gt;TODAY()),"Scheduled",IF(IF(C36&lt;&gt;"",C36,B36)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="8" t="str">
+        <f aca="true">IF(A37="","",IF(I37="Hidden","Hidden",IF(AND(H37&lt;&gt;"",H37&gt;TODAY()),"Scheduled",IF(IF(C37&lt;&gt;"",C37,B37)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="8" t="str">
+        <f aca="true">IF(A38="","",IF(I38="Hidden","Hidden",IF(AND(H38&lt;&gt;"",H38&gt;TODAY()),"Scheduled",IF(IF(C38&lt;&gt;"",C38,B38)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="8" t="str">
+        <f aca="true">IF(A39="","",IF(I39="Hidden","Hidden",IF(AND(H39&lt;&gt;"",H39&gt;TODAY()),"Scheduled",IF(IF(C39&lt;&gt;"",C39,B39)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="8" t="str">
+        <f aca="true">IF(A40="","",IF(I40="Hidden","Hidden",IF(AND(H40&lt;&gt;"",H40&gt;TODAY()),"Scheduled",IF(IF(C40&lt;&gt;"",C40,B40)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="8" t="str">
+        <f aca="true">IF(A41="","",IF(I41="Hidden","Hidden",IF(AND(H41&lt;&gt;"",H41&gt;TODAY()),"Scheduled",IF(IF(C41&lt;&gt;"",C41,B41)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="8" t="str">
+        <f aca="true">IF(A42="","",IF(I42="Hidden","Hidden",IF(AND(H42&lt;&gt;"",H42&gt;TODAY()),"Scheduled",IF(IF(C42&lt;&gt;"",C42,B42)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="8" t="str">
+        <f aca="true">IF(A43="","",IF(I43="Hidden","Hidden",IF(AND(H43&lt;&gt;"",H43&gt;TODAY()),"Scheduled",IF(IF(C43&lt;&gt;"",C43,B43)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="8" t="str">
+        <f aca="true">IF(A44="","",IF(I44="Hidden","Hidden",IF(AND(H44&lt;&gt;"",H44&gt;TODAY()),"Scheduled",IF(IF(C44&lt;&gt;"",C44,B44)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="8" t="str">
+        <f aca="true">IF(A45="","",IF(I45="Hidden","Hidden",IF(AND(H45&lt;&gt;"",H45&gt;TODAY()),"Scheduled",IF(IF(C45&lt;&gt;"",C45,B45)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="8" t="str">
+        <f aca="true">IF(A46="","",IF(I46="Hidden","Hidden",IF(AND(H46&lt;&gt;"",H46&gt;TODAY()),"Scheduled",IF(IF(C46&lt;&gt;"",C46,B46)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="8" t="str">
+        <f aca="true">IF(A47="","",IF(I47="Hidden","Hidden",IF(AND(H47&lt;&gt;"",H47&gt;TODAY()),"Scheduled",IF(IF(C47&lt;&gt;"",C47,B47)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="8" t="str">
+        <f aca="true">IF(A48="","",IF(I48="Hidden","Hidden",IF(AND(H48&lt;&gt;"",H48&gt;TODAY()),"Scheduled",IF(IF(C48&lt;&gt;"",C48,B48)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="8" t="str">
+        <f aca="true">IF(A49="","",IF(I49="Hidden","Hidden",IF(AND(H49&lt;&gt;"",H49&gt;TODAY()),"Scheduled",IF(IF(C49&lt;&gt;"",C49,B49)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="8" t="str">
+        <f aca="true">IF(A50="","",IF(I50="Hidden","Hidden",IF(AND(H50&lt;&gt;"",H50&gt;TODAY()),"Scheduled",IF(IF(C50&lt;&gt;"",C50,B50)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="8" t="str">
+        <f aca="true">IF(A51="","",IF(I51="Hidden","Hidden",IF(AND(H51&lt;&gt;"",H51&gt;TODAY()),"Scheduled",IF(IF(C51&lt;&gt;"",C51,B51)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="8" t="str">
+        <f aca="true">IF(A52="","",IF(I52="Hidden","Hidden",IF(AND(H52&lt;&gt;"",H52&gt;TODAY()),"Scheduled",IF(IF(C52&lt;&gt;"",C52,B52)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="8" t="str">
+        <f aca="true">IF(A53="","",IF(I53="Hidden","Hidden",IF(AND(H53&lt;&gt;"",H53&gt;TODAY()),"Scheduled",IF(IF(C53&lt;&gt;"",C53,B53)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="8" t="str">
+        <f aca="true">IF(A54="","",IF(I54="Hidden","Hidden",IF(AND(H54&lt;&gt;"",H54&gt;TODAY()),"Scheduled",IF(IF(C54&lt;&gt;"",C54,B54)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="8" t="str">
+        <f aca="true">IF(A55="","",IF(I55="Hidden","Hidden",IF(AND(H55&lt;&gt;"",H55&gt;TODAY()),"Scheduled",IF(IF(C55&lt;&gt;"",C55,B55)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="8" t="str">
+        <f aca="true">IF(A56="","",IF(I56="Hidden","Hidden",IF(AND(H56&lt;&gt;"",H56&gt;TODAY()),"Scheduled",IF(IF(C56&lt;&gt;"",C56,B56)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="5"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="8" t="str">
+        <f aca="true">IF(A57="","",IF(I57="Hidden","Hidden",IF(AND(H57&lt;&gt;"",H57&gt;TODAY()),"Scheduled",IF(IF(C57&lt;&gt;"",C57,B57)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="8" t="str">
+        <f aca="true">IF(A58="","",IF(I58="Hidden","Hidden",IF(AND(H58&lt;&gt;"",H58&gt;TODAY()),"Scheduled",IF(IF(C58&lt;&gt;"",C58,B58)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="8" t="str">
+        <f aca="true">IF(A59="","",IF(I59="Hidden","Hidden",IF(AND(H59&lt;&gt;"",H59&gt;TODAY()),"Scheduled",IF(IF(C59&lt;&gt;"",C59,B59)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="8" t="str">
+        <f aca="true">IF(A60="","",IF(I60="Hidden","Hidden",IF(AND(H60&lt;&gt;"",H60&gt;TODAY()),"Scheduled",IF(IF(C60&lt;&gt;"",C60,B60)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="5"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="8" t="str">
+        <f aca="true">IF(A61="","",IF(I61="Hidden","Hidden",IF(AND(H61&lt;&gt;"",H61&gt;TODAY()),"Scheduled",IF(IF(C61&lt;&gt;"",C61,B61)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5"/>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="8" t="str">
+        <f aca="true">IF(A62="","",IF(I62="Hidden","Hidden",IF(AND(H62&lt;&gt;"",H62&gt;TODAY()),"Scheduled",IF(IF(C62&lt;&gt;"",C62,B62)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="8" t="str">
+        <f aca="true">IF(A63="","",IF(I63="Hidden","Hidden",IF(AND(H63&lt;&gt;"",H63&gt;TODAY()),"Scheduled",IF(IF(C63&lt;&gt;"",C63,B63)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5"/>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="8" t="str">
+        <f aca="true">IF(A64="","",IF(I64="Hidden","Hidden",IF(AND(H64&lt;&gt;"",H64&gt;TODAY()),"Scheduled",IF(IF(C64&lt;&gt;"",C64,B64)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="5"/>
+      <c r="J65" s="8" t="str">
+        <f aca="true">IF(A65="","",IF(I65="Hidden","Hidden",IF(AND(H65&lt;&gt;"",H65&gt;TODAY()),"Scheduled",IF(IF(C65&lt;&gt;"",C65,B65)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5"/>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="7"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="8" t="str">
+        <f aca="true">IF(A66="","",IF(I66="Hidden","Hidden",IF(AND(H66&lt;&gt;"",H66&gt;TODAY()),"Scheduled",IF(IF(C66&lt;&gt;"",C66,B66)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="8" t="str">
+        <f aca="true">IF(A67="","",IF(I67="Hidden","Hidden",IF(AND(H67&lt;&gt;"",H67&gt;TODAY()),"Scheduled",IF(IF(C67&lt;&gt;"",C67,B67)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5"/>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="7"/>
+      <c r="I68" s="5"/>
+      <c r="J68" s="8" t="str">
+        <f aca="true">IF(A68="","",IF(I68="Hidden","Hidden",IF(AND(H68&lt;&gt;"",H68&gt;TODAY()),"Scheduled",IF(IF(C68&lt;&gt;"",C68,B68)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="7"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="8" t="str">
+        <f aca="true">IF(A69="","",IF(I69="Hidden","Hidden",IF(AND(H69&lt;&gt;"",H69&gt;TODAY()),"Scheduled",IF(IF(C69&lt;&gt;"",C69,B69)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5"/>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="7"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="8" t="str">
+        <f aca="true">IF(A70="","",IF(I70="Hidden","Hidden",IF(AND(H70&lt;&gt;"",H70&gt;TODAY()),"Scheduled",IF(IF(C70&lt;&gt;"",C70,B70)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="7"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="8" t="str">
+        <f aca="true">IF(A71="","",IF(I71="Hidden","Hidden",IF(AND(H71&lt;&gt;"",H71&gt;TODAY()),"Scheduled",IF(IF(C71&lt;&gt;"",C71,B71)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="7"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="8" t="str">
+        <f aca="true">IF(A72="","",IF(I72="Hidden","Hidden",IF(AND(H72&lt;&gt;"",H72&gt;TODAY()),"Scheduled",IF(IF(C72&lt;&gt;"",C72,B72)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="7"/>
+      <c r="I73" s="5"/>
+      <c r="J73" s="8" t="str">
+        <f aca="true">IF(A73="","",IF(I73="Hidden","Hidden",IF(AND(H73&lt;&gt;"",H73&gt;TODAY()),"Scheduled",IF(IF(C73&lt;&gt;"",C73,B73)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="7"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="8" t="str">
+        <f aca="true">IF(A74="","",IF(I74="Hidden","Hidden",IF(AND(H74&lt;&gt;"",H74&gt;TODAY()),"Scheduled",IF(IF(C74&lt;&gt;"",C74,B74)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="7"/>
+      <c r="I75" s="5"/>
+      <c r="J75" s="8" t="str">
+        <f aca="true">IF(A75="","",IF(I75="Hidden","Hidden",IF(AND(H75&lt;&gt;"",H75&gt;TODAY()),"Scheduled",IF(IF(C75&lt;&gt;"",C75,B75)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="7"/>
+      <c r="I76" s="5"/>
+      <c r="J76" s="8" t="str">
+        <f aca="true">IF(A76="","",IF(I76="Hidden","Hidden",IF(AND(H76&lt;&gt;"",H76&gt;TODAY()),"Scheduled",IF(IF(C76&lt;&gt;"",C76,B76)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5"/>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5"/>
+      <c r="H77" s="7"/>
+      <c r="I77" s="5"/>
+      <c r="J77" s="8" t="str">
+        <f aca="true">IF(A77="","",IF(I77="Hidden","Hidden",IF(AND(H77&lt;&gt;"",H77&gt;TODAY()),"Scheduled",IF(IF(C77&lt;&gt;"",C77,B77)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5"/>
+      <c r="B78" s="7"/>
+      <c r="C78" s="7"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5"/>
+      <c r="H78" s="7"/>
+      <c r="I78" s="5"/>
+      <c r="J78" s="8" t="str">
+        <f aca="true">IF(A78="","",IF(I78="Hidden","Hidden",IF(AND(H78&lt;&gt;"",H78&gt;TODAY()),"Scheduled",IF(IF(C78&lt;&gt;"",C78,B78)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="5"/>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="7"/>
+      <c r="I79" s="5"/>
+      <c r="J79" s="8" t="str">
+        <f aca="true">IF(A79="","",IF(I79="Hidden","Hidden",IF(AND(H79&lt;&gt;"",H79&gt;TODAY()),"Scheduled",IF(IF(C79&lt;&gt;"",C79,B79)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5"/>
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="7"/>
+      <c r="I80" s="5"/>
+      <c r="J80" s="8" t="str">
+        <f aca="true">IF(A80="","",IF(I80="Hidden","Hidden",IF(AND(H80&lt;&gt;"",H80&gt;TODAY()),"Scheduled",IF(IF(C80&lt;&gt;"",C80,B80)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5"/>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="7"/>
+      <c r="I81" s="5"/>
+      <c r="J81" s="8" t="str">
+        <f aca="true">IF(A81="","",IF(I81="Hidden","Hidden",IF(AND(H81&lt;&gt;"",H81&gt;TODAY()),"Scheduled",IF(IF(C81&lt;&gt;"",C81,B81)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5"/>
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="7"/>
+      <c r="I82" s="5"/>
+      <c r="J82" s="8" t="str">
+        <f aca="true">IF(A82="","",IF(I82="Hidden","Hidden",IF(AND(H82&lt;&gt;"",H82&gt;TODAY()),"Scheduled",IF(IF(C82&lt;&gt;"",C82,B82)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5"/>
+      <c r="B83" s="7"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="7"/>
+      <c r="I83" s="5"/>
+      <c r="J83" s="8" t="str">
+        <f aca="true">IF(A83="","",IF(I83="Hidden","Hidden",IF(AND(H83&lt;&gt;"",H83&gt;TODAY()),"Scheduled",IF(IF(C83&lt;&gt;"",C83,B83)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="5"/>
+      <c r="B84" s="7"/>
+      <c r="C84" s="7"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="7"/>
+      <c r="I84" s="5"/>
+      <c r="J84" s="8" t="str">
+        <f aca="true">IF(A84="","",IF(I84="Hidden","Hidden",IF(AND(H84&lt;&gt;"",H84&gt;TODAY()),"Scheduled",IF(IF(C84&lt;&gt;"",C84,B84)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="5"/>
+      <c r="B85" s="7"/>
+      <c r="C85" s="7"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="7"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="8" t="str">
+        <f aca="true">IF(A85="","",IF(I85="Hidden","Hidden",IF(AND(H85&lt;&gt;"",H85&gt;TODAY()),"Scheduled",IF(IF(C85&lt;&gt;"",C85,B85)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="5"/>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5"/>
+      <c r="H86" s="7"/>
+      <c r="I86" s="5"/>
+      <c r="J86" s="8" t="str">
+        <f aca="true">IF(A86="","",IF(I86="Hidden","Hidden",IF(AND(H86&lt;&gt;"",H86&gt;TODAY()),"Scheduled",IF(IF(C86&lt;&gt;"",C86,B86)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="5"/>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
+      <c r="H87" s="7"/>
+      <c r="I87" s="5"/>
+      <c r="J87" s="8" t="str">
+        <f aca="true">IF(A87="","",IF(I87="Hidden","Hidden",IF(AND(H87&lt;&gt;"",H87&gt;TODAY()),"Scheduled",IF(IF(C87&lt;&gt;"",C87,B87)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="5"/>
+      <c r="B88" s="7"/>
+      <c r="C88" s="7"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="7"/>
+      <c r="I88" s="5"/>
+      <c r="J88" s="8" t="str">
+        <f aca="true">IF(A88="","",IF(I88="Hidden","Hidden",IF(AND(H88&lt;&gt;"",H88&gt;TODAY()),"Scheduled",IF(IF(C88&lt;&gt;"",C88,B88)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="5"/>
+      <c r="B89" s="7"/>
+      <c r="C89" s="7"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="7"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="8" t="str">
+        <f aca="true">IF(A89="","",IF(I89="Hidden","Hidden",IF(AND(H89&lt;&gt;"",H89&gt;TODAY()),"Scheduled",IF(IF(C89&lt;&gt;"",C89,B89)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="5"/>
+      <c r="B90" s="7"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="7"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="8" t="str">
+        <f aca="true">IF(A90="","",IF(I90="Hidden","Hidden",IF(AND(H90&lt;&gt;"",H90&gt;TODAY()),"Scheduled",IF(IF(C90&lt;&gt;"",C90,B90)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="5"/>
+      <c r="B91" s="7"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="7"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="8" t="str">
+        <f aca="true">IF(A91="","",IF(I91="Hidden","Hidden",IF(AND(H91&lt;&gt;"",H91&gt;TODAY()),"Scheduled",IF(IF(C91&lt;&gt;"",C91,B91)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="5"/>
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="7"/>
+      <c r="I92" s="5"/>
+      <c r="J92" s="8" t="str">
+        <f aca="true">IF(A92="","",IF(I92="Hidden","Hidden",IF(AND(H92&lt;&gt;"",H92&gt;TODAY()),"Scheduled",IF(IF(C92&lt;&gt;"",C92,B92)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="5"/>
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="7"/>
+      <c r="I93" s="5"/>
+      <c r="J93" s="8" t="str">
+        <f aca="true">IF(A93="","",IF(I93="Hidden","Hidden",IF(AND(H93&lt;&gt;"",H93&gt;TODAY()),"Scheduled",IF(IF(C93&lt;&gt;"",C93,B93)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="5"/>
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="7"/>
+      <c r="I94" s="5"/>
+      <c r="J94" s="8" t="str">
+        <f aca="true">IF(A94="","",IF(I94="Hidden","Hidden",IF(AND(H94&lt;&gt;"",H94&gt;TODAY()),"Scheduled",IF(IF(C94&lt;&gt;"",C94,B94)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="5"/>
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="7"/>
+      <c r="I95" s="5"/>
+      <c r="J95" s="8" t="str">
+        <f aca="true">IF(A95="","",IF(I95="Hidden","Hidden",IF(AND(H95&lt;&gt;"",H95&gt;TODAY()),"Scheduled",IF(IF(C95&lt;&gt;"",C95,B95)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="5"/>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="5"/>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="7"/>
+      <c r="I96" s="5"/>
+      <c r="J96" s="8" t="str">
+        <f aca="true">IF(A96="","",IF(I96="Hidden","Hidden",IF(AND(H96&lt;&gt;"",H96&gt;TODAY()),"Scheduled",IF(IF(C96&lt;&gt;"",C96,B96)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="5"/>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="5"/>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="7"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="8" t="str">
+        <f aca="true">IF(A97="","",IF(I97="Hidden","Hidden",IF(AND(H97&lt;&gt;"",H97&gt;TODAY()),"Scheduled",IF(IF(C97&lt;&gt;"",C97,B97)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="5"/>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="7"/>
+      <c r="I98" s="5"/>
+      <c r="J98" s="8" t="str">
+        <f aca="true">IF(A98="","",IF(I98="Hidden","Hidden",IF(AND(H98&lt;&gt;"",H98&gt;TODAY()),"Scheduled",IF(IF(C98&lt;&gt;"",C98,B98)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="5"/>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="7"/>
+      <c r="I99" s="5"/>
+      <c r="J99" s="8" t="str">
+        <f aca="true">IF(A99="","",IF(I99="Hidden","Hidden",IF(AND(H99&lt;&gt;"",H99&gt;TODAY()),"Scheduled",IF(IF(C99&lt;&gt;"",C99,B99)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="5"/>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="5"/>
+      <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5"/>
+      <c r="H100" s="7"/>
+      <c r="I100" s="5"/>
+      <c r="J100" s="8" t="str">
+        <f aca="true">IF(A100="","",IF(I100="Hidden","Hidden",IF(AND(H100&lt;&gt;"",H100&gt;TODAY()),"Scheduled",IF(IF(C100&lt;&gt;"",C100,B100)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="5"/>
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="5"/>
+      <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
+      <c r="G101" s="5"/>
+      <c r="H101" s="7"/>
+      <c r="I101" s="5"/>
+      <c r="J101" s="8" t="str">
+        <f aca="true">IF(A101="","",IF(I101="Hidden","Hidden",IF(AND(H101&lt;&gt;"",H101&gt;TODAY()),"Scheduled",IF(IF(C101&lt;&gt;"",C101,B101)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="5"/>
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="5"/>
+      <c r="E102" s="5"/>
+      <c r="F102" s="5"/>
+      <c r="G102" s="5"/>
+      <c r="H102" s="7"/>
+      <c r="I102" s="5"/>
+      <c r="J102" s="8" t="str">
+        <f aca="true">IF(A102="","",IF(I102="Hidden","Hidden",IF(AND(H102&lt;&gt;"",H102&gt;TODAY()),"Scheduled",IF(IF(C102&lt;&gt;"",C102,B102)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="5"/>
+      <c r="B103" s="7"/>
+      <c r="C103" s="7"/>
+      <c r="D103" s="5"/>
+      <c r="E103" s="5"/>
+      <c r="F103" s="5"/>
+      <c r="G103" s="5"/>
+      <c r="H103" s="7"/>
+      <c r="I103" s="5"/>
+      <c r="J103" s="8" t="str">
+        <f aca="true">IF(A103="","",IF(I103="Hidden","Hidden",IF(AND(H103&lt;&gt;"",H103&gt;TODAY()),"Scheduled",IF(IF(C103&lt;&gt;"",C103,B103)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="5"/>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7"/>
+      <c r="D104" s="5"/>
+      <c r="E104" s="5"/>
+      <c r="F104" s="5"/>
+      <c r="G104" s="5"/>
+      <c r="H104" s="7"/>
+      <c r="I104" s="5"/>
+      <c r="J104" s="8" t="str">
+        <f aca="true">IF(A104="","",IF(I104="Hidden","Hidden",IF(AND(H104&lt;&gt;"",H104&gt;TODAY()),"Scheduled",IF(IF(C104&lt;&gt;"",C104,B104)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="5"/>
+      <c r="B105" s="7"/>
+      <c r="C105" s="7"/>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
+      <c r="G105" s="5"/>
+      <c r="H105" s="7"/>
+      <c r="I105" s="5"/>
+      <c r="J105" s="8" t="str">
+        <f aca="true">IF(A105="","",IF(I105="Hidden","Hidden",IF(AND(H105&lt;&gt;"",H105&gt;TODAY()),"Scheduled",IF(IF(C105&lt;&gt;"",C105,B105)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="5"/>
+      <c r="B106" s="7"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="5"/>
+      <c r="E106" s="5"/>
+      <c r="F106" s="5"/>
+      <c r="G106" s="5"/>
+      <c r="H106" s="7"/>
+      <c r="I106" s="5"/>
+      <c r="J106" s="8" t="str">
+        <f aca="true">IF(A106="","",IF(I106="Hidden","Hidden",IF(AND(H106&lt;&gt;"",H106&gt;TODAY()),"Scheduled",IF(IF(C106&lt;&gt;"",C106,B106)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="5"/>
+      <c r="B107" s="7"/>
+      <c r="C107" s="7"/>
+      <c r="D107" s="5"/>
+      <c r="E107" s="5"/>
+      <c r="F107" s="5"/>
+      <c r="G107" s="5"/>
+      <c r="H107" s="7"/>
+      <c r="I107" s="5"/>
+      <c r="J107" s="8" t="str">
+        <f aca="true">IF(A107="","",IF(I107="Hidden","Hidden",IF(AND(H107&lt;&gt;"",H107&gt;TODAY()),"Scheduled",IF(IF(C107&lt;&gt;"",C107,B107)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="5"/>
+      <c r="B108" s="7"/>
+      <c r="C108" s="7"/>
+      <c r="D108" s="5"/>
+      <c r="E108" s="5"/>
+      <c r="F108" s="5"/>
+      <c r="G108" s="5"/>
+      <c r="H108" s="7"/>
+      <c r="I108" s="5"/>
+      <c r="J108" s="8" t="str">
+        <f aca="true">IF(A108="","",IF(I108="Hidden","Hidden",IF(AND(H108&lt;&gt;"",H108&gt;TODAY()),"Scheduled",IF(IF(C108&lt;&gt;"",C108,B108)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="5"/>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7"/>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
+      <c r="G109" s="5"/>
+      <c r="H109" s="7"/>
+      <c r="I109" s="5"/>
+      <c r="J109" s="8" t="str">
+        <f aca="true">IF(A109="","",IF(I109="Hidden","Hidden",IF(AND(H109&lt;&gt;"",H109&gt;TODAY()),"Scheduled",IF(IF(C109&lt;&gt;"",C109,B109)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="5"/>
+      <c r="B110" s="7"/>
+      <c r="C110" s="7"/>
+      <c r="D110" s="5"/>
+      <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
+      <c r="G110" s="5"/>
+      <c r="H110" s="7"/>
+      <c r="I110" s="5"/>
+      <c r="J110" s="8" t="str">
+        <f aca="true">IF(A110="","",IF(I110="Hidden","Hidden",IF(AND(H110&lt;&gt;"",H110&gt;TODAY()),"Scheduled",IF(IF(C110&lt;&gt;"",C110,B110)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="5"/>
+      <c r="B111" s="7"/>
+      <c r="C111" s="7"/>
+      <c r="D111" s="5"/>
+      <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
+      <c r="G111" s="5"/>
+      <c r="H111" s="7"/>
+      <c r="I111" s="5"/>
+      <c r="J111" s="8" t="str">
+        <f aca="true">IF(A111="","",IF(I111="Hidden","Hidden",IF(AND(H111&lt;&gt;"",H111&gt;TODAY()),"Scheduled",IF(IF(C111&lt;&gt;"",C111,B111)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="5"/>
+      <c r="B112" s="7"/>
+      <c r="C112" s="7"/>
+      <c r="D112" s="5"/>
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" s="5"/>
+      <c r="H112" s="7"/>
+      <c r="I112" s="5"/>
+      <c r="J112" s="8" t="str">
+        <f aca="true">IF(A112="","",IF(I112="Hidden","Hidden",IF(AND(H112&lt;&gt;"",H112&gt;TODAY()),"Scheduled",IF(IF(C112&lt;&gt;"",C112,B112)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="5"/>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="5"/>
+      <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
+      <c r="G113" s="5"/>
+      <c r="H113" s="7"/>
+      <c r="I113" s="5"/>
+      <c r="J113" s="8" t="str">
+        <f aca="true">IF(A113="","",IF(I113="Hidden","Hidden",IF(AND(H113&lt;&gt;"",H113&gt;TODAY()),"Scheduled",IF(IF(C113&lt;&gt;"",C113,B113)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="5"/>
+      <c r="B114" s="7"/>
+      <c r="C114" s="7"/>
+      <c r="D114" s="5"/>
+      <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
+      <c r="G114" s="5"/>
+      <c r="H114" s="7"/>
+      <c r="I114" s="5"/>
+      <c r="J114" s="8" t="str">
+        <f aca="true">IF(A114="","",IF(I114="Hidden","Hidden",IF(AND(H114&lt;&gt;"",H114&gt;TODAY()),"Scheduled",IF(IF(C114&lt;&gt;"",C114,B114)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="5"/>
+      <c r="B115" s="7"/>
+      <c r="C115" s="7"/>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="7"/>
+      <c r="I115" s="5"/>
+      <c r="J115" s="8" t="str">
+        <f aca="true">IF(A115="","",IF(I115="Hidden","Hidden",IF(AND(H115&lt;&gt;"",H115&gt;TODAY()),"Scheduled",IF(IF(C115&lt;&gt;"",C115,B115)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="5"/>
+      <c r="B116" s="7"/>
+      <c r="C116" s="7"/>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
+      <c r="G116" s="5"/>
+      <c r="H116" s="7"/>
+      <c r="I116" s="5"/>
+      <c r="J116" s="8" t="str">
+        <f aca="true">IF(A116="","",IF(I116="Hidden","Hidden",IF(AND(H116&lt;&gt;"",H116&gt;TODAY()),"Scheduled",IF(IF(C116&lt;&gt;"",C116,B116)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="5"/>
+      <c r="B117" s="7"/>
+      <c r="C117" s="7"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="7"/>
+      <c r="I117" s="5"/>
+      <c r="J117" s="8" t="str">
+        <f aca="true">IF(A117="","",IF(I117="Hidden","Hidden",IF(AND(H117&lt;&gt;"",H117&gt;TODAY()),"Scheduled",IF(IF(C117&lt;&gt;"",C117,B117)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="5"/>
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="7"/>
+      <c r="I118" s="5"/>
+      <c r="J118" s="8" t="str">
+        <f aca="true">IF(A118="","",IF(I118="Hidden","Hidden",IF(AND(H118&lt;&gt;"",H118&gt;TODAY()),"Scheduled",IF(IF(C118&lt;&gt;"",C118,B118)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="5"/>
+      <c r="B119" s="7"/>
+      <c r="C119" s="7"/>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="7"/>
+      <c r="I119" s="5"/>
+      <c r="J119" s="8" t="str">
+        <f aca="true">IF(A119="","",IF(I119="Hidden","Hidden",IF(AND(H119&lt;&gt;"",H119&gt;TODAY()),"Scheduled",IF(IF(C119&lt;&gt;"",C119,B119)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="5"/>
+      <c r="B120" s="7"/>
+      <c r="C120" s="7"/>
+      <c r="D120" s="5"/>
+      <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
+      <c r="G120" s="5"/>
+      <c r="H120" s="7"/>
+      <c r="I120" s="5"/>
+      <c r="J120" s="8" t="str">
+        <f aca="true">IF(A120="","",IF(I120="Hidden","Hidden",IF(AND(H120&lt;&gt;"",H120&gt;TODAY()),"Scheduled",IF(IF(C120&lt;&gt;"",C120,B120)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="5"/>
+      <c r="B121" s="7"/>
+      <c r="C121" s="7"/>
+      <c r="D121" s="5"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
+      <c r="G121" s="5"/>
+      <c r="H121" s="7"/>
+      <c r="I121" s="5"/>
+      <c r="J121" s="8" t="str">
+        <f aca="true">IF(A121="","",IF(I121="Hidden","Hidden",IF(AND(H121&lt;&gt;"",H121&gt;TODAY()),"Scheduled",IF(IF(C121&lt;&gt;"",C121,B121)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="5"/>
+      <c r="B122" s="7"/>
+      <c r="C122" s="7"/>
+      <c r="D122" s="5"/>
+      <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
+      <c r="G122" s="5"/>
+      <c r="H122" s="7"/>
+      <c r="I122" s="5"/>
+      <c r="J122" s="8" t="str">
+        <f aca="true">IF(A122="","",IF(I122="Hidden","Hidden",IF(AND(H122&lt;&gt;"",H122&gt;TODAY()),"Scheduled",IF(IF(C122&lt;&gt;"",C122,B122)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="5"/>
+      <c r="B123" s="7"/>
+      <c r="C123" s="7"/>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="7"/>
+      <c r="I123" s="5"/>
+      <c r="J123" s="8" t="str">
+        <f aca="true">IF(A123="","",IF(I123="Hidden","Hidden",IF(AND(H123&lt;&gt;"",H123&gt;TODAY()),"Scheduled",IF(IF(C123&lt;&gt;"",C123,B123)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="5"/>
+      <c r="B124" s="7"/>
+      <c r="C124" s="7"/>
+      <c r="D124" s="5"/>
+      <c r="E124" s="5"/>
+      <c r="F124" s="5"/>
+      <c r="G124" s="5"/>
+      <c r="H124" s="7"/>
+      <c r="I124" s="5"/>
+      <c r="J124" s="8" t="str">
+        <f aca="true">IF(A124="","",IF(I124="Hidden","Hidden",IF(AND(H124&lt;&gt;"",H124&gt;TODAY()),"Scheduled",IF(IF(C124&lt;&gt;"",C124,B124)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="5"/>
+      <c r="B125" s="7"/>
+      <c r="C125" s="7"/>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
+      <c r="G125" s="5"/>
+      <c r="H125" s="7"/>
+      <c r="I125" s="5"/>
+      <c r="J125" s="8" t="str">
+        <f aca="true">IF(A125="","",IF(I125="Hidden","Hidden",IF(AND(H125&lt;&gt;"",H125&gt;TODAY()),"Scheduled",IF(IF(C125&lt;&gt;"",C125,B125)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="5"/>
+      <c r="B126" s="7"/>
+      <c r="C126" s="7"/>
+      <c r="D126" s="5"/>
+      <c r="E126" s="5"/>
+      <c r="F126" s="5"/>
+      <c r="G126" s="5"/>
+      <c r="H126" s="7"/>
+      <c r="I126" s="5"/>
+      <c r="J126" s="8" t="str">
+        <f aca="true">IF(A126="","",IF(I126="Hidden","Hidden",IF(AND(H126&lt;&gt;"",H126&gt;TODAY()),"Scheduled",IF(IF(C126&lt;&gt;"",C126,B126)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="5"/>
+      <c r="B127" s="7"/>
+      <c r="C127" s="7"/>
+      <c r="D127" s="5"/>
+      <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
+      <c r="G127" s="5"/>
+      <c r="H127" s="7"/>
+      <c r="I127" s="5"/>
+      <c r="J127" s="8" t="str">
+        <f aca="true">IF(A127="","",IF(I127="Hidden","Hidden",IF(AND(H127&lt;&gt;"",H127&gt;TODAY()),"Scheduled",IF(IF(C127&lt;&gt;"",C127,B127)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="5"/>
+      <c r="B128" s="7"/>
+      <c r="C128" s="7"/>
+      <c r="D128" s="5"/>
+      <c r="E128" s="5"/>
+      <c r="F128" s="5"/>
+      <c r="G128" s="5"/>
+      <c r="H128" s="7"/>
+      <c r="I128" s="5"/>
+      <c r="J128" s="8" t="str">
+        <f aca="true">IF(A128="","",IF(I128="Hidden","Hidden",IF(AND(H128&lt;&gt;"",H128&gt;TODAY()),"Scheduled",IF(IF(C128&lt;&gt;"",C128,B128)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="5"/>
+      <c r="B129" s="7"/>
+      <c r="C129" s="7"/>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5"/>
+      <c r="H129" s="7"/>
+      <c r="I129" s="5"/>
+      <c r="J129" s="8" t="str">
+        <f aca="true">IF(A129="","",IF(I129="Hidden","Hidden",IF(AND(H129&lt;&gt;"",H129&gt;TODAY()),"Scheduled",IF(IF(C129&lt;&gt;"",C129,B129)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="5"/>
+      <c r="B130" s="7"/>
+      <c r="C130" s="7"/>
+      <c r="D130" s="5"/>
+      <c r="E130" s="5"/>
+      <c r="F130" s="5"/>
+      <c r="G130" s="5"/>
+      <c r="H130" s="7"/>
+      <c r="I130" s="5"/>
+      <c r="J130" s="8" t="str">
+        <f aca="true">IF(A130="","",IF(I130="Hidden","Hidden",IF(AND(H130&lt;&gt;"",H130&gt;TODAY()),"Scheduled",IF(IF(C130&lt;&gt;"",C130,B130)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="5"/>
+      <c r="B131" s="7"/>
+      <c r="C131" s="7"/>
+      <c r="D131" s="5"/>
+      <c r="E131" s="5"/>
+      <c r="F131" s="5"/>
+      <c r="G131" s="5"/>
+      <c r="H131" s="7"/>
+      <c r="I131" s="5"/>
+      <c r="J131" s="8" t="str">
+        <f aca="true">IF(A131="","",IF(I131="Hidden","Hidden",IF(AND(H131&lt;&gt;"",H131&gt;TODAY()),"Scheduled",IF(IF(C131&lt;&gt;"",C131,B131)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="5"/>
+      <c r="B132" s="7"/>
+      <c r="C132" s="7"/>
+      <c r="D132" s="5"/>
+      <c r="E132" s="5"/>
+      <c r="F132" s="5"/>
+      <c r="G132" s="5"/>
+      <c r="H132" s="7"/>
+      <c r="I132" s="5"/>
+      <c r="J132" s="8" t="str">
+        <f aca="true">IF(A132="","",IF(I132="Hidden","Hidden",IF(AND(H132&lt;&gt;"",H132&gt;TODAY()),"Scheduled",IF(IF(C132&lt;&gt;"",C132,B132)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="5"/>
+      <c r="B133" s="7"/>
+      <c r="C133" s="7"/>
+      <c r="D133" s="5"/>
+      <c r="E133" s="5"/>
+      <c r="F133" s="5"/>
+      <c r="G133" s="5"/>
+      <c r="H133" s="7"/>
+      <c r="I133" s="5"/>
+      <c r="J133" s="8" t="str">
+        <f aca="true">IF(A133="","",IF(I133="Hidden","Hidden",IF(AND(H133&lt;&gt;"",H133&gt;TODAY()),"Scheduled",IF(IF(C133&lt;&gt;"",C133,B133)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="5"/>
+      <c r="B134" s="7"/>
+      <c r="C134" s="7"/>
+      <c r="D134" s="5"/>
+      <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5"/>
+      <c r="H134" s="7"/>
+      <c r="I134" s="5"/>
+      <c r="J134" s="8" t="str">
+        <f aca="true">IF(A134="","",IF(I134="Hidden","Hidden",IF(AND(H134&lt;&gt;"",H134&gt;TODAY()),"Scheduled",IF(IF(C134&lt;&gt;"",C134,B134)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="5"/>
+      <c r="B135" s="7"/>
+      <c r="C135" s="7"/>
+      <c r="D135" s="5"/>
+      <c r="E135" s="5"/>
+      <c r="F135" s="5"/>
+      <c r="G135" s="5"/>
+      <c r="H135" s="7"/>
+      <c r="I135" s="5"/>
+      <c r="J135" s="8" t="str">
+        <f aca="true">IF(A135="","",IF(I135="Hidden","Hidden",IF(AND(H135&lt;&gt;"",H135&gt;TODAY()),"Scheduled",IF(IF(C135&lt;&gt;"",C135,B135)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="5"/>
+      <c r="B136" s="7"/>
+      <c r="C136" s="7"/>
+      <c r="D136" s="5"/>
+      <c r="E136" s="5"/>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5"/>
+      <c r="H136" s="7"/>
+      <c r="I136" s="5"/>
+      <c r="J136" s="8" t="str">
+        <f aca="true">IF(A136="","",IF(I136="Hidden","Hidden",IF(AND(H136&lt;&gt;"",H136&gt;TODAY()),"Scheduled",IF(IF(C136&lt;&gt;"",C136,B136)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="5"/>
+      <c r="B137" s="7"/>
+      <c r="C137" s="7"/>
+      <c r="D137" s="5"/>
+      <c r="E137" s="5"/>
+      <c r="F137" s="5"/>
+      <c r="G137" s="5"/>
+      <c r="H137" s="7"/>
+      <c r="I137" s="5"/>
+      <c r="J137" s="8" t="str">
+        <f aca="true">IF(A137="","",IF(I137="Hidden","Hidden",IF(AND(H137&lt;&gt;"",H137&gt;TODAY()),"Scheduled",IF(IF(C137&lt;&gt;"",C137,B137)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="5"/>
+      <c r="B138" s="7"/>
+      <c r="C138" s="7"/>
+      <c r="D138" s="5"/>
+      <c r="E138" s="5"/>
+      <c r="F138" s="5"/>
+      <c r="G138" s="5"/>
+      <c r="H138" s="7"/>
+      <c r="I138" s="5"/>
+      <c r="J138" s="8" t="str">
+        <f aca="true">IF(A138="","",IF(I138="Hidden","Hidden",IF(AND(H138&lt;&gt;"",H138&gt;TODAY()),"Scheduled",IF(IF(C138&lt;&gt;"",C138,B138)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="5"/>
+      <c r="B139" s="7"/>
+      <c r="C139" s="7"/>
+      <c r="D139" s="5"/>
+      <c r="E139" s="5"/>
+      <c r="F139" s="5"/>
+      <c r="G139" s="5"/>
+      <c r="H139" s="7"/>
+      <c r="I139" s="5"/>
+      <c r="J139" s="8" t="str">
+        <f aca="true">IF(A139="","",IF(I139="Hidden","Hidden",IF(AND(H139&lt;&gt;"",H139&gt;TODAY()),"Scheduled",IF(IF(C139&lt;&gt;"",C139,B139)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="5"/>
+      <c r="B140" s="7"/>
+      <c r="C140" s="7"/>
+      <c r="D140" s="5"/>
+      <c r="E140" s="5"/>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5"/>
+      <c r="H140" s="7"/>
+      <c r="I140" s="5"/>
+      <c r="J140" s="8" t="str">
+        <f aca="true">IF(A140="","",IF(I140="Hidden","Hidden",IF(AND(H140&lt;&gt;"",H140&gt;TODAY()),"Scheduled",IF(IF(C140&lt;&gt;"",C140,B140)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="5"/>
+      <c r="B141" s="7"/>
+      <c r="C141" s="7"/>
+      <c r="D141" s="5"/>
+      <c r="E141" s="5"/>
+      <c r="F141" s="5"/>
+      <c r="G141" s="5"/>
+      <c r="H141" s="7"/>
+      <c r="I141" s="5"/>
+      <c r="J141" s="8" t="str">
+        <f aca="true">IF(A141="","",IF(I141="Hidden","Hidden",IF(AND(H141&lt;&gt;"",H141&gt;TODAY()),"Scheduled",IF(IF(C141&lt;&gt;"",C141,B141)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="5"/>
+      <c r="B142" s="7"/>
+      <c r="C142" s="7"/>
+      <c r="D142" s="5"/>
+      <c r="E142" s="5"/>
+      <c r="F142" s="5"/>
+      <c r="G142" s="5"/>
+      <c r="H142" s="7"/>
+      <c r="I142" s="5"/>
+      <c r="J142" s="8" t="str">
+        <f aca="true">IF(A142="","",IF(I142="Hidden","Hidden",IF(AND(H142&lt;&gt;"",H142&gt;TODAY()),"Scheduled",IF(IF(C142&lt;&gt;"",C142,B142)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="5"/>
+      <c r="B143" s="7"/>
+      <c r="C143" s="7"/>
+      <c r="D143" s="5"/>
+      <c r="E143" s="5"/>
+      <c r="F143" s="5"/>
+      <c r="G143" s="5"/>
+      <c r="H143" s="7"/>
+      <c r="I143" s="5"/>
+      <c r="J143" s="8" t="str">
+        <f aca="true">IF(A143="","",IF(I143="Hidden","Hidden",IF(AND(H143&lt;&gt;"",H143&gt;TODAY()),"Scheduled",IF(IF(C143&lt;&gt;"",C143,B143)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="5"/>
+      <c r="B144" s="7"/>
+      <c r="C144" s="7"/>
+      <c r="D144" s="5"/>
+      <c r="E144" s="5"/>
+      <c r="F144" s="5"/>
+      <c r="G144" s="5"/>
+      <c r="H144" s="7"/>
+      <c r="I144" s="5"/>
+      <c r="J144" s="8" t="str">
+        <f aca="true">IF(A144="","",IF(I144="Hidden","Hidden",IF(AND(H144&lt;&gt;"",H144&gt;TODAY()),"Scheduled",IF(IF(C144&lt;&gt;"",C144,B144)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="5"/>
+      <c r="B145" s="7"/>
+      <c r="C145" s="7"/>
+      <c r="D145" s="5"/>
+      <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
+      <c r="G145" s="5"/>
+      <c r="H145" s="7"/>
+      <c r="I145" s="5"/>
+      <c r="J145" s="8" t="str">
+        <f aca="true">IF(A145="","",IF(I145="Hidden","Hidden",IF(AND(H145&lt;&gt;"",H145&gt;TODAY()),"Scheduled",IF(IF(C145&lt;&gt;"",C145,B145)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="5"/>
+      <c r="B146" s="7"/>
+      <c r="C146" s="7"/>
+      <c r="D146" s="5"/>
+      <c r="E146" s="5"/>
+      <c r="F146" s="5"/>
+      <c r="G146" s="5"/>
+      <c r="H146" s="7"/>
+      <c r="I146" s="5"/>
+      <c r="J146" s="8" t="str">
+        <f aca="true">IF(A146="","",IF(I146="Hidden","Hidden",IF(AND(H146&lt;&gt;"",H146&gt;TODAY()),"Scheduled",IF(IF(C146&lt;&gt;"",C146,B146)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="5"/>
+      <c r="B147" s="7"/>
+      <c r="C147" s="7"/>
+      <c r="D147" s="5"/>
+      <c r="E147" s="5"/>
+      <c r="F147" s="5"/>
+      <c r="G147" s="5"/>
+      <c r="H147" s="7"/>
+      <c r="I147" s="5"/>
+      <c r="J147" s="8" t="str">
+        <f aca="true">IF(A147="","",IF(I147="Hidden","Hidden",IF(AND(H147&lt;&gt;"",H147&gt;TODAY()),"Scheduled",IF(IF(C147&lt;&gt;"",C147,B147)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="5"/>
+      <c r="B148" s="7"/>
+      <c r="C148" s="7"/>
+      <c r="D148" s="5"/>
+      <c r="E148" s="5"/>
+      <c r="F148" s="5"/>
+      <c r="G148" s="5"/>
+      <c r="H148" s="7"/>
+      <c r="I148" s="5"/>
+      <c r="J148" s="8" t="str">
+        <f aca="true">IF(A148="","",IF(I148="Hidden","Hidden",IF(AND(H148&lt;&gt;"",H148&gt;TODAY()),"Scheduled",IF(IF(C148&lt;&gt;"",C148,B148)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="5"/>
+      <c r="B149" s="7"/>
+      <c r="C149" s="7"/>
+      <c r="D149" s="5"/>
+      <c r="E149" s="5"/>
+      <c r="F149" s="5"/>
+      <c r="G149" s="5"/>
+      <c r="H149" s="7"/>
+      <c r="I149" s="5"/>
+      <c r="J149" s="8" t="str">
+        <f aca="true">IF(A149="","",IF(I149="Hidden","Hidden",IF(AND(H149&lt;&gt;"",H149&gt;TODAY()),"Scheduled",IF(IF(C149&lt;&gt;"",C149,B149)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="5"/>
+      <c r="B150" s="7"/>
+      <c r="C150" s="7"/>
+      <c r="D150" s="5"/>
+      <c r="E150" s="5"/>
+      <c r="F150" s="5"/>
+      <c r="G150" s="5"/>
+      <c r="H150" s="7"/>
+      <c r="I150" s="5"/>
+      <c r="J150" s="8" t="str">
+        <f aca="true">IF(A150="","",IF(I150="Hidden","Hidden",IF(AND(H150&lt;&gt;"",H150&gt;TODAY()),"Scheduled",IF(IF(C150&lt;&gt;"",C150,B150)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="5"/>
+      <c r="B151" s="7"/>
+      <c r="C151" s="7"/>
+      <c r="D151" s="5"/>
+      <c r="E151" s="5"/>
+      <c r="F151" s="5"/>
+      <c r="G151" s="5"/>
+      <c r="H151" s="7"/>
+      <c r="I151" s="5"/>
+      <c r="J151" s="8" t="str">
+        <f aca="true">IF(A151="","",IF(I151="Hidden","Hidden",IF(AND(H151&lt;&gt;"",H151&gt;TODAY()),"Scheduled",IF(IF(C151&lt;&gt;"",C151,B151)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="5"/>
+      <c r="B152" s="7"/>
+      <c r="C152" s="7"/>
+      <c r="D152" s="5"/>
+      <c r="E152" s="5"/>
+      <c r="F152" s="5"/>
+      <c r="G152" s="5"/>
+      <c r="H152" s="7"/>
+      <c r="I152" s="5"/>
+      <c r="J152" s="8" t="str">
+        <f aca="true">IF(A152="","",IF(I152="Hidden","Hidden",IF(AND(H152&lt;&gt;"",H152&gt;TODAY()),"Scheduled",IF(IF(C152&lt;&gt;"",C152,B152)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="5"/>
+      <c r="B153" s="7"/>
+      <c r="C153" s="7"/>
+      <c r="D153" s="5"/>
+      <c r="E153" s="5"/>
+      <c r="F153" s="5"/>
+      <c r="G153" s="5"/>
+      <c r="H153" s="7"/>
+      <c r="I153" s="5"/>
+      <c r="J153" s="8" t="str">
+        <f aca="true">IF(A153="","",IF(I153="Hidden","Hidden",IF(AND(H153&lt;&gt;"",H153&gt;TODAY()),"Scheduled",IF(IF(C153&lt;&gt;"",C153,B153)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="5"/>
+      <c r="B154" s="7"/>
+      <c r="C154" s="7"/>
+      <c r="D154" s="5"/>
+      <c r="E154" s="5"/>
+      <c r="F154" s="5"/>
+      <c r="G154" s="5"/>
+      <c r="H154" s="7"/>
+      <c r="I154" s="5"/>
+      <c r="J154" s="8" t="str">
+        <f aca="true">IF(A154="","",IF(I154="Hidden","Hidden",IF(AND(H154&lt;&gt;"",H154&gt;TODAY()),"Scheduled",IF(IF(C154&lt;&gt;"",C154,B154)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="5"/>
+      <c r="B155" s="7"/>
+      <c r="C155" s="7"/>
+      <c r="D155" s="5"/>
+      <c r="E155" s="5"/>
+      <c r="F155" s="5"/>
+      <c r="G155" s="5"/>
+      <c r="H155" s="7"/>
+      <c r="I155" s="5"/>
+      <c r="J155" s="8" t="str">
+        <f aca="true">IF(A155="","",IF(I155="Hidden","Hidden",IF(AND(H155&lt;&gt;"",H155&gt;TODAY()),"Scheduled",IF(IF(C155&lt;&gt;"",C155,B155)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="5"/>
+      <c r="B156" s="7"/>
+      <c r="C156" s="7"/>
+      <c r="D156" s="5"/>
+      <c r="E156" s="5"/>
+      <c r="F156" s="5"/>
+      <c r="G156" s="5"/>
+      <c r="H156" s="7"/>
+      <c r="I156" s="5"/>
+      <c r="J156" s="8" t="str">
+        <f aca="true">IF(A156="","",IF(I156="Hidden","Hidden",IF(AND(H156&lt;&gt;"",H156&gt;TODAY()),"Scheduled",IF(IF(C156&lt;&gt;"",C156,B156)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="5"/>
+      <c r="B157" s="7"/>
+      <c r="C157" s="7"/>
+      <c r="D157" s="5"/>
+      <c r="E157" s="5"/>
+      <c r="F157" s="5"/>
+      <c r="G157" s="5"/>
+      <c r="H157" s="7"/>
+      <c r="I157" s="5"/>
+      <c r="J157" s="8" t="str">
+        <f aca="true">IF(A157="","",IF(I157="Hidden","Hidden",IF(AND(H157&lt;&gt;"",H157&gt;TODAY()),"Scheduled",IF(IF(C157&lt;&gt;"",C157,B157)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="5"/>
+      <c r="B158" s="7"/>
+      <c r="C158" s="7"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="5"/>
+      <c r="F158" s="5"/>
+      <c r="G158" s="5"/>
+      <c r="H158" s="7"/>
+      <c r="I158" s="5"/>
+      <c r="J158" s="8" t="str">
+        <f aca="true">IF(A158="","",IF(I158="Hidden","Hidden",IF(AND(H158&lt;&gt;"",H158&gt;TODAY()),"Scheduled",IF(IF(C158&lt;&gt;"",C158,B158)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="5"/>
+      <c r="B159" s="7"/>
+      <c r="C159" s="7"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="5"/>
+      <c r="H159" s="7"/>
+      <c r="I159" s="5"/>
+      <c r="J159" s="8" t="str">
+        <f aca="true">IF(A159="","",IF(I159="Hidden","Hidden",IF(AND(H159&lt;&gt;"",H159&gt;TODAY()),"Scheduled",IF(IF(C159&lt;&gt;"",C159,B159)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="5"/>
+      <c r="B160" s="7"/>
+      <c r="C160" s="7"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="5"/>
+      <c r="F160" s="5"/>
+      <c r="G160" s="5"/>
+      <c r="H160" s="7"/>
+      <c r="I160" s="5"/>
+      <c r="J160" s="8" t="str">
+        <f aca="true">IF(A160="","",IF(I160="Hidden","Hidden",IF(AND(H160&lt;&gt;"",H160&gt;TODAY()),"Scheduled",IF(IF(C160&lt;&gt;"",C160,B160)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="5"/>
+      <c r="B161" s="7"/>
+      <c r="C161" s="7"/>
+      <c r="D161" s="5"/>
+      <c r="E161" s="5"/>
+      <c r="F161" s="5"/>
+      <c r="G161" s="5"/>
+      <c r="H161" s="7"/>
+      <c r="I161" s="5"/>
+      <c r="J161" s="8" t="str">
+        <f aca="true">IF(A161="","",IF(I161="Hidden","Hidden",IF(AND(H161&lt;&gt;"",H161&gt;TODAY()),"Scheduled",IF(IF(C161&lt;&gt;"",C161,B161)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="5"/>
+      <c r="B162" s="7"/>
+      <c r="C162" s="7"/>
+      <c r="D162" s="5"/>
+      <c r="E162" s="5"/>
+      <c r="F162" s="5"/>
+      <c r="G162" s="5"/>
+      <c r="H162" s="7"/>
+      <c r="I162" s="5"/>
+      <c r="J162" s="8" t="str">
+        <f aca="true">IF(A162="","",IF(I162="Hidden","Hidden",IF(AND(H162&lt;&gt;"",H162&gt;TODAY()),"Scheduled",IF(IF(C162&lt;&gt;"",C162,B162)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="5"/>
+      <c r="B163" s="7"/>
+      <c r="C163" s="7"/>
+      <c r="D163" s="5"/>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
+      <c r="G163" s="5"/>
+      <c r="H163" s="7"/>
+      <c r="I163" s="5"/>
+      <c r="J163" s="8" t="str">
+        <f aca="true">IF(A163="","",IF(I163="Hidden","Hidden",IF(AND(H163&lt;&gt;"",H163&gt;TODAY()),"Scheduled",IF(IF(C163&lt;&gt;"",C163,B163)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="5"/>
+      <c r="B164" s="7"/>
+      <c r="C164" s="7"/>
+      <c r="D164" s="5"/>
+      <c r="E164" s="5"/>
+      <c r="F164" s="5"/>
+      <c r="G164" s="5"/>
+      <c r="H164" s="7"/>
+      <c r="I164" s="5"/>
+      <c r="J164" s="8" t="str">
+        <f aca="true">IF(A164="","",IF(I164="Hidden","Hidden",IF(AND(H164&lt;&gt;"",H164&gt;TODAY()),"Scheduled",IF(IF(C164&lt;&gt;"",C164,B164)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="5"/>
+      <c r="B165" s="7"/>
+      <c r="C165" s="7"/>
+      <c r="D165" s="5"/>
+      <c r="E165" s="5"/>
+      <c r="F165" s="5"/>
+      <c r="G165" s="5"/>
+      <c r="H165" s="7"/>
+      <c r="I165" s="5"/>
+      <c r="J165" s="8" t="str">
+        <f aca="true">IF(A165="","",IF(I165="Hidden","Hidden",IF(AND(H165&lt;&gt;"",H165&gt;TODAY()),"Scheduled",IF(IF(C165&lt;&gt;"",C165,B165)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="5"/>
+      <c r="B166" s="7"/>
+      <c r="C166" s="7"/>
+      <c r="D166" s="5"/>
+      <c r="E166" s="5"/>
+      <c r="F166" s="5"/>
+      <c r="G166" s="5"/>
+      <c r="H166" s="7"/>
+      <c r="I166" s="5"/>
+      <c r="J166" s="8" t="str">
+        <f aca="true">IF(A166="","",IF(I166="Hidden","Hidden",IF(AND(H166&lt;&gt;"",H166&gt;TODAY()),"Scheduled",IF(IF(C166&lt;&gt;"",C166,B166)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="5"/>
+      <c r="B167" s="7"/>
+      <c r="C167" s="7"/>
+      <c r="D167" s="5"/>
+      <c r="E167" s="5"/>
+      <c r="F167" s="5"/>
+      <c r="G167" s="5"/>
+      <c r="H167" s="7"/>
+      <c r="I167" s="5"/>
+      <c r="J167" s="8" t="str">
+        <f aca="true">IF(A167="","",IF(I167="Hidden","Hidden",IF(AND(H167&lt;&gt;"",H167&gt;TODAY()),"Scheduled",IF(IF(C167&lt;&gt;"",C167,B167)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="5"/>
+      <c r="B168" s="7"/>
+      <c r="C168" s="7"/>
+      <c r="D168" s="5"/>
+      <c r="E168" s="5"/>
+      <c r="F168" s="5"/>
+      <c r="G168" s="5"/>
+      <c r="H168" s="7"/>
+      <c r="I168" s="5"/>
+      <c r="J168" s="8" t="str">
+        <f aca="true">IF(A168="","",IF(I168="Hidden","Hidden",IF(AND(H168&lt;&gt;"",H168&gt;TODAY()),"Scheduled",IF(IF(C168&lt;&gt;"",C168,B168)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="5"/>
+      <c r="B169" s="7"/>
+      <c r="C169" s="7"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5"/>
+      <c r="G169" s="5"/>
+      <c r="H169" s="7"/>
+      <c r="I169" s="5"/>
+      <c r="J169" s="8" t="str">
+        <f aca="true">IF(A169="","",IF(I169="Hidden","Hidden",IF(AND(H169&lt;&gt;"",H169&gt;TODAY()),"Scheduled",IF(IF(C169&lt;&gt;"",C169,B169)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="5"/>
+      <c r="B170" s="7"/>
+      <c r="C170" s="7"/>
+      <c r="D170" s="5"/>
+      <c r="E170" s="5"/>
+      <c r="F170" s="5"/>
+      <c r="G170" s="5"/>
+      <c r="H170" s="7"/>
+      <c r="I170" s="5"/>
+      <c r="J170" s="8" t="str">
+        <f aca="true">IF(A170="","",IF(I170="Hidden","Hidden",IF(AND(H170&lt;&gt;"",H170&gt;TODAY()),"Scheduled",IF(IF(C170&lt;&gt;"",C170,B170)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="5"/>
+      <c r="B171" s="7"/>
+      <c r="C171" s="7"/>
+      <c r="D171" s="5"/>
+      <c r="E171" s="5"/>
+      <c r="F171" s="5"/>
+      <c r="G171" s="5"/>
+      <c r="H171" s="7"/>
+      <c r="I171" s="5"/>
+      <c r="J171" s="8" t="str">
+        <f aca="true">IF(A171="","",IF(I171="Hidden","Hidden",IF(AND(H171&lt;&gt;"",H171&gt;TODAY()),"Scheduled",IF(IF(C171&lt;&gt;"",C171,B171)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="5"/>
+      <c r="B172" s="7"/>
+      <c r="C172" s="7"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+      <c r="F172" s="5"/>
+      <c r="G172" s="5"/>
+      <c r="H172" s="7"/>
+      <c r="I172" s="5"/>
+      <c r="J172" s="8" t="str">
+        <f aca="true">IF(A172="","",IF(I172="Hidden","Hidden",IF(AND(H172&lt;&gt;"",H172&gt;TODAY()),"Scheduled",IF(IF(C172&lt;&gt;"",C172,B172)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="5"/>
+      <c r="B173" s="7"/>
+      <c r="C173" s="7"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+      <c r="F173" s="5"/>
+      <c r="G173" s="5"/>
+      <c r="H173" s="7"/>
+      <c r="I173" s="5"/>
+      <c r="J173" s="8" t="str">
+        <f aca="true">IF(A173="","",IF(I173="Hidden","Hidden",IF(AND(H173&lt;&gt;"",H173&gt;TODAY()),"Scheduled",IF(IF(C173&lt;&gt;"",C173,B173)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="5"/>
+      <c r="B174" s="7"/>
+      <c r="C174" s="7"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="5"/>
+      <c r="F174" s="5"/>
+      <c r="G174" s="5"/>
+      <c r="H174" s="7"/>
+      <c r="I174" s="5"/>
+      <c r="J174" s="8" t="str">
+        <f aca="true">IF(A174="","",IF(I174="Hidden","Hidden",IF(AND(H174&lt;&gt;"",H174&gt;TODAY()),"Scheduled",IF(IF(C174&lt;&gt;"",C174,B174)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="5"/>
+      <c r="B175" s="7"/>
+      <c r="C175" s="7"/>
+      <c r="D175" s="5"/>
+      <c r="E175" s="5"/>
+      <c r="F175" s="5"/>
+      <c r="G175" s="5"/>
+      <c r="H175" s="7"/>
+      <c r="I175" s="5"/>
+      <c r="J175" s="8" t="str">
+        <f aca="true">IF(A175="","",IF(I175="Hidden","Hidden",IF(AND(H175&lt;&gt;"",H175&gt;TODAY()),"Scheduled",IF(IF(C175&lt;&gt;"",C175,B175)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="5"/>
+      <c r="B176" s="7"/>
+      <c r="C176" s="7"/>
+      <c r="D176" s="5"/>
+      <c r="E176" s="5"/>
+      <c r="F176" s="5"/>
+      <c r="G176" s="5"/>
+      <c r="H176" s="7"/>
+      <c r="I176" s="5"/>
+      <c r="J176" s="8" t="str">
+        <f aca="true">IF(A176="","",IF(I176="Hidden","Hidden",IF(AND(H176&lt;&gt;"",H176&gt;TODAY()),"Scheduled",IF(IF(C176&lt;&gt;"",C176,B176)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="5"/>
+      <c r="B177" s="7"/>
+      <c r="C177" s="7"/>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
+      <c r="F177" s="5"/>
+      <c r="G177" s="5"/>
+      <c r="H177" s="7"/>
+      <c r="I177" s="5"/>
+      <c r="J177" s="8" t="str">
+        <f aca="true">IF(A177="","",IF(I177="Hidden","Hidden",IF(AND(H177&lt;&gt;"",H177&gt;TODAY()),"Scheduled",IF(IF(C177&lt;&gt;"",C177,B177)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="5"/>
+      <c r="B178" s="7"/>
+      <c r="C178" s="7"/>
+      <c r="D178" s="5"/>
+      <c r="E178" s="5"/>
+      <c r="F178" s="5"/>
+      <c r="G178" s="5"/>
+      <c r="H178" s="7"/>
+      <c r="I178" s="5"/>
+      <c r="J178" s="8" t="str">
+        <f aca="true">IF(A178="","",IF(I178="Hidden","Hidden",IF(AND(H178&lt;&gt;"",H178&gt;TODAY()),"Scheduled",IF(IF(C178&lt;&gt;"",C178,B178)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="5"/>
+      <c r="B179" s="7"/>
+      <c r="C179" s="7"/>
+      <c r="D179" s="5"/>
+      <c r="E179" s="5"/>
+      <c r="F179" s="5"/>
+      <c r="G179" s="5"/>
+      <c r="H179" s="7"/>
+      <c r="I179" s="5"/>
+      <c r="J179" s="8" t="str">
+        <f aca="true">IF(A179="","",IF(I179="Hidden","Hidden",IF(AND(H179&lt;&gt;"",H179&gt;TODAY()),"Scheduled",IF(IF(C179&lt;&gt;"",C179,B179)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="5"/>
+      <c r="B180" s="7"/>
+      <c r="C180" s="7"/>
+      <c r="D180" s="5"/>
+      <c r="E180" s="5"/>
+      <c r="F180" s="5"/>
+      <c r="G180" s="5"/>
+      <c r="H180" s="7"/>
+      <c r="I180" s="5"/>
+      <c r="J180" s="8" t="str">
+        <f aca="true">IF(A180="","",IF(I180="Hidden","Hidden",IF(AND(H180&lt;&gt;"",H180&gt;TODAY()),"Scheduled",IF(IF(C180&lt;&gt;"",C180,B180)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="5"/>
+      <c r="B181" s="7"/>
+      <c r="C181" s="7"/>
+      <c r="D181" s="5"/>
+      <c r="E181" s="5"/>
+      <c r="F181" s="5"/>
+      <c r="G181" s="5"/>
+      <c r="H181" s="7"/>
+      <c r="I181" s="5"/>
+      <c r="J181" s="8" t="str">
+        <f aca="true">IF(A181="","",IF(I181="Hidden","Hidden",IF(AND(H181&lt;&gt;"",H181&gt;TODAY()),"Scheduled",IF(IF(C181&lt;&gt;"",C181,B181)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="5"/>
+      <c r="B182" s="7"/>
+      <c r="C182" s="7"/>
+      <c r="D182" s="5"/>
+      <c r="E182" s="5"/>
+      <c r="F182" s="5"/>
+      <c r="G182" s="5"/>
+      <c r="H182" s="7"/>
+      <c r="I182" s="5"/>
+      <c r="J182" s="8" t="str">
+        <f aca="true">IF(A182="","",IF(I182="Hidden","Hidden",IF(AND(H182&lt;&gt;"",H182&gt;TODAY()),"Scheduled",IF(IF(C182&lt;&gt;"",C182,B182)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="5"/>
+      <c r="B183" s="7"/>
+      <c r="C183" s="7"/>
+      <c r="D183" s="5"/>
+      <c r="E183" s="5"/>
+      <c r="F183" s="5"/>
+      <c r="G183" s="5"/>
+      <c r="H183" s="7"/>
+      <c r="I183" s="5"/>
+      <c r="J183" s="8" t="str">
+        <f aca="true">IF(A183="","",IF(I183="Hidden","Hidden",IF(AND(H183&lt;&gt;"",H183&gt;TODAY()),"Scheduled",IF(IF(C183&lt;&gt;"",C183,B183)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="5"/>
+      <c r="B184" s="7"/>
+      <c r="C184" s="7"/>
+      <c r="D184" s="5"/>
+      <c r="E184" s="5"/>
+      <c r="F184" s="5"/>
+      <c r="G184" s="5"/>
+      <c r="H184" s="7"/>
+      <c r="I184" s="5"/>
+      <c r="J184" s="8" t="str">
+        <f aca="true">IF(A184="","",IF(I184="Hidden","Hidden",IF(AND(H184&lt;&gt;"",H184&gt;TODAY()),"Scheduled",IF(IF(C184&lt;&gt;"",C184,B184)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="5"/>
+      <c r="B185" s="7"/>
+      <c r="C185" s="7"/>
+      <c r="D185" s="5"/>
+      <c r="E185" s="5"/>
+      <c r="F185" s="5"/>
+      <c r="G185" s="5"/>
+      <c r="H185" s="7"/>
+      <c r="I185" s="5"/>
+      <c r="J185" s="8" t="str">
+        <f aca="true">IF(A185="","",IF(I185="Hidden","Hidden",IF(AND(H185&lt;&gt;"",H185&gt;TODAY()),"Scheduled",IF(IF(C185&lt;&gt;"",C185,B185)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="5"/>
+      <c r="B186" s="7"/>
+      <c r="C186" s="7"/>
+      <c r="D186" s="5"/>
+      <c r="E186" s="5"/>
+      <c r="F186" s="5"/>
+      <c r="G186" s="5"/>
+      <c r="H186" s="7"/>
+      <c r="I186" s="5"/>
+      <c r="J186" s="8" t="str">
+        <f aca="true">IF(A186="","",IF(I186="Hidden","Hidden",IF(AND(H186&lt;&gt;"",H186&gt;TODAY()),"Scheduled",IF(IF(C186&lt;&gt;"",C186,B186)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="5"/>
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+      <c r="D187" s="5"/>
+      <c r="E187" s="5"/>
+      <c r="F187" s="5"/>
+      <c r="G187" s="5"/>
+      <c r="H187" s="7"/>
+      <c r="I187" s="5"/>
+      <c r="J187" s="8" t="str">
+        <f aca="true">IF(A187="","",IF(I187="Hidden","Hidden",IF(AND(H187&lt;&gt;"",H187&gt;TODAY()),"Scheduled",IF(IF(C187&lt;&gt;"",C187,B187)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="5"/>
+      <c r="B188" s="7"/>
+      <c r="C188" s="7"/>
+      <c r="D188" s="5"/>
+      <c r="E188" s="5"/>
+      <c r="F188" s="5"/>
+      <c r="G188" s="5"/>
+      <c r="H188" s="7"/>
+      <c r="I188" s="5"/>
+      <c r="J188" s="8" t="str">
+        <f aca="true">IF(A188="","",IF(I188="Hidden","Hidden",IF(AND(H188&lt;&gt;"",H188&gt;TODAY()),"Scheduled",IF(IF(C188&lt;&gt;"",C188,B188)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="5"/>
+      <c r="B189" s="7"/>
+      <c r="C189" s="7"/>
+      <c r="D189" s="5"/>
+      <c r="E189" s="5"/>
+      <c r="F189" s="5"/>
+      <c r="G189" s="5"/>
+      <c r="H189" s="7"/>
+      <c r="I189" s="5"/>
+      <c r="J189" s="8" t="str">
+        <f aca="true">IF(A189="","",IF(I189="Hidden","Hidden",IF(AND(H189&lt;&gt;"",H189&gt;TODAY()),"Scheduled",IF(IF(C189&lt;&gt;"",C189,B189)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="5"/>
+      <c r="B190" s="7"/>
+      <c r="C190" s="7"/>
+      <c r="D190" s="5"/>
+      <c r="E190" s="5"/>
+      <c r="F190" s="5"/>
+      <c r="G190" s="5"/>
+      <c r="H190" s="7"/>
+      <c r="I190" s="5"/>
+      <c r="J190" s="8" t="str">
+        <f aca="true">IF(A190="","",IF(I190="Hidden","Hidden",IF(AND(H190&lt;&gt;"",H190&gt;TODAY()),"Scheduled",IF(IF(C190&lt;&gt;"",C190,B190)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="5"/>
+      <c r="B191" s="7"/>
+      <c r="C191" s="7"/>
+      <c r="D191" s="5"/>
+      <c r="E191" s="5"/>
+      <c r="F191" s="5"/>
+      <c r="G191" s="5"/>
+      <c r="H191" s="7"/>
+      <c r="I191" s="5"/>
+      <c r="J191" s="8" t="str">
+        <f aca="true">IF(A191="","",IF(I191="Hidden","Hidden",IF(AND(H191&lt;&gt;"",H191&gt;TODAY()),"Scheduled",IF(IF(C191&lt;&gt;"",C191,B191)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="5"/>
+      <c r="B192" s="7"/>
+      <c r="C192" s="7"/>
+      <c r="D192" s="5"/>
+      <c r="E192" s="5"/>
+      <c r="F192" s="5"/>
+      <c r="G192" s="5"/>
+      <c r="H192" s="7"/>
+      <c r="I192" s="5"/>
+      <c r="J192" s="8" t="str">
+        <f aca="true">IF(A192="","",IF(I192="Hidden","Hidden",IF(AND(H192&lt;&gt;"",H192&gt;TODAY()),"Scheduled",IF(IF(C192&lt;&gt;"",C192,B192)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="5"/>
+      <c r="B193" s="7"/>
+      <c r="C193" s="7"/>
+      <c r="D193" s="5"/>
+      <c r="E193" s="5"/>
+      <c r="F193" s="5"/>
+      <c r="G193" s="5"/>
+      <c r="H193" s="7"/>
+      <c r="I193" s="5"/>
+      <c r="J193" s="8" t="str">
+        <f aca="true">IF(A193="","",IF(I193="Hidden","Hidden",IF(AND(H193&lt;&gt;"",H193&gt;TODAY()),"Scheduled",IF(IF(C193&lt;&gt;"",C193,B193)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="5"/>
+      <c r="B194" s="7"/>
+      <c r="C194" s="7"/>
+      <c r="D194" s="5"/>
+      <c r="E194" s="5"/>
+      <c r="F194" s="5"/>
+      <c r="G194" s="5"/>
+      <c r="H194" s="7"/>
+      <c r="I194" s="5"/>
+      <c r="J194" s="8" t="str">
+        <f aca="true">IF(A194="","",IF(I194="Hidden","Hidden",IF(AND(H194&lt;&gt;"",H194&gt;TODAY()),"Scheduled",IF(IF(C194&lt;&gt;"",C194,B194)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="5"/>
+      <c r="B195" s="7"/>
+      <c r="C195" s="7"/>
+      <c r="D195" s="5"/>
+      <c r="E195" s="5"/>
+      <c r="F195" s="5"/>
+      <c r="G195" s="5"/>
+      <c r="H195" s="7"/>
+      <c r="I195" s="5"/>
+      <c r="J195" s="8" t="str">
+        <f aca="true">IF(A195="","",IF(I195="Hidden","Hidden",IF(AND(H195&lt;&gt;"",H195&gt;TODAY()),"Scheduled",IF(IF(C195&lt;&gt;"",C195,B195)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="5"/>
+      <c r="B196" s="7"/>
+      <c r="C196" s="7"/>
+      <c r="D196" s="5"/>
+      <c r="E196" s="5"/>
+      <c r="F196" s="5"/>
+      <c r="G196" s="5"/>
+      <c r="H196" s="7"/>
+      <c r="I196" s="5"/>
+      <c r="J196" s="8" t="str">
+        <f aca="true">IF(A196="","",IF(I196="Hidden","Hidden",IF(AND(H196&lt;&gt;"",H196&gt;TODAY()),"Scheduled",IF(IF(C196&lt;&gt;"",C196,B196)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="5"/>
+      <c r="B197" s="7"/>
+      <c r="C197" s="7"/>
+      <c r="D197" s="5"/>
+      <c r="E197" s="5"/>
+      <c r="F197" s="5"/>
+      <c r="G197" s="5"/>
+      <c r="H197" s="7"/>
+      <c r="I197" s="5"/>
+      <c r="J197" s="8" t="str">
+        <f aca="true">IF(A197="","",IF(I197="Hidden","Hidden",IF(AND(H197&lt;&gt;"",H197&gt;TODAY()),"Scheduled",IF(IF(C197&lt;&gt;"",C197,B197)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="5"/>
+      <c r="B198" s="7"/>
+      <c r="C198" s="7"/>
+      <c r="D198" s="5"/>
+      <c r="E198" s="5"/>
+      <c r="F198" s="5"/>
+      <c r="G198" s="5"/>
+      <c r="H198" s="7"/>
+      <c r="I198" s="5"/>
+      <c r="J198" s="8" t="str">
+        <f aca="true">IF(A198="","",IF(I198="Hidden","Hidden",IF(AND(H198&lt;&gt;"",H198&gt;TODAY()),"Scheduled",IF(IF(C198&lt;&gt;"",C198,B198)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="5"/>
+      <c r="B199" s="7"/>
+      <c r="C199" s="7"/>
+      <c r="D199" s="5"/>
+      <c r="E199" s="5"/>
+      <c r="F199" s="5"/>
+      <c r="G199" s="5"/>
+      <c r="H199" s="7"/>
+      <c r="I199" s="5"/>
+      <c r="J199" s="8" t="str">
+        <f aca="true">IF(A199="","",IF(I199="Hidden","Hidden",IF(AND(H199&lt;&gt;"",H199&gt;TODAY()),"Scheduled",IF(IF(C199&lt;&gt;"",C199,B199)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="5"/>
+      <c r="B200" s="7"/>
+      <c r="C200" s="7"/>
+      <c r="D200" s="5"/>
+      <c r="E200" s="5"/>
+      <c r="F200" s="5"/>
+      <c r="G200" s="5"/>
+      <c r="H200" s="7"/>
+      <c r="I200" s="5"/>
+      <c r="J200" s="8" t="str">
+        <f aca="true">IF(A200="","",IF(I200="Hidden","Hidden",IF(AND(H200&lt;&gt;"",H200&gt;TODAY()),"Scheduled",IF(IF(C200&lt;&gt;"",C200,B200)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J2:J200">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>OR(J2="Showing",J2="Regular",J2="Special, in effect")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>J2="Scheduled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>OR(J2="Expired",J2="Hidden")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:C200 H2:H200" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F200" type="list">
+      <formula1>"Yes"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I2:I200" type="list">
+      <formula1>"Live,Hidden"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 5-5-5 menu to the menu board for 9-10 October
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="198">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -345,6 +345,12 @@
   </si>
   <si>
     <t xml:space="preserve">Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 5-5-5 menu: Friday 9 and Saturday 10 October</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fish &amp; chips. Curry. Wagyu burger. 5 bean chilli &amp; rice. Sausage &amp; mash with onion gravy.</t>
   </si>
   <si>
     <t xml:space="preserve">New Year's Eve BBQ: Thursday 31 December</t>
@@ -5540,7 +5546,7 @@
         <v>46304</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>46387</v>
+        <v>46305</v>
       </c>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
@@ -5552,25 +5558,27 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>14.95</v>
-      </c>
+      <c r="D5" s="9"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="G5" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>46387</v>
+      </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
         <v>60</v>
@@ -5580,9 +5588,9 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>92</v>
@@ -5591,7 +5599,7 @@
         <v>93</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>13.95</v>
+        <v>14.95</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
@@ -5611,7 +5619,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>94</v>
@@ -5640,7 +5648,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>96</v>
@@ -5669,14 +5677,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="5"/>
+      <c r="C9" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="D9" s="9" t="n">
-        <v>11.95</v>
+        <v>13.95</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
@@ -5696,20 +5706,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>101</v>
-      </c>
+      <c r="C10" s="5"/>
       <c r="D10" s="9" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>11.95</v>
+      </c>
+      <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
         <v>86</v>
       </c>
@@ -5725,21 +5731,21 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="9" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>86</v>
@@ -5756,16 +5762,22 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="9" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="F12" s="5" t="s">
         <v>86</v>
       </c>
@@ -5783,15 +5795,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B13" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="9" t="n">
-        <v>13.95</v>
-      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="9"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
         <v>86</v>
@@ -5810,14 +5820,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="9" t="n">
-        <v>14.95</v>
+        <v>13.95</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
@@ -5837,14 +5847,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="9" t="n">
-        <v>14.5</v>
+        <v>14.95</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
@@ -5864,14 +5874,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="9" t="n">
-        <v>15.95</v>
+        <v>14.5</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
@@ -5891,16 +5901,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C17" s="5" t="s">
         <v>112</v>
       </c>
+      <c r="C17" s="5"/>
       <c r="D17" s="9" t="n">
-        <v>16.95</v>
+        <v>15.95</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
@@ -5920,14 +5928,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C18" s="5"/>
       <c r="D18" s="9" t="n">
-        <v>5.95</v>
+        <v>16.95</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
@@ -5947,10 +5957,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9" t="n">
@@ -5974,10 +5984,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="9" t="n">
@@ -6001,16 +6011,18 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C21" s="5"/>
-      <c r="D21" s="9"/>
+      <c r="D21" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
@@ -6035,7 +6047,7 @@
       <c r="D22" s="9"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
@@ -6054,13 +6066,13 @@
         <v>70</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="9"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
@@ -6079,15 +6091,13 @@
         <v>70</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="9"/>
-      <c r="E24" s="5" t="s">
-        <v>102</v>
-      </c>
+      <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -6102,20 +6112,30 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
+      <c r="A25" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>123</v>
+      </c>
       <c r="C25" s="5"/>
       <c r="D25" s="9"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>120</v>
+      </c>
       <c r="G25" s="5"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
+      <c r="K25" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="L25" s="8" t="str">
         <f aca="true">IF(B25&amp;C25="","",IF(K25="Hidden","Hidden",IF(AND(H25&lt;&gt;"",H25&gt;TODAY()),"Scheduled",IF(AND(I25&lt;&gt;"",I25&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9166,19 +9186,19 @@
         <v>78</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>82</v>
@@ -9198,13 +9218,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -9225,13 +9245,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -9252,13 +9272,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -9279,13 +9299,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -9306,13 +9326,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -9333,10 +9353,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -9358,13 +9378,13 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -9385,13 +9405,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -9412,13 +9432,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -9439,13 +9459,13 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -9466,13 +9486,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -9493,13 +9513,13 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -9520,13 +9540,13 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -9547,13 +9567,13 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -9574,13 +9594,13 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -9601,10 +9621,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="9"/>
@@ -9626,10 +9646,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9"/>
@@ -9651,10 +9671,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9"/>
@@ -13162,7 +13182,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>82</v>
@@ -13179,7 +13199,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46304</v>
@@ -13197,7 +13217,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -13215,7 +13235,7 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46357</v>
@@ -15244,25 +15264,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>77</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>82</v>
@@ -15276,21 +15296,21 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46564</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>46508</v>
@@ -15305,23 +15325,23 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46592</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>59</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>46553</v>
@@ -18346,22 +18366,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>82</v>
@@ -18378,22 +18398,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>46304</v>

</xml_diff>

<commit_message>
Site review fixes: mobile hero, sticky call bar, hero badge, trimmed NYE repeats, SEO (meta, OG, JSON-LD, sitemap, robots), optional analytics and Ads tracking, remove concept footer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="230">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -382,12 +382,6 @@
     <t xml:space="preserve">Fish &amp; chips. Curry. Wagyu burger. 5 bean chilli &amp; rice. Sausage &amp; mash with onion gravy.</t>
   </si>
   <si>
-    <t xml:space="preserve">New Year's Eve BBQ: Thursday 31 December</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoked brisket, creamy mac and cheese, burgers and sausages with caramelised onions. Please book.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mains</t>
   </si>
   <si>
@@ -629,9 +623,6 @@
   </si>
   <si>
     <t xml:space="preserve">Christmas morning: we're open for drinks, with free mince pies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Year's Eve BBQ: smoked brisket, creamy mac and cheese, burgers and sausages with caramelised onions. Call to book.</t>
   </si>
   <si>
     <t xml:space="preserve">Event</t>
@@ -5696,27 +5687,25 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
+      <c r="A5" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="B5" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="9"/>
+        <v>93</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>14.95</v>
+      </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="I5" s="7" t="n">
-        <v>46387</v>
-      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
         <v>62</v>
@@ -5726,9 +5715,9 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>94</v>
@@ -5737,7 +5726,7 @@
         <v>95</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>14.95</v>
+        <v>13.95</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
@@ -5757,7 +5746,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>96</v>
@@ -5786,7 +5775,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>98</v>
@@ -5815,16 +5804,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>101</v>
-      </c>
+      <c r="C9" s="5"/>
       <c r="D9" s="9" t="n">
-        <v>13.95</v>
+        <v>11.95</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
@@ -5844,16 +5831,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="5"/>
+      <c r="C10" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="D10" s="9" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="E10" s="5"/>
+        <v>10.95</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="F10" s="5" t="s">
         <v>88</v>
       </c>
@@ -5869,21 +5860,21 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>88</v>
@@ -5900,22 +5891,16 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" s="5" t="s">
         <v>107</v>
       </c>
+      <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>106</v>
-      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
         <v>88</v>
       </c>
@@ -5933,13 +5918,15 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D13" s="9"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="9" t="n">
+        <v>13.95</v>
+      </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
         <v>88</v>
@@ -5958,14 +5945,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="9" t="n">
-        <v>13.95</v>
+        <v>14.95</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
@@ -5985,14 +5972,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="9" t="n">
-        <v>14.95</v>
+        <v>14.5</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
@@ -6012,14 +5999,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="9" t="n">
-        <v>14.5</v>
+        <v>15.95</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
@@ -6039,14 +6026,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C17" s="5"/>
       <c r="D17" s="9" t="n">
-        <v>15.95</v>
+        <v>16.95</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
@@ -6066,16 +6055,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C18" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="C18" s="5"/>
       <c r="D18" s="9" t="n">
-        <v>16.95</v>
+        <v>5.95</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
@@ -6095,10 +6082,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9" t="n">
@@ -6122,10 +6109,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="9" t="n">
@@ -6149,18 +6136,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C21" s="5"/>
-      <c r="D21" s="9" t="n">
-        <v>5.95</v>
-      </c>
+      <c r="D21" s="9"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
@@ -6185,7 +6170,7 @@
       <c r="D22" s="9"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
@@ -6204,13 +6189,13 @@
         <v>72</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="9"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
@@ -6229,13 +6214,15 @@
         <v>72</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="9"/>
-      <c r="E24" s="5"/>
+      <c r="E24" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="F24" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -6250,30 +6237,20 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>125</v>
-      </c>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="9"/>
-      <c r="E25" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>122</v>
-      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="5"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="5"/>
-      <c r="K25" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="K25" s="5"/>
       <c r="L25" s="8" t="str">
         <f aca="true">IF(B25&amp;C25="","",IF(K25="Hidden","Hidden",IF(AND(H25&lt;&gt;"",H25&gt;TODAY()),"Scheduled",IF(AND(I25&lt;&gt;"",I25&lt;TODAY()),"Expired","Showing"))))</f>
-        <v>Showing</v>
+        <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9324,19 +9301,19 @@
         <v>80</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -9356,13 +9333,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -9383,13 +9360,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -9410,13 +9387,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>139</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -9437,13 +9414,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -9464,13 +9441,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -9491,10 +9468,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -9516,13 +9493,13 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>145</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -9543,13 +9520,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -9570,13 +9547,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -9597,13 +9574,13 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -9624,13 +9601,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -9651,13 +9628,13 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -9678,13 +9655,13 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>161</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -9705,13 +9682,13 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -9732,13 +9709,13 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -9759,10 +9736,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="9"/>
@@ -9784,10 +9761,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>169</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9"/>
@@ -9809,10 +9786,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9"/>
@@ -13320,7 +13297,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>84</v>
@@ -13337,7 +13314,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46304</v>
@@ -13355,7 +13332,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -13371,22 +13348,14 @@
         <v>Scheduled</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>46357</v>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>46387</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>62</v>
-      </c>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="8" t="str">
         <f aca="true">IF(A4="","",IF(D4="Hidden","Hidden",IF(AND(B4&lt;&gt;"",B4&gt;TODAY()),"Scheduled",IF(AND(C4&lt;&gt;"",C4&lt;TODAY()),"Expired","Showing"))))</f>
-        <v>Scheduled</v>
+        <v/>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15402,25 +15371,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>178</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>84</v>
@@ -15434,7 +15403,7 @@
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46387</v>
@@ -15442,11 +15411,11 @@
       <c r="C2" s="7"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>46304</v>
@@ -15461,21 +15430,21 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46564</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>46508</v>
@@ -15490,23 +15459,23 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46592</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="5" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>61</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46553</v>
@@ -18516,22 +18485,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>196</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>84</v>
@@ -18548,22 +18517,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>46304</v>
@@ -21604,31 +21573,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="E1" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>204</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>207</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -21645,27 +21614,27 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>6.5</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -21679,10 +21648,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>2</v>
@@ -21690,14 +21659,14 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -21711,10 +21680,10 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
@@ -21724,14 +21693,14 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -21745,10 +21714,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>28.4</v>
@@ -21757,19 +21726,19 @@
         <v>2600</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>227</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -21783,10 +21752,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>20.3</v>
@@ -21795,19 +21764,19 @@
         <v>850</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>232</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>

</xml_diff>

<commit_message>
Add Christmas party dinner section driven by Menu tab (shown 10 Oct to 23 Dec)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="254">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -382,7 +382,82 @@
     <t xml:space="preserve">Fish &amp; chips. Curry. Wagyu burger. 5 bean chilli &amp; rice. Sausage &amp; mash with onion gravy.</t>
   </si>
   <si>
+    <t xml:space="preserve">2 courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 courses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">King prawn &amp; avocado cocktail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baked brie with cranberry sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Served with sourdough toasts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creamy garlic mushrooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On garlic ciabatta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salmon en croute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With dauphinoise and tenderstem broccoli. Baked salmon available gluten free.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roast chicken breast, skin on</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filled with sage and onion stuffing, with buttery mash and seasonal greens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asparagus, spinach &amp; ricotta tortellini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In a creamy herb and garlic sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desserts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional Christmas pudding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With brandy sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferrero Rocher cheesecake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With runny cream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple &amp; cinnamon crumble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topped with clotted cream</t>
   </si>
   <si>
     <t xml:space="preserve">Steak &amp; Timothy Taylor ale pie</t>
@@ -419,9 +494,6 @@
   </si>
   <si>
     <t xml:space="preserve">Creamy mash, garden peas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
   </si>
   <si>
     <t xml:space="preserve">Honey-soaked halloumi</t>
@@ -5686,26 +5758,28 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>93</v>
-      </c>
+      <c r="C5" s="5"/>
       <c r="D5" s="9" t="n">
-        <v>14.95</v>
+        <v>16.95</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G5" s="5"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="H5" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
         <v>62</v>
@@ -5717,24 +5791,26 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>95</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="C6" s="5"/>
       <c r="D6" s="9" t="n">
-        <v>13.95</v>
+        <v>21.95</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+      <c r="H6" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
         <v>62</v>
@@ -5746,24 +5822,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G7" s="5"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="H7" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
         <v>62</v>
@@ -5775,24 +5853,28 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="9"/>
+      <c r="E8" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G8" s="5"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="H8" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
         <v>62</v>
@@ -5804,22 +5886,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="9" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="E9" s="5"/>
+      <c r="C9" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="9"/>
+      <c r="E9" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F9" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G9" s="5"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="H9" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
         <v>62</v>
@@ -5829,28 +5917,28 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="E10" s="5" t="s">
         <v>104</v>
       </c>
+      <c r="D10" s="9"/>
+      <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+      <c r="H10" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
         <v>62</v>
@@ -5862,7 +5950,7 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>105</v>
@@ -5870,18 +5958,20 @@
       <c r="C11" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>13.95</v>
-      </c>
+      <c r="D11" s="9"/>
       <c r="E11" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="H11" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5" t="s">
         <v>62</v>
@@ -5893,20 +5983,28 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="5"/>
       <c r="C12" s="5" t="s">
         <v>108</v>
       </c>
       <c r="D12" s="9"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="5" t="s">
+        <v>109</v>
+      </c>
       <c r="F12" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="H12" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J12" s="5"/>
       <c r="K12" s="5" t="s">
         <v>62</v>
@@ -5918,22 +6016,26 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="9" t="n">
-        <v>13.95</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D13" s="9"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G13" s="5"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
+      <c r="H13" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J13" s="5"/>
       <c r="K13" s="5" t="s">
         <v>62</v>
@@ -5945,22 +6047,26 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="9" t="n">
-        <v>14.95</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" s="9"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
+      <c r="H14" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J14" s="5"/>
       <c r="K14" s="5" t="s">
         <v>62</v>
@@ -5972,22 +6078,26 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="9" t="n">
-        <v>14.5</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D15" s="9"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
+      <c r="H15" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5" t="s">
         <v>62</v>
@@ -5997,16 +6107,18 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="5"/>
+        <v>117</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>118</v>
+      </c>
       <c r="D16" s="9" t="n">
-        <v>15.95</v>
+        <v>14.95</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
@@ -6026,16 +6138,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>16.95</v>
+        <v>13.95</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
@@ -6055,14 +6167,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C18" s="5"/>
+        <v>121</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>122</v>
+      </c>
       <c r="D18" s="9" t="n">
-        <v>5.95</v>
+        <v>13.95</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
@@ -6082,14 +6196,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C19" s="5"/>
+        <v>123</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>124</v>
+      </c>
       <c r="D19" s="9" t="n">
-        <v>5.95</v>
+        <v>13.95</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
@@ -6109,14 +6225,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="9" t="n">
-        <v>5.95</v>
+        <v>11.95</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
@@ -6136,16 +6252,22 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="5"/>
+        <v>127</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>109</v>
+      </c>
       <c r="F21" s="5" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
@@ -6159,18 +6281,24 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="5"/>
+        <v>129</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>109</v>
+      </c>
       <c r="F22" s="5" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
@@ -6186,16 +6314,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C23" s="5"/>
+        <v>131</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5" t="s">
+        <v>132</v>
+      </c>
       <c r="D23" s="9"/>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
@@ -6211,18 +6339,18 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C24" s="5"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="5" t="s">
-        <v>104</v>
-      </c>
+      <c r="D24" s="9" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -6237,190 +6365,296 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
+      <c r="A25" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="C25" s="5"/>
-      <c r="D25" s="9"/>
+      <c r="D25" s="9" t="n">
+        <v>14.95</v>
+      </c>
       <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="F25" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G25" s="5"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
+      <c r="K25" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L25" s="8" t="str">
         <f aca="true">IF(B25&amp;C25="","",IF(K25="Hidden","Hidden",IF(AND(H25&lt;&gt;"",H25&gt;TODAY()),"Scheduled",IF(AND(I25&lt;&gt;"",I25&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
+      <c r="A26" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="C26" s="5"/>
-      <c r="D26" s="9"/>
+      <c r="D26" s="9" t="n">
+        <v>14.5</v>
+      </c>
       <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="F26" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G26" s="5"/>
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
+      <c r="K26" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L26" s="8" t="str">
         <f aca="true">IF(B26&amp;C26="","",IF(K26="Hidden","Hidden",IF(AND(H26&lt;&gt;"",H26&gt;TODAY()),"Scheduled",IF(AND(I26&lt;&gt;"",I26&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
+      <c r="A27" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>136</v>
+      </c>
       <c r="C27" s="5"/>
-      <c r="D27" s="9"/>
+      <c r="D27" s="9" t="n">
+        <v>15.95</v>
+      </c>
       <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
+      <c r="F27" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G27" s="5"/>
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
+      <c r="K27" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L27" s="8" t="str">
         <f aca="true">IF(B27&amp;C27="","",IF(K27="Hidden","Hidden",IF(AND(H27&lt;&gt;"",H27&gt;TODAY()),"Scheduled",IF(AND(I27&lt;&gt;"",I27&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="9"/>
+      <c r="A28" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>16.95</v>
+      </c>
       <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+      <c r="F28" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G28" s="5"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
       <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
+      <c r="K28" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L28" s="8" t="str">
         <f aca="true">IF(B28&amp;C28="","",IF(K28="Hidden","Hidden",IF(AND(H28&lt;&gt;"",H28&gt;TODAY()),"Scheduled",IF(AND(I28&lt;&gt;"",I28&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
+      <c r="A29" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>140</v>
+      </c>
       <c r="C29" s="5"/>
-      <c r="D29" s="9"/>
+      <c r="D29" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
+      <c r="F29" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G29" s="5"/>
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
+      <c r="K29" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L29" s="8" t="str">
         <f aca="true">IF(B29&amp;C29="","",IF(K29="Hidden","Hidden",IF(AND(H29&lt;&gt;"",H29&gt;TODAY()),"Scheduled",IF(AND(I29&lt;&gt;"",I29&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
+      <c r="A30" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="C30" s="5"/>
-      <c r="D30" s="9"/>
+      <c r="D30" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+      <c r="F30" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G30" s="5"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
+      <c r="K30" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L30" s="8" t="str">
         <f aca="true">IF(B30&amp;C30="","",IF(K30="Hidden","Hidden",IF(AND(H30&lt;&gt;"",H30&gt;TODAY()),"Scheduled",IF(AND(I30&lt;&gt;"",I30&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
+      <c r="A31" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>142</v>
+      </c>
       <c r="C31" s="5"/>
-      <c r="D31" s="9"/>
+      <c r="D31" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
+      <c r="F31" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G31" s="5"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
+      <c r="K31" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L31" s="8" t="str">
         <f aca="true">IF(B31&amp;C31="","",IF(K31="Hidden","Hidden",IF(AND(H31&lt;&gt;"",H31&gt;TODAY()),"Scheduled",IF(AND(I31&lt;&gt;"",I31&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
+      <c r="A32" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>143</v>
+      </c>
       <c r="C32" s="5"/>
       <c r="D32" s="9"/>
       <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
+      <c r="F32" s="5" t="s">
+        <v>144</v>
+      </c>
       <c r="G32" s="5"/>
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
+      <c r="K32" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L32" s="8" t="str">
         <f aca="true">IF(B32&amp;C32="","",IF(K32="Hidden","Hidden",IF(AND(H32&lt;&gt;"",H32&gt;TODAY()),"Scheduled",IF(AND(I32&lt;&gt;"",I32&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
+      <c r="A33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="C33" s="5"/>
       <c r="D33" s="9"/>
       <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
+      <c r="F33" s="5" t="s">
+        <v>144</v>
+      </c>
       <c r="G33" s="5"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
+      <c r="K33" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L33" s="8" t="str">
         <f aca="true">IF(B33&amp;C33="","",IF(K33="Hidden","Hidden",IF(AND(H33&lt;&gt;"",H33&gt;TODAY()),"Scheduled",IF(AND(I33&lt;&gt;"",I33&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
+      <c r="A34" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>146</v>
+      </c>
       <c r="C34" s="5"/>
       <c r="D34" s="9"/>
       <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
+      <c r="F34" s="5" t="s">
+        <v>144</v>
+      </c>
       <c r="G34" s="5"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
+      <c r="K34" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L34" s="8" t="str">
         <f aca="true">IF(B34&amp;C34="","",IF(K34="Hidden","Hidden",IF(AND(H34&lt;&gt;"",H34&gt;TODAY()),"Scheduled",IF(AND(I34&lt;&gt;"",I34&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
+      <c r="A35" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>147</v>
+      </c>
       <c r="C35" s="5"/>
       <c r="D35" s="9"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
+      <c r="E35" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>144</v>
+      </c>
       <c r="G35" s="5"/>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
+      <c r="K35" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L35" s="8" t="str">
         <f aca="true">IF(B35&amp;C35="","",IF(K35="Hidden","Hidden",IF(AND(H35&lt;&gt;"",H35&gt;TODAY()),"Scheduled",IF(AND(I35&lt;&gt;"",I35&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9301,19 +9535,19 @@
         <v>80</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -9333,13 +9567,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -9360,13 +9594,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -9387,13 +9621,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -9414,13 +9648,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -9441,13 +9675,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -9468,10 +9702,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -9493,13 +9727,13 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -9520,13 +9754,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -9547,13 +9781,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -9574,13 +9808,13 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -9601,13 +9835,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>153</v>
+        <v>177</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>154</v>
+        <v>178</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -9628,13 +9862,13 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -9655,13 +9889,13 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>157</v>
+        <v>181</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>159</v>
+        <v>183</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -9682,13 +9916,13 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>162</v>
+        <v>186</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -9709,13 +9943,13 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -9736,10 +9970,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="9"/>
@@ -9761,10 +9995,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9"/>
@@ -9786,10 +10020,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9"/>
@@ -13297,7 +13531,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>84</v>
@@ -13314,7 +13548,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46304</v>
@@ -13332,7 +13566,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -15371,25 +15605,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>84</v>
@@ -15403,7 +15637,7 @@
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46387</v>
@@ -15411,11 +15645,11 @@
       <c r="C2" s="7"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>46304</v>
@@ -15430,21 +15664,21 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46564</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="5" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>46508</v>
@@ -15459,23 +15693,23 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46592</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="5" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>61</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46553</v>
@@ -18485,22 +18719,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>190</v>
+        <v>214</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>84</v>
@@ -18517,22 +18751,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>195</v>
+        <v>219</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>196</v>
+        <v>220</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>198</v>
+        <v>222</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>46304</v>
@@ -21573,31 +21807,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>203</v>
+        <v>227</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>206</v>
+        <v>230</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -21614,27 +21848,27 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>207</v>
+        <v>231</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>6.5</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>209</v>
+        <v>233</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -21648,10 +21882,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>207</v>
+        <v>231</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>213</v>
+        <v>237</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>2</v>
@@ -21659,14 +21893,14 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -21680,10 +21914,10 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>207</v>
+        <v>231</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
@@ -21693,14 +21927,14 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>217</v>
+        <v>241</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>218</v>
+        <v>242</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -21714,10 +21948,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>219</v>
+        <v>243</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>28.4</v>
@@ -21726,19 +21960,19 @@
         <v>2600</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>223</v>
+        <v>247</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -21752,10 +21986,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>219</v>
+        <v>243</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>225</v>
+        <v>249</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>20.3</v>
@@ -21764,19 +21998,19 @@
         <v>850</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>226</v>
+        <v>250</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>228</v>
+        <v>252</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>229</v>
+        <v>253</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>

</xml_diff>

<commit_message>
Chronological flow: faded-photo hero, menu then events in date order, Halloween quiz with artwork, Christmas menu inside events
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="264">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -715,6 +715,36 @@
     <t xml:space="preserve">Booking note</t>
   </si>
   <si>
+    <t xml:space="preserve">Image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menu group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halloween Quiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Royal Oak quiz goes Halloween. Fancy dress optional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call 01765 677198 to book a table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/halloween.svg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas party dinner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home-cooked festive food in our private room, for 20 to 30 guests. Two or three courses, with vegetarian and gluten-free choices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Call 01765 677198 to book your party</t>
+  </si>
+  <si>
     <t xml:space="preserve">New Year's Eve BBQ</t>
   </si>
   <si>
@@ -763,16 +793,16 @@
     <t xml:space="preserve">Button link</t>
   </si>
   <si>
-    <t xml:space="preserve">Thursday 31 December</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Year's Eve BBQ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mexican Dave is on the grill, with plenty of Mexican flavours on the go. There may even be the odd frozen margarita behind the bar. Please book.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoked brisket | Creamy mac and cheese | Burgers and sausages with caramelised onions | Frozen margaritas behind the bar, maybe</t>
+    <t xml:space="preserve">EXAMPLE: Beer festival</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE (hidden): a big headline panel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE (hidden): use this tab for one big announcement near the top of the page. Copy this row, change it and set Status to Live.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cask ales all weekend | Live music | Food all day</t>
   </si>
   <si>
     <t xml:space="preserve">Call to book</t>
@@ -15589,7 +15619,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -15597,10 +15627,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15632,124 +15664,170 @@
         <v>58</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>46387</v>
+        <v>46326</v>
       </c>
       <c r="C2" s="7"/>
-      <c r="D2" s="5"/>
+      <c r="D2" s="5" t="s">
+        <v>205</v>
+      </c>
       <c r="E2" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>46304</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="H2" s="7"/>
       <c r="I2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J2" s="8" t="str">
+      <c r="J2" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="K2" s="5"/>
+      <c r="L2" s="8" t="str">
         <f aca="true">IF(A2="","",IF(I2="Hidden","Hidden",IF(AND(H2&lt;&gt;"",H2&gt;TODAY()),"Scheduled",IF(IF(C2&lt;&gt;"",C2,B2)&lt;TODAY(),"Expired","Showing"))))</f>
         <v>Showing</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B3" s="7" t="n">
-        <v>46564</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="5" t="s">
-        <v>206</v>
-      </c>
+        <v>46357</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>46379</v>
+      </c>
+      <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H3" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="8" t="str">
+        <f aca="true">IF(A3="","",IF(I3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(IF(C3&lt;&gt;"",C3,B3)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v>Showing</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>46387</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="8" t="str">
+        <f aca="true">IF(A4="","",IF(I4="Hidden","Hidden",IF(AND(H4&lt;&gt;"",H4&gt;TODAY()),"Scheduled",IF(IF(C4&lt;&gt;"",C4,B4)&lt;TODAY(),"Expired","Showing"))))</f>
+        <v>Showing</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>46564</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="H5" s="7" t="n">
         <v>46508</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I5" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="8" t="str">
-        <f aca="true">IF(A3="","",IF(I3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(IF(C3&lt;&gt;"",C3,B3)&lt;TODAY(),"Expired","Showing"))))</f>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="8" t="str">
+        <f aca="true">IF(A5="","",IF(I5="Hidden","Hidden",IF(AND(H5&lt;&gt;"",H5&gt;TODAY()),"Scheduled",IF(IF(C5&lt;&gt;"",C5,B5)&lt;TODAY(),"Expired","Showing"))))</f>
         <v>Hidden</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B4" s="7" t="n">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>46592</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="C6" s="7"/>
+      <c r="D6" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="H4" s="7" t="n">
+      <c r="G6" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <v>46553</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="8" t="str">
-        <f aca="true">IF(A4="","",IF(I4="Hidden","Hidden",IF(AND(H4&lt;&gt;"",H4&gt;TODAY()),"Scheduled",IF(IF(C4&lt;&gt;"",C4,B4)&lt;TODAY(),"Expired","Showing"))))</f>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="8" t="str">
+        <f aca="true">IF(A6="","",IF(I6="Hidden","Hidden",IF(AND(H6&lt;&gt;"",H6&gt;TODAY()),"Scheduled",IF(IF(C6&lt;&gt;"",C6,B6)&lt;TODAY(),"Expired","Showing"))))</f>
         <v>Hidden</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="8" t="str">
-        <f aca="true">IF(A5="","",IF(I5="Hidden","Hidden",IF(AND(H5&lt;&gt;"",H5&gt;TODAY()),"Scheduled",IF(IF(C5&lt;&gt;"",C5,B5)&lt;TODAY(),"Expired","Showing"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="8" t="str">
-        <f aca="true">IF(A6="","",IF(I6="Hidden","Hidden",IF(AND(H6&lt;&gt;"",H6&gt;TODAY()),"Scheduled",IF(IF(C6&lt;&gt;"",C6,B6)&lt;TODAY(),"Expired","Showing"))))</f>
-        <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15762,7 +15840,9 @@
       <c r="G7" s="5"/>
       <c r="H7" s="7"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="8" t="str">
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="8" t="str">
         <f aca="true">IF(A7="","",IF(I7="Hidden","Hidden",IF(AND(H7&lt;&gt;"",H7&gt;TODAY()),"Scheduled",IF(IF(C7&lt;&gt;"",C7,B7)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15777,7 +15857,9 @@
       <c r="G8" s="5"/>
       <c r="H8" s="7"/>
       <c r="I8" s="5"/>
-      <c r="J8" s="8" t="str">
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="8" t="str">
         <f aca="true">IF(A8="","",IF(I8="Hidden","Hidden",IF(AND(H8&lt;&gt;"",H8&gt;TODAY()),"Scheduled",IF(IF(C8&lt;&gt;"",C8,B8)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15792,7 +15874,9 @@
       <c r="G9" s="5"/>
       <c r="H9" s="7"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="8" t="str">
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="8" t="str">
         <f aca="true">IF(A9="","",IF(I9="Hidden","Hidden",IF(AND(H9&lt;&gt;"",H9&gt;TODAY()),"Scheduled",IF(IF(C9&lt;&gt;"",C9,B9)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15807,7 +15891,9 @@
       <c r="G10" s="5"/>
       <c r="H10" s="7"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="8" t="str">
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="8" t="str">
         <f aca="true">IF(A10="","",IF(I10="Hidden","Hidden",IF(AND(H10&lt;&gt;"",H10&gt;TODAY()),"Scheduled",IF(IF(C10&lt;&gt;"",C10,B10)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15822,7 +15908,9 @@
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>
       <c r="I11" s="5"/>
-      <c r="J11" s="8" t="str">
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="8" t="str">
         <f aca="true">IF(A11="","",IF(I11="Hidden","Hidden",IF(AND(H11&lt;&gt;"",H11&gt;TODAY()),"Scheduled",IF(IF(C11&lt;&gt;"",C11,B11)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15837,7 +15925,9 @@
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="8" t="str">
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="8" t="str">
         <f aca="true">IF(A12="","",IF(I12="Hidden","Hidden",IF(AND(H12&lt;&gt;"",H12&gt;TODAY()),"Scheduled",IF(IF(C12&lt;&gt;"",C12,B12)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15852,7 +15942,9 @@
       <c r="G13" s="5"/>
       <c r="H13" s="7"/>
       <c r="I13" s="5"/>
-      <c r="J13" s="8" t="str">
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="8" t="str">
         <f aca="true">IF(A13="","",IF(I13="Hidden","Hidden",IF(AND(H13&lt;&gt;"",H13&gt;TODAY()),"Scheduled",IF(IF(C13&lt;&gt;"",C13,B13)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15867,7 +15959,9 @@
       <c r="G14" s="5"/>
       <c r="H14" s="7"/>
       <c r="I14" s="5"/>
-      <c r="J14" s="8" t="str">
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="8" t="str">
         <f aca="true">IF(A14="","",IF(I14="Hidden","Hidden",IF(AND(H14&lt;&gt;"",H14&gt;TODAY()),"Scheduled",IF(IF(C14&lt;&gt;"",C14,B14)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15882,7 +15976,9 @@
       <c r="G15" s="5"/>
       <c r="H15" s="7"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="8" t="str">
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="8" t="str">
         <f aca="true">IF(A15="","",IF(I15="Hidden","Hidden",IF(AND(H15&lt;&gt;"",H15&gt;TODAY()),"Scheduled",IF(IF(C15&lt;&gt;"",C15,B15)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15897,7 +15993,9 @@
       <c r="G16" s="5"/>
       <c r="H16" s="7"/>
       <c r="I16" s="5"/>
-      <c r="J16" s="8" t="str">
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="8" t="str">
         <f aca="true">IF(A16="","",IF(I16="Hidden","Hidden",IF(AND(H16&lt;&gt;"",H16&gt;TODAY()),"Scheduled",IF(IF(C16&lt;&gt;"",C16,B16)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15912,7 +16010,9 @@
       <c r="G17" s="5"/>
       <c r="H17" s="7"/>
       <c r="I17" s="5"/>
-      <c r="J17" s="8" t="str">
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="8" t="str">
         <f aca="true">IF(A17="","",IF(I17="Hidden","Hidden",IF(AND(H17&lt;&gt;"",H17&gt;TODAY()),"Scheduled",IF(IF(C17&lt;&gt;"",C17,B17)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15927,7 +16027,9 @@
       <c r="G18" s="5"/>
       <c r="H18" s="7"/>
       <c r="I18" s="5"/>
-      <c r="J18" s="8" t="str">
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="8" t="str">
         <f aca="true">IF(A18="","",IF(I18="Hidden","Hidden",IF(AND(H18&lt;&gt;"",H18&gt;TODAY()),"Scheduled",IF(IF(C18&lt;&gt;"",C18,B18)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15942,7 +16044,9 @@
       <c r="G19" s="5"/>
       <c r="H19" s="7"/>
       <c r="I19" s="5"/>
-      <c r="J19" s="8" t="str">
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="8" t="str">
         <f aca="true">IF(A19="","",IF(I19="Hidden","Hidden",IF(AND(H19&lt;&gt;"",H19&gt;TODAY()),"Scheduled",IF(IF(C19&lt;&gt;"",C19,B19)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15957,7 +16061,9 @@
       <c r="G20" s="5"/>
       <c r="H20" s="7"/>
       <c r="I20" s="5"/>
-      <c r="J20" s="8" t="str">
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="8" t="str">
         <f aca="true">IF(A20="","",IF(I20="Hidden","Hidden",IF(AND(H20&lt;&gt;"",H20&gt;TODAY()),"Scheduled",IF(IF(C20&lt;&gt;"",C20,B20)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15972,7 +16078,9 @@
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="8" t="str">
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="8" t="str">
         <f aca="true">IF(A21="","",IF(I21="Hidden","Hidden",IF(AND(H21&lt;&gt;"",H21&gt;TODAY()),"Scheduled",IF(IF(C21&lt;&gt;"",C21,B21)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -15987,7 +16095,9 @@
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
       <c r="I22" s="5"/>
-      <c r="J22" s="8" t="str">
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="8" t="str">
         <f aca="true">IF(A22="","",IF(I22="Hidden","Hidden",IF(AND(H22&lt;&gt;"",H22&gt;TODAY()),"Scheduled",IF(IF(C22&lt;&gt;"",C22,B22)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16002,7 +16112,9 @@
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
       <c r="I23" s="5"/>
-      <c r="J23" s="8" t="str">
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="8" t="str">
         <f aca="true">IF(A23="","",IF(I23="Hidden","Hidden",IF(AND(H23&lt;&gt;"",H23&gt;TODAY()),"Scheduled",IF(IF(C23&lt;&gt;"",C23,B23)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16017,7 +16129,9 @@
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="8" t="str">
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="8" t="str">
         <f aca="true">IF(A24="","",IF(I24="Hidden","Hidden",IF(AND(H24&lt;&gt;"",H24&gt;TODAY()),"Scheduled",IF(IF(C24&lt;&gt;"",C24,B24)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16032,7 +16146,9 @@
       <c r="G25" s="5"/>
       <c r="H25" s="7"/>
       <c r="I25" s="5"/>
-      <c r="J25" s="8" t="str">
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="8" t="str">
         <f aca="true">IF(A25="","",IF(I25="Hidden","Hidden",IF(AND(H25&lt;&gt;"",H25&gt;TODAY()),"Scheduled",IF(IF(C25&lt;&gt;"",C25,B25)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16047,7 +16163,9 @@
       <c r="G26" s="5"/>
       <c r="H26" s="7"/>
       <c r="I26" s="5"/>
-      <c r="J26" s="8" t="str">
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="8" t="str">
         <f aca="true">IF(A26="","",IF(I26="Hidden","Hidden",IF(AND(H26&lt;&gt;"",H26&gt;TODAY()),"Scheduled",IF(IF(C26&lt;&gt;"",C26,B26)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16062,7 +16180,9 @@
       <c r="G27" s="5"/>
       <c r="H27" s="7"/>
       <c r="I27" s="5"/>
-      <c r="J27" s="8" t="str">
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="8" t="str">
         <f aca="true">IF(A27="","",IF(I27="Hidden","Hidden",IF(AND(H27&lt;&gt;"",H27&gt;TODAY()),"Scheduled",IF(IF(C27&lt;&gt;"",C27,B27)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16077,7 +16197,9 @@
       <c r="G28" s="5"/>
       <c r="H28" s="7"/>
       <c r="I28" s="5"/>
-      <c r="J28" s="8" t="str">
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="8" t="str">
         <f aca="true">IF(A28="","",IF(I28="Hidden","Hidden",IF(AND(H28&lt;&gt;"",H28&gt;TODAY()),"Scheduled",IF(IF(C28&lt;&gt;"",C28,B28)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16092,7 +16214,9 @@
       <c r="G29" s="5"/>
       <c r="H29" s="7"/>
       <c r="I29" s="5"/>
-      <c r="J29" s="8" t="str">
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="8" t="str">
         <f aca="true">IF(A29="","",IF(I29="Hidden","Hidden",IF(AND(H29&lt;&gt;"",H29&gt;TODAY()),"Scheduled",IF(IF(C29&lt;&gt;"",C29,B29)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16107,7 +16231,9 @@
       <c r="G30" s="5"/>
       <c r="H30" s="7"/>
       <c r="I30" s="5"/>
-      <c r="J30" s="8" t="str">
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="8" t="str">
         <f aca="true">IF(A30="","",IF(I30="Hidden","Hidden",IF(AND(H30&lt;&gt;"",H30&gt;TODAY()),"Scheduled",IF(IF(C30&lt;&gt;"",C30,B30)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16122,7 +16248,9 @@
       <c r="G31" s="5"/>
       <c r="H31" s="7"/>
       <c r="I31" s="5"/>
-      <c r="J31" s="8" t="str">
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="8" t="str">
         <f aca="true">IF(A31="","",IF(I31="Hidden","Hidden",IF(AND(H31&lt;&gt;"",H31&gt;TODAY()),"Scheduled",IF(IF(C31&lt;&gt;"",C31,B31)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16137,7 +16265,9 @@
       <c r="G32" s="5"/>
       <c r="H32" s="7"/>
       <c r="I32" s="5"/>
-      <c r="J32" s="8" t="str">
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="8" t="str">
         <f aca="true">IF(A32="","",IF(I32="Hidden","Hidden",IF(AND(H32&lt;&gt;"",H32&gt;TODAY()),"Scheduled",IF(IF(C32&lt;&gt;"",C32,B32)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16152,7 +16282,9 @@
       <c r="G33" s="5"/>
       <c r="H33" s="7"/>
       <c r="I33" s="5"/>
-      <c r="J33" s="8" t="str">
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="8" t="str">
         <f aca="true">IF(A33="","",IF(I33="Hidden","Hidden",IF(AND(H33&lt;&gt;"",H33&gt;TODAY()),"Scheduled",IF(IF(C33&lt;&gt;"",C33,B33)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16167,7 +16299,9 @@
       <c r="G34" s="5"/>
       <c r="H34" s="7"/>
       <c r="I34" s="5"/>
-      <c r="J34" s="8" t="str">
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="8" t="str">
         <f aca="true">IF(A34="","",IF(I34="Hidden","Hidden",IF(AND(H34&lt;&gt;"",H34&gt;TODAY()),"Scheduled",IF(IF(C34&lt;&gt;"",C34,B34)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16182,7 +16316,9 @@
       <c r="G35" s="5"/>
       <c r="H35" s="7"/>
       <c r="I35" s="5"/>
-      <c r="J35" s="8" t="str">
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="8" t="str">
         <f aca="true">IF(A35="","",IF(I35="Hidden","Hidden",IF(AND(H35&lt;&gt;"",H35&gt;TODAY()),"Scheduled",IF(IF(C35&lt;&gt;"",C35,B35)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16197,7 +16333,9 @@
       <c r="G36" s="5"/>
       <c r="H36" s="7"/>
       <c r="I36" s="5"/>
-      <c r="J36" s="8" t="str">
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="8" t="str">
         <f aca="true">IF(A36="","",IF(I36="Hidden","Hidden",IF(AND(H36&lt;&gt;"",H36&gt;TODAY()),"Scheduled",IF(IF(C36&lt;&gt;"",C36,B36)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16212,7 +16350,9 @@
       <c r="G37" s="5"/>
       <c r="H37" s="7"/>
       <c r="I37" s="5"/>
-      <c r="J37" s="8" t="str">
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="8" t="str">
         <f aca="true">IF(A37="","",IF(I37="Hidden","Hidden",IF(AND(H37&lt;&gt;"",H37&gt;TODAY()),"Scheduled",IF(IF(C37&lt;&gt;"",C37,B37)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16227,7 +16367,9 @@
       <c r="G38" s="5"/>
       <c r="H38" s="7"/>
       <c r="I38" s="5"/>
-      <c r="J38" s="8" t="str">
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="8" t="str">
         <f aca="true">IF(A38="","",IF(I38="Hidden","Hidden",IF(AND(H38&lt;&gt;"",H38&gt;TODAY()),"Scheduled",IF(IF(C38&lt;&gt;"",C38,B38)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16242,7 +16384,9 @@
       <c r="G39" s="5"/>
       <c r="H39" s="7"/>
       <c r="I39" s="5"/>
-      <c r="J39" s="8" t="str">
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="8" t="str">
         <f aca="true">IF(A39="","",IF(I39="Hidden","Hidden",IF(AND(H39&lt;&gt;"",H39&gt;TODAY()),"Scheduled",IF(IF(C39&lt;&gt;"",C39,B39)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16257,7 +16401,9 @@
       <c r="G40" s="5"/>
       <c r="H40" s="7"/>
       <c r="I40" s="5"/>
-      <c r="J40" s="8" t="str">
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+      <c r="L40" s="8" t="str">
         <f aca="true">IF(A40="","",IF(I40="Hidden","Hidden",IF(AND(H40&lt;&gt;"",H40&gt;TODAY()),"Scheduled",IF(IF(C40&lt;&gt;"",C40,B40)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16272,7 +16418,9 @@
       <c r="G41" s="5"/>
       <c r="H41" s="7"/>
       <c r="I41" s="5"/>
-      <c r="J41" s="8" t="str">
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+      <c r="L41" s="8" t="str">
         <f aca="true">IF(A41="","",IF(I41="Hidden","Hidden",IF(AND(H41&lt;&gt;"",H41&gt;TODAY()),"Scheduled",IF(IF(C41&lt;&gt;"",C41,B41)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16287,7 +16435,9 @@
       <c r="G42" s="5"/>
       <c r="H42" s="7"/>
       <c r="I42" s="5"/>
-      <c r="J42" s="8" t="str">
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
+      <c r="L42" s="8" t="str">
         <f aca="true">IF(A42="","",IF(I42="Hidden","Hidden",IF(AND(H42&lt;&gt;"",H42&gt;TODAY()),"Scheduled",IF(IF(C42&lt;&gt;"",C42,B42)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16302,7 +16452,9 @@
       <c r="G43" s="5"/>
       <c r="H43" s="7"/>
       <c r="I43" s="5"/>
-      <c r="J43" s="8" t="str">
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+      <c r="L43" s="8" t="str">
         <f aca="true">IF(A43="","",IF(I43="Hidden","Hidden",IF(AND(H43&lt;&gt;"",H43&gt;TODAY()),"Scheduled",IF(IF(C43&lt;&gt;"",C43,B43)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16317,7 +16469,9 @@
       <c r="G44" s="5"/>
       <c r="H44" s="7"/>
       <c r="I44" s="5"/>
-      <c r="J44" s="8" t="str">
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+      <c r="L44" s="8" t="str">
         <f aca="true">IF(A44="","",IF(I44="Hidden","Hidden",IF(AND(H44&lt;&gt;"",H44&gt;TODAY()),"Scheduled",IF(IF(C44&lt;&gt;"",C44,B44)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16332,7 +16486,9 @@
       <c r="G45" s="5"/>
       <c r="H45" s="7"/>
       <c r="I45" s="5"/>
-      <c r="J45" s="8" t="str">
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="8" t="str">
         <f aca="true">IF(A45="","",IF(I45="Hidden","Hidden",IF(AND(H45&lt;&gt;"",H45&gt;TODAY()),"Scheduled",IF(IF(C45&lt;&gt;"",C45,B45)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16347,7 +16503,9 @@
       <c r="G46" s="5"/>
       <c r="H46" s="7"/>
       <c r="I46" s="5"/>
-      <c r="J46" s="8" t="str">
+      <c r="J46" s="5"/>
+      <c r="K46" s="5"/>
+      <c r="L46" s="8" t="str">
         <f aca="true">IF(A46="","",IF(I46="Hidden","Hidden",IF(AND(H46&lt;&gt;"",H46&gt;TODAY()),"Scheduled",IF(IF(C46&lt;&gt;"",C46,B46)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16362,7 +16520,9 @@
       <c r="G47" s="5"/>
       <c r="H47" s="7"/>
       <c r="I47" s="5"/>
-      <c r="J47" s="8" t="str">
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="8" t="str">
         <f aca="true">IF(A47="","",IF(I47="Hidden","Hidden",IF(AND(H47&lt;&gt;"",H47&gt;TODAY()),"Scheduled",IF(IF(C47&lt;&gt;"",C47,B47)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16377,7 +16537,9 @@
       <c r="G48" s="5"/>
       <c r="H48" s="7"/>
       <c r="I48" s="5"/>
-      <c r="J48" s="8" t="str">
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="8" t="str">
         <f aca="true">IF(A48="","",IF(I48="Hidden","Hidden",IF(AND(H48&lt;&gt;"",H48&gt;TODAY()),"Scheduled",IF(IF(C48&lt;&gt;"",C48,B48)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16392,7 +16554,9 @@
       <c r="G49" s="5"/>
       <c r="H49" s="7"/>
       <c r="I49" s="5"/>
-      <c r="J49" s="8" t="str">
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="8" t="str">
         <f aca="true">IF(A49="","",IF(I49="Hidden","Hidden",IF(AND(H49&lt;&gt;"",H49&gt;TODAY()),"Scheduled",IF(IF(C49&lt;&gt;"",C49,B49)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16407,7 +16571,9 @@
       <c r="G50" s="5"/>
       <c r="H50" s="7"/>
       <c r="I50" s="5"/>
-      <c r="J50" s="8" t="str">
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="8" t="str">
         <f aca="true">IF(A50="","",IF(I50="Hidden","Hidden",IF(AND(H50&lt;&gt;"",H50&gt;TODAY()),"Scheduled",IF(IF(C50&lt;&gt;"",C50,B50)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16422,7 +16588,9 @@
       <c r="G51" s="5"/>
       <c r="H51" s="7"/>
       <c r="I51" s="5"/>
-      <c r="J51" s="8" t="str">
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="8" t="str">
         <f aca="true">IF(A51="","",IF(I51="Hidden","Hidden",IF(AND(H51&lt;&gt;"",H51&gt;TODAY()),"Scheduled",IF(IF(C51&lt;&gt;"",C51,B51)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16437,7 +16605,9 @@
       <c r="G52" s="5"/>
       <c r="H52" s="7"/>
       <c r="I52" s="5"/>
-      <c r="J52" s="8" t="str">
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="8" t="str">
         <f aca="true">IF(A52="","",IF(I52="Hidden","Hidden",IF(AND(H52&lt;&gt;"",H52&gt;TODAY()),"Scheduled",IF(IF(C52&lt;&gt;"",C52,B52)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16452,7 +16622,9 @@
       <c r="G53" s="5"/>
       <c r="H53" s="7"/>
       <c r="I53" s="5"/>
-      <c r="J53" s="8" t="str">
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+      <c r="L53" s="8" t="str">
         <f aca="true">IF(A53="","",IF(I53="Hidden","Hidden",IF(AND(H53&lt;&gt;"",H53&gt;TODAY()),"Scheduled",IF(IF(C53&lt;&gt;"",C53,B53)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16467,7 +16639,9 @@
       <c r="G54" s="5"/>
       <c r="H54" s="7"/>
       <c r="I54" s="5"/>
-      <c r="J54" s="8" t="str">
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="8" t="str">
         <f aca="true">IF(A54="","",IF(I54="Hidden","Hidden",IF(AND(H54&lt;&gt;"",H54&gt;TODAY()),"Scheduled",IF(IF(C54&lt;&gt;"",C54,B54)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16482,7 +16656,9 @@
       <c r="G55" s="5"/>
       <c r="H55" s="7"/>
       <c r="I55" s="5"/>
-      <c r="J55" s="8" t="str">
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="8" t="str">
         <f aca="true">IF(A55="","",IF(I55="Hidden","Hidden",IF(AND(H55&lt;&gt;"",H55&gt;TODAY()),"Scheduled",IF(IF(C55&lt;&gt;"",C55,B55)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16497,7 +16673,9 @@
       <c r="G56" s="5"/>
       <c r="H56" s="7"/>
       <c r="I56" s="5"/>
-      <c r="J56" s="8" t="str">
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="8" t="str">
         <f aca="true">IF(A56="","",IF(I56="Hidden","Hidden",IF(AND(H56&lt;&gt;"",H56&gt;TODAY()),"Scheduled",IF(IF(C56&lt;&gt;"",C56,B56)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16512,7 +16690,9 @@
       <c r="G57" s="5"/>
       <c r="H57" s="7"/>
       <c r="I57" s="5"/>
-      <c r="J57" s="8" t="str">
+      <c r="J57" s="5"/>
+      <c r="K57" s="5"/>
+      <c r="L57" s="8" t="str">
         <f aca="true">IF(A57="","",IF(I57="Hidden","Hidden",IF(AND(H57&lt;&gt;"",H57&gt;TODAY()),"Scheduled",IF(IF(C57&lt;&gt;"",C57,B57)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16527,7 +16707,9 @@
       <c r="G58" s="5"/>
       <c r="H58" s="7"/>
       <c r="I58" s="5"/>
-      <c r="J58" s="8" t="str">
+      <c r="J58" s="5"/>
+      <c r="K58" s="5"/>
+      <c r="L58" s="8" t="str">
         <f aca="true">IF(A58="","",IF(I58="Hidden","Hidden",IF(AND(H58&lt;&gt;"",H58&gt;TODAY()),"Scheduled",IF(IF(C58&lt;&gt;"",C58,B58)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16542,7 +16724,9 @@
       <c r="G59" s="5"/>
       <c r="H59" s="7"/>
       <c r="I59" s="5"/>
-      <c r="J59" s="8" t="str">
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+      <c r="L59" s="8" t="str">
         <f aca="true">IF(A59="","",IF(I59="Hidden","Hidden",IF(AND(H59&lt;&gt;"",H59&gt;TODAY()),"Scheduled",IF(IF(C59&lt;&gt;"",C59,B59)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16557,7 +16741,9 @@
       <c r="G60" s="5"/>
       <c r="H60" s="7"/>
       <c r="I60" s="5"/>
-      <c r="J60" s="8" t="str">
+      <c r="J60" s="5"/>
+      <c r="K60" s="5"/>
+      <c r="L60" s="8" t="str">
         <f aca="true">IF(A60="","",IF(I60="Hidden","Hidden",IF(AND(H60&lt;&gt;"",H60&gt;TODAY()),"Scheduled",IF(IF(C60&lt;&gt;"",C60,B60)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16572,7 +16758,9 @@
       <c r="G61" s="5"/>
       <c r="H61" s="7"/>
       <c r="I61" s="5"/>
-      <c r="J61" s="8" t="str">
+      <c r="J61" s="5"/>
+      <c r="K61" s="5"/>
+      <c r="L61" s="8" t="str">
         <f aca="true">IF(A61="","",IF(I61="Hidden","Hidden",IF(AND(H61&lt;&gt;"",H61&gt;TODAY()),"Scheduled",IF(IF(C61&lt;&gt;"",C61,B61)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16587,7 +16775,9 @@
       <c r="G62" s="5"/>
       <c r="H62" s="7"/>
       <c r="I62" s="5"/>
-      <c r="J62" s="8" t="str">
+      <c r="J62" s="5"/>
+      <c r="K62" s="5"/>
+      <c r="L62" s="8" t="str">
         <f aca="true">IF(A62="","",IF(I62="Hidden","Hidden",IF(AND(H62&lt;&gt;"",H62&gt;TODAY()),"Scheduled",IF(IF(C62&lt;&gt;"",C62,B62)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16602,7 +16792,9 @@
       <c r="G63" s="5"/>
       <c r="H63" s="7"/>
       <c r="I63" s="5"/>
-      <c r="J63" s="8" t="str">
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+      <c r="L63" s="8" t="str">
         <f aca="true">IF(A63="","",IF(I63="Hidden","Hidden",IF(AND(H63&lt;&gt;"",H63&gt;TODAY()),"Scheduled",IF(IF(C63&lt;&gt;"",C63,B63)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16617,7 +16809,9 @@
       <c r="G64" s="5"/>
       <c r="H64" s="7"/>
       <c r="I64" s="5"/>
-      <c r="J64" s="8" t="str">
+      <c r="J64" s="5"/>
+      <c r="K64" s="5"/>
+      <c r="L64" s="8" t="str">
         <f aca="true">IF(A64="","",IF(I64="Hidden","Hidden",IF(AND(H64&lt;&gt;"",H64&gt;TODAY()),"Scheduled",IF(IF(C64&lt;&gt;"",C64,B64)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16632,7 +16826,9 @@
       <c r="G65" s="5"/>
       <c r="H65" s="7"/>
       <c r="I65" s="5"/>
-      <c r="J65" s="8" t="str">
+      <c r="J65" s="5"/>
+      <c r="K65" s="5"/>
+      <c r="L65" s="8" t="str">
         <f aca="true">IF(A65="","",IF(I65="Hidden","Hidden",IF(AND(H65&lt;&gt;"",H65&gt;TODAY()),"Scheduled",IF(IF(C65&lt;&gt;"",C65,B65)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16647,7 +16843,9 @@
       <c r="G66" s="5"/>
       <c r="H66" s="7"/>
       <c r="I66" s="5"/>
-      <c r="J66" s="8" t="str">
+      <c r="J66" s="5"/>
+      <c r="K66" s="5"/>
+      <c r="L66" s="8" t="str">
         <f aca="true">IF(A66="","",IF(I66="Hidden","Hidden",IF(AND(H66&lt;&gt;"",H66&gt;TODAY()),"Scheduled",IF(IF(C66&lt;&gt;"",C66,B66)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16662,7 +16860,9 @@
       <c r="G67" s="5"/>
       <c r="H67" s="7"/>
       <c r="I67" s="5"/>
-      <c r="J67" s="8" t="str">
+      <c r="J67" s="5"/>
+      <c r="K67" s="5"/>
+      <c r="L67" s="8" t="str">
         <f aca="true">IF(A67="","",IF(I67="Hidden","Hidden",IF(AND(H67&lt;&gt;"",H67&gt;TODAY()),"Scheduled",IF(IF(C67&lt;&gt;"",C67,B67)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16677,7 +16877,9 @@
       <c r="G68" s="5"/>
       <c r="H68" s="7"/>
       <c r="I68" s="5"/>
-      <c r="J68" s="8" t="str">
+      <c r="J68" s="5"/>
+      <c r="K68" s="5"/>
+      <c r="L68" s="8" t="str">
         <f aca="true">IF(A68="","",IF(I68="Hidden","Hidden",IF(AND(H68&lt;&gt;"",H68&gt;TODAY()),"Scheduled",IF(IF(C68&lt;&gt;"",C68,B68)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16692,7 +16894,9 @@
       <c r="G69" s="5"/>
       <c r="H69" s="7"/>
       <c r="I69" s="5"/>
-      <c r="J69" s="8" t="str">
+      <c r="J69" s="5"/>
+      <c r="K69" s="5"/>
+      <c r="L69" s="8" t="str">
         <f aca="true">IF(A69="","",IF(I69="Hidden","Hidden",IF(AND(H69&lt;&gt;"",H69&gt;TODAY()),"Scheduled",IF(IF(C69&lt;&gt;"",C69,B69)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16707,7 +16911,9 @@
       <c r="G70" s="5"/>
       <c r="H70" s="7"/>
       <c r="I70" s="5"/>
-      <c r="J70" s="8" t="str">
+      <c r="J70" s="5"/>
+      <c r="K70" s="5"/>
+      <c r="L70" s="8" t="str">
         <f aca="true">IF(A70="","",IF(I70="Hidden","Hidden",IF(AND(H70&lt;&gt;"",H70&gt;TODAY()),"Scheduled",IF(IF(C70&lt;&gt;"",C70,B70)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16722,7 +16928,9 @@
       <c r="G71" s="5"/>
       <c r="H71" s="7"/>
       <c r="I71" s="5"/>
-      <c r="J71" s="8" t="str">
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+      <c r="L71" s="8" t="str">
         <f aca="true">IF(A71="","",IF(I71="Hidden","Hidden",IF(AND(H71&lt;&gt;"",H71&gt;TODAY()),"Scheduled",IF(IF(C71&lt;&gt;"",C71,B71)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16737,7 +16945,9 @@
       <c r="G72" s="5"/>
       <c r="H72" s="7"/>
       <c r="I72" s="5"/>
-      <c r="J72" s="8" t="str">
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+      <c r="L72" s="8" t="str">
         <f aca="true">IF(A72="","",IF(I72="Hidden","Hidden",IF(AND(H72&lt;&gt;"",H72&gt;TODAY()),"Scheduled",IF(IF(C72&lt;&gt;"",C72,B72)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16752,7 +16962,9 @@
       <c r="G73" s="5"/>
       <c r="H73" s="7"/>
       <c r="I73" s="5"/>
-      <c r="J73" s="8" t="str">
+      <c r="J73" s="5"/>
+      <c r="K73" s="5"/>
+      <c r="L73" s="8" t="str">
         <f aca="true">IF(A73="","",IF(I73="Hidden","Hidden",IF(AND(H73&lt;&gt;"",H73&gt;TODAY()),"Scheduled",IF(IF(C73&lt;&gt;"",C73,B73)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16767,7 +16979,9 @@
       <c r="G74" s="5"/>
       <c r="H74" s="7"/>
       <c r="I74" s="5"/>
-      <c r="J74" s="8" t="str">
+      <c r="J74" s="5"/>
+      <c r="K74" s="5"/>
+      <c r="L74" s="8" t="str">
         <f aca="true">IF(A74="","",IF(I74="Hidden","Hidden",IF(AND(H74&lt;&gt;"",H74&gt;TODAY()),"Scheduled",IF(IF(C74&lt;&gt;"",C74,B74)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16782,7 +16996,9 @@
       <c r="G75" s="5"/>
       <c r="H75" s="7"/>
       <c r="I75" s="5"/>
-      <c r="J75" s="8" t="str">
+      <c r="J75" s="5"/>
+      <c r="K75" s="5"/>
+      <c r="L75" s="8" t="str">
         <f aca="true">IF(A75="","",IF(I75="Hidden","Hidden",IF(AND(H75&lt;&gt;"",H75&gt;TODAY()),"Scheduled",IF(IF(C75&lt;&gt;"",C75,B75)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16797,7 +17013,9 @@
       <c r="G76" s="5"/>
       <c r="H76" s="7"/>
       <c r="I76" s="5"/>
-      <c r="J76" s="8" t="str">
+      <c r="J76" s="5"/>
+      <c r="K76" s="5"/>
+      <c r="L76" s="8" t="str">
         <f aca="true">IF(A76="","",IF(I76="Hidden","Hidden",IF(AND(H76&lt;&gt;"",H76&gt;TODAY()),"Scheduled",IF(IF(C76&lt;&gt;"",C76,B76)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16812,7 +17030,9 @@
       <c r="G77" s="5"/>
       <c r="H77" s="7"/>
       <c r="I77" s="5"/>
-      <c r="J77" s="8" t="str">
+      <c r="J77" s="5"/>
+      <c r="K77" s="5"/>
+      <c r="L77" s="8" t="str">
         <f aca="true">IF(A77="","",IF(I77="Hidden","Hidden",IF(AND(H77&lt;&gt;"",H77&gt;TODAY()),"Scheduled",IF(IF(C77&lt;&gt;"",C77,B77)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16827,7 +17047,9 @@
       <c r="G78" s="5"/>
       <c r="H78" s="7"/>
       <c r="I78" s="5"/>
-      <c r="J78" s="8" t="str">
+      <c r="J78" s="5"/>
+      <c r="K78" s="5"/>
+      <c r="L78" s="8" t="str">
         <f aca="true">IF(A78="","",IF(I78="Hidden","Hidden",IF(AND(H78&lt;&gt;"",H78&gt;TODAY()),"Scheduled",IF(IF(C78&lt;&gt;"",C78,B78)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16842,7 +17064,9 @@
       <c r="G79" s="5"/>
       <c r="H79" s="7"/>
       <c r="I79" s="5"/>
-      <c r="J79" s="8" t="str">
+      <c r="J79" s="5"/>
+      <c r="K79" s="5"/>
+      <c r="L79" s="8" t="str">
         <f aca="true">IF(A79="","",IF(I79="Hidden","Hidden",IF(AND(H79&lt;&gt;"",H79&gt;TODAY()),"Scheduled",IF(IF(C79&lt;&gt;"",C79,B79)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16857,7 +17081,9 @@
       <c r="G80" s="5"/>
       <c r="H80" s="7"/>
       <c r="I80" s="5"/>
-      <c r="J80" s="8" t="str">
+      <c r="J80" s="5"/>
+      <c r="K80" s="5"/>
+      <c r="L80" s="8" t="str">
         <f aca="true">IF(A80="","",IF(I80="Hidden","Hidden",IF(AND(H80&lt;&gt;"",H80&gt;TODAY()),"Scheduled",IF(IF(C80&lt;&gt;"",C80,B80)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16872,7 +17098,9 @@
       <c r="G81" s="5"/>
       <c r="H81" s="7"/>
       <c r="I81" s="5"/>
-      <c r="J81" s="8" t="str">
+      <c r="J81" s="5"/>
+      <c r="K81" s="5"/>
+      <c r="L81" s="8" t="str">
         <f aca="true">IF(A81="","",IF(I81="Hidden","Hidden",IF(AND(H81&lt;&gt;"",H81&gt;TODAY()),"Scheduled",IF(IF(C81&lt;&gt;"",C81,B81)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16887,7 +17115,9 @@
       <c r="G82" s="5"/>
       <c r="H82" s="7"/>
       <c r="I82" s="5"/>
-      <c r="J82" s="8" t="str">
+      <c r="J82" s="5"/>
+      <c r="K82" s="5"/>
+      <c r="L82" s="8" t="str">
         <f aca="true">IF(A82="","",IF(I82="Hidden","Hidden",IF(AND(H82&lt;&gt;"",H82&gt;TODAY()),"Scheduled",IF(IF(C82&lt;&gt;"",C82,B82)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16902,7 +17132,9 @@
       <c r="G83" s="5"/>
       <c r="H83" s="7"/>
       <c r="I83" s="5"/>
-      <c r="J83" s="8" t="str">
+      <c r="J83" s="5"/>
+      <c r="K83" s="5"/>
+      <c r="L83" s="8" t="str">
         <f aca="true">IF(A83="","",IF(I83="Hidden","Hidden",IF(AND(H83&lt;&gt;"",H83&gt;TODAY()),"Scheduled",IF(IF(C83&lt;&gt;"",C83,B83)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16917,7 +17149,9 @@
       <c r="G84" s="5"/>
       <c r="H84" s="7"/>
       <c r="I84" s="5"/>
-      <c r="J84" s="8" t="str">
+      <c r="J84" s="5"/>
+      <c r="K84" s="5"/>
+      <c r="L84" s="8" t="str">
         <f aca="true">IF(A84="","",IF(I84="Hidden","Hidden",IF(AND(H84&lt;&gt;"",H84&gt;TODAY()),"Scheduled",IF(IF(C84&lt;&gt;"",C84,B84)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16932,7 +17166,9 @@
       <c r="G85" s="5"/>
       <c r="H85" s="7"/>
       <c r="I85" s="5"/>
-      <c r="J85" s="8" t="str">
+      <c r="J85" s="5"/>
+      <c r="K85" s="5"/>
+      <c r="L85" s="8" t="str">
         <f aca="true">IF(A85="","",IF(I85="Hidden","Hidden",IF(AND(H85&lt;&gt;"",H85&gt;TODAY()),"Scheduled",IF(IF(C85&lt;&gt;"",C85,B85)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16947,7 +17183,9 @@
       <c r="G86" s="5"/>
       <c r="H86" s="7"/>
       <c r="I86" s="5"/>
-      <c r="J86" s="8" t="str">
+      <c r="J86" s="5"/>
+      <c r="K86" s="5"/>
+      <c r="L86" s="8" t="str">
         <f aca="true">IF(A86="","",IF(I86="Hidden","Hidden",IF(AND(H86&lt;&gt;"",H86&gt;TODAY()),"Scheduled",IF(IF(C86&lt;&gt;"",C86,B86)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16962,7 +17200,9 @@
       <c r="G87" s="5"/>
       <c r="H87" s="7"/>
       <c r="I87" s="5"/>
-      <c r="J87" s="8" t="str">
+      <c r="J87" s="5"/>
+      <c r="K87" s="5"/>
+      <c r="L87" s="8" t="str">
         <f aca="true">IF(A87="","",IF(I87="Hidden","Hidden",IF(AND(H87&lt;&gt;"",H87&gt;TODAY()),"Scheduled",IF(IF(C87&lt;&gt;"",C87,B87)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16977,7 +17217,9 @@
       <c r="G88" s="5"/>
       <c r="H88" s="7"/>
       <c r="I88" s="5"/>
-      <c r="J88" s="8" t="str">
+      <c r="J88" s="5"/>
+      <c r="K88" s="5"/>
+      <c r="L88" s="8" t="str">
         <f aca="true">IF(A88="","",IF(I88="Hidden","Hidden",IF(AND(H88&lt;&gt;"",H88&gt;TODAY()),"Scheduled",IF(IF(C88&lt;&gt;"",C88,B88)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -16992,7 +17234,9 @@
       <c r="G89" s="5"/>
       <c r="H89" s="7"/>
       <c r="I89" s="5"/>
-      <c r="J89" s="8" t="str">
+      <c r="J89" s="5"/>
+      <c r="K89" s="5"/>
+      <c r="L89" s="8" t="str">
         <f aca="true">IF(A89="","",IF(I89="Hidden","Hidden",IF(AND(H89&lt;&gt;"",H89&gt;TODAY()),"Scheduled",IF(IF(C89&lt;&gt;"",C89,B89)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17007,7 +17251,9 @@
       <c r="G90" s="5"/>
       <c r="H90" s="7"/>
       <c r="I90" s="5"/>
-      <c r="J90" s="8" t="str">
+      <c r="J90" s="5"/>
+      <c r="K90" s="5"/>
+      <c r="L90" s="8" t="str">
         <f aca="true">IF(A90="","",IF(I90="Hidden","Hidden",IF(AND(H90&lt;&gt;"",H90&gt;TODAY()),"Scheduled",IF(IF(C90&lt;&gt;"",C90,B90)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17022,7 +17268,9 @@
       <c r="G91" s="5"/>
       <c r="H91" s="7"/>
       <c r="I91" s="5"/>
-      <c r="J91" s="8" t="str">
+      <c r="J91" s="5"/>
+      <c r="K91" s="5"/>
+      <c r="L91" s="8" t="str">
         <f aca="true">IF(A91="","",IF(I91="Hidden","Hidden",IF(AND(H91&lt;&gt;"",H91&gt;TODAY()),"Scheduled",IF(IF(C91&lt;&gt;"",C91,B91)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17037,7 +17285,9 @@
       <c r="G92" s="5"/>
       <c r="H92" s="7"/>
       <c r="I92" s="5"/>
-      <c r="J92" s="8" t="str">
+      <c r="J92" s="5"/>
+      <c r="K92" s="5"/>
+      <c r="L92" s="8" t="str">
         <f aca="true">IF(A92="","",IF(I92="Hidden","Hidden",IF(AND(H92&lt;&gt;"",H92&gt;TODAY()),"Scheduled",IF(IF(C92&lt;&gt;"",C92,B92)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17052,7 +17302,9 @@
       <c r="G93" s="5"/>
       <c r="H93" s="7"/>
       <c r="I93" s="5"/>
-      <c r="J93" s="8" t="str">
+      <c r="J93" s="5"/>
+      <c r="K93" s="5"/>
+      <c r="L93" s="8" t="str">
         <f aca="true">IF(A93="","",IF(I93="Hidden","Hidden",IF(AND(H93&lt;&gt;"",H93&gt;TODAY()),"Scheduled",IF(IF(C93&lt;&gt;"",C93,B93)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17067,7 +17319,9 @@
       <c r="G94" s="5"/>
       <c r="H94" s="7"/>
       <c r="I94" s="5"/>
-      <c r="J94" s="8" t="str">
+      <c r="J94" s="5"/>
+      <c r="K94" s="5"/>
+      <c r="L94" s="8" t="str">
         <f aca="true">IF(A94="","",IF(I94="Hidden","Hidden",IF(AND(H94&lt;&gt;"",H94&gt;TODAY()),"Scheduled",IF(IF(C94&lt;&gt;"",C94,B94)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17082,7 +17336,9 @@
       <c r="G95" s="5"/>
       <c r="H95" s="7"/>
       <c r="I95" s="5"/>
-      <c r="J95" s="8" t="str">
+      <c r="J95" s="5"/>
+      <c r="K95" s="5"/>
+      <c r="L95" s="8" t="str">
         <f aca="true">IF(A95="","",IF(I95="Hidden","Hidden",IF(AND(H95&lt;&gt;"",H95&gt;TODAY()),"Scheduled",IF(IF(C95&lt;&gt;"",C95,B95)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17097,7 +17353,9 @@
       <c r="G96" s="5"/>
       <c r="H96" s="7"/>
       <c r="I96" s="5"/>
-      <c r="J96" s="8" t="str">
+      <c r="J96" s="5"/>
+      <c r="K96" s="5"/>
+      <c r="L96" s="8" t="str">
         <f aca="true">IF(A96="","",IF(I96="Hidden","Hidden",IF(AND(H96&lt;&gt;"",H96&gt;TODAY()),"Scheduled",IF(IF(C96&lt;&gt;"",C96,B96)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17112,7 +17370,9 @@
       <c r="G97" s="5"/>
       <c r="H97" s="7"/>
       <c r="I97" s="5"/>
-      <c r="J97" s="8" t="str">
+      <c r="J97" s="5"/>
+      <c r="K97" s="5"/>
+      <c r="L97" s="8" t="str">
         <f aca="true">IF(A97="","",IF(I97="Hidden","Hidden",IF(AND(H97&lt;&gt;"",H97&gt;TODAY()),"Scheduled",IF(IF(C97&lt;&gt;"",C97,B97)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17127,7 +17387,9 @@
       <c r="G98" s="5"/>
       <c r="H98" s="7"/>
       <c r="I98" s="5"/>
-      <c r="J98" s="8" t="str">
+      <c r="J98" s="5"/>
+      <c r="K98" s="5"/>
+      <c r="L98" s="8" t="str">
         <f aca="true">IF(A98="","",IF(I98="Hidden","Hidden",IF(AND(H98&lt;&gt;"",H98&gt;TODAY()),"Scheduled",IF(IF(C98&lt;&gt;"",C98,B98)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17142,7 +17404,9 @@
       <c r="G99" s="5"/>
       <c r="H99" s="7"/>
       <c r="I99" s="5"/>
-      <c r="J99" s="8" t="str">
+      <c r="J99" s="5"/>
+      <c r="K99" s="5"/>
+      <c r="L99" s="8" t="str">
         <f aca="true">IF(A99="","",IF(I99="Hidden","Hidden",IF(AND(H99&lt;&gt;"",H99&gt;TODAY()),"Scheduled",IF(IF(C99&lt;&gt;"",C99,B99)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17157,7 +17421,9 @@
       <c r="G100" s="5"/>
       <c r="H100" s="7"/>
       <c r="I100" s="5"/>
-      <c r="J100" s="8" t="str">
+      <c r="J100" s="5"/>
+      <c r="K100" s="5"/>
+      <c r="L100" s="8" t="str">
         <f aca="true">IF(A100="","",IF(I100="Hidden","Hidden",IF(AND(H100&lt;&gt;"",H100&gt;TODAY()),"Scheduled",IF(IF(C100&lt;&gt;"",C100,B100)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17172,7 +17438,9 @@
       <c r="G101" s="5"/>
       <c r="H101" s="7"/>
       <c r="I101" s="5"/>
-      <c r="J101" s="8" t="str">
+      <c r="J101" s="5"/>
+      <c r="K101" s="5"/>
+      <c r="L101" s="8" t="str">
         <f aca="true">IF(A101="","",IF(I101="Hidden","Hidden",IF(AND(H101&lt;&gt;"",H101&gt;TODAY()),"Scheduled",IF(IF(C101&lt;&gt;"",C101,B101)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17187,7 +17455,9 @@
       <c r="G102" s="5"/>
       <c r="H102" s="7"/>
       <c r="I102" s="5"/>
-      <c r="J102" s="8" t="str">
+      <c r="J102" s="5"/>
+      <c r="K102" s="5"/>
+      <c r="L102" s="8" t="str">
         <f aca="true">IF(A102="","",IF(I102="Hidden","Hidden",IF(AND(H102&lt;&gt;"",H102&gt;TODAY()),"Scheduled",IF(IF(C102&lt;&gt;"",C102,B102)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17202,7 +17472,9 @@
       <c r="G103" s="5"/>
       <c r="H103" s="7"/>
       <c r="I103" s="5"/>
-      <c r="J103" s="8" t="str">
+      <c r="J103" s="5"/>
+      <c r="K103" s="5"/>
+      <c r="L103" s="8" t="str">
         <f aca="true">IF(A103="","",IF(I103="Hidden","Hidden",IF(AND(H103&lt;&gt;"",H103&gt;TODAY()),"Scheduled",IF(IF(C103&lt;&gt;"",C103,B103)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17217,7 +17489,9 @@
       <c r="G104" s="5"/>
       <c r="H104" s="7"/>
       <c r="I104" s="5"/>
-      <c r="J104" s="8" t="str">
+      <c r="J104" s="5"/>
+      <c r="K104" s="5"/>
+      <c r="L104" s="8" t="str">
         <f aca="true">IF(A104="","",IF(I104="Hidden","Hidden",IF(AND(H104&lt;&gt;"",H104&gt;TODAY()),"Scheduled",IF(IF(C104&lt;&gt;"",C104,B104)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17232,7 +17506,9 @@
       <c r="G105" s="5"/>
       <c r="H105" s="7"/>
       <c r="I105" s="5"/>
-      <c r="J105" s="8" t="str">
+      <c r="J105" s="5"/>
+      <c r="K105" s="5"/>
+      <c r="L105" s="8" t="str">
         <f aca="true">IF(A105="","",IF(I105="Hidden","Hidden",IF(AND(H105&lt;&gt;"",H105&gt;TODAY()),"Scheduled",IF(IF(C105&lt;&gt;"",C105,B105)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17247,7 +17523,9 @@
       <c r="G106" s="5"/>
       <c r="H106" s="7"/>
       <c r="I106" s="5"/>
-      <c r="J106" s="8" t="str">
+      <c r="J106" s="5"/>
+      <c r="K106" s="5"/>
+      <c r="L106" s="8" t="str">
         <f aca="true">IF(A106="","",IF(I106="Hidden","Hidden",IF(AND(H106&lt;&gt;"",H106&gt;TODAY()),"Scheduled",IF(IF(C106&lt;&gt;"",C106,B106)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17262,7 +17540,9 @@
       <c r="G107" s="5"/>
       <c r="H107" s="7"/>
       <c r="I107" s="5"/>
-      <c r="J107" s="8" t="str">
+      <c r="J107" s="5"/>
+      <c r="K107" s="5"/>
+      <c r="L107" s="8" t="str">
         <f aca="true">IF(A107="","",IF(I107="Hidden","Hidden",IF(AND(H107&lt;&gt;"",H107&gt;TODAY()),"Scheduled",IF(IF(C107&lt;&gt;"",C107,B107)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17277,7 +17557,9 @@
       <c r="G108" s="5"/>
       <c r="H108" s="7"/>
       <c r="I108" s="5"/>
-      <c r="J108" s="8" t="str">
+      <c r="J108" s="5"/>
+      <c r="K108" s="5"/>
+      <c r="L108" s="8" t="str">
         <f aca="true">IF(A108="","",IF(I108="Hidden","Hidden",IF(AND(H108&lt;&gt;"",H108&gt;TODAY()),"Scheduled",IF(IF(C108&lt;&gt;"",C108,B108)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17292,7 +17574,9 @@
       <c r="G109" s="5"/>
       <c r="H109" s="7"/>
       <c r="I109" s="5"/>
-      <c r="J109" s="8" t="str">
+      <c r="J109" s="5"/>
+      <c r="K109" s="5"/>
+      <c r="L109" s="8" t="str">
         <f aca="true">IF(A109="","",IF(I109="Hidden","Hidden",IF(AND(H109&lt;&gt;"",H109&gt;TODAY()),"Scheduled",IF(IF(C109&lt;&gt;"",C109,B109)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17307,7 +17591,9 @@
       <c r="G110" s="5"/>
       <c r="H110" s="7"/>
       <c r="I110" s="5"/>
-      <c r="J110" s="8" t="str">
+      <c r="J110" s="5"/>
+      <c r="K110" s="5"/>
+      <c r="L110" s="8" t="str">
         <f aca="true">IF(A110="","",IF(I110="Hidden","Hidden",IF(AND(H110&lt;&gt;"",H110&gt;TODAY()),"Scheduled",IF(IF(C110&lt;&gt;"",C110,B110)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17322,7 +17608,9 @@
       <c r="G111" s="5"/>
       <c r="H111" s="7"/>
       <c r="I111" s="5"/>
-      <c r="J111" s="8" t="str">
+      <c r="J111" s="5"/>
+      <c r="K111" s="5"/>
+      <c r="L111" s="8" t="str">
         <f aca="true">IF(A111="","",IF(I111="Hidden","Hidden",IF(AND(H111&lt;&gt;"",H111&gt;TODAY()),"Scheduled",IF(IF(C111&lt;&gt;"",C111,B111)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17337,7 +17625,9 @@
       <c r="G112" s="5"/>
       <c r="H112" s="7"/>
       <c r="I112" s="5"/>
-      <c r="J112" s="8" t="str">
+      <c r="J112" s="5"/>
+      <c r="K112" s="5"/>
+      <c r="L112" s="8" t="str">
         <f aca="true">IF(A112="","",IF(I112="Hidden","Hidden",IF(AND(H112&lt;&gt;"",H112&gt;TODAY()),"Scheduled",IF(IF(C112&lt;&gt;"",C112,B112)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17352,7 +17642,9 @@
       <c r="G113" s="5"/>
       <c r="H113" s="7"/>
       <c r="I113" s="5"/>
-      <c r="J113" s="8" t="str">
+      <c r="J113" s="5"/>
+      <c r="K113" s="5"/>
+      <c r="L113" s="8" t="str">
         <f aca="true">IF(A113="","",IF(I113="Hidden","Hidden",IF(AND(H113&lt;&gt;"",H113&gt;TODAY()),"Scheduled",IF(IF(C113&lt;&gt;"",C113,B113)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17367,7 +17659,9 @@
       <c r="G114" s="5"/>
       <c r="H114" s="7"/>
       <c r="I114" s="5"/>
-      <c r="J114" s="8" t="str">
+      <c r="J114" s="5"/>
+      <c r="K114" s="5"/>
+      <c r="L114" s="8" t="str">
         <f aca="true">IF(A114="","",IF(I114="Hidden","Hidden",IF(AND(H114&lt;&gt;"",H114&gt;TODAY()),"Scheduled",IF(IF(C114&lt;&gt;"",C114,B114)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17382,7 +17676,9 @@
       <c r="G115" s="5"/>
       <c r="H115" s="7"/>
       <c r="I115" s="5"/>
-      <c r="J115" s="8" t="str">
+      <c r="J115" s="5"/>
+      <c r="K115" s="5"/>
+      <c r="L115" s="8" t="str">
         <f aca="true">IF(A115="","",IF(I115="Hidden","Hidden",IF(AND(H115&lt;&gt;"",H115&gt;TODAY()),"Scheduled",IF(IF(C115&lt;&gt;"",C115,B115)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17397,7 +17693,9 @@
       <c r="G116" s="5"/>
       <c r="H116" s="7"/>
       <c r="I116" s="5"/>
-      <c r="J116" s="8" t="str">
+      <c r="J116" s="5"/>
+      <c r="K116" s="5"/>
+      <c r="L116" s="8" t="str">
         <f aca="true">IF(A116="","",IF(I116="Hidden","Hidden",IF(AND(H116&lt;&gt;"",H116&gt;TODAY()),"Scheduled",IF(IF(C116&lt;&gt;"",C116,B116)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17412,7 +17710,9 @@
       <c r="G117" s="5"/>
       <c r="H117" s="7"/>
       <c r="I117" s="5"/>
-      <c r="J117" s="8" t="str">
+      <c r="J117" s="5"/>
+      <c r="K117" s="5"/>
+      <c r="L117" s="8" t="str">
         <f aca="true">IF(A117="","",IF(I117="Hidden","Hidden",IF(AND(H117&lt;&gt;"",H117&gt;TODAY()),"Scheduled",IF(IF(C117&lt;&gt;"",C117,B117)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17427,7 +17727,9 @@
       <c r="G118" s="5"/>
       <c r="H118" s="7"/>
       <c r="I118" s="5"/>
-      <c r="J118" s="8" t="str">
+      <c r="J118" s="5"/>
+      <c r="K118" s="5"/>
+      <c r="L118" s="8" t="str">
         <f aca="true">IF(A118="","",IF(I118="Hidden","Hidden",IF(AND(H118&lt;&gt;"",H118&gt;TODAY()),"Scheduled",IF(IF(C118&lt;&gt;"",C118,B118)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17442,7 +17744,9 @@
       <c r="G119" s="5"/>
       <c r="H119" s="7"/>
       <c r="I119" s="5"/>
-      <c r="J119" s="8" t="str">
+      <c r="J119" s="5"/>
+      <c r="K119" s="5"/>
+      <c r="L119" s="8" t="str">
         <f aca="true">IF(A119="","",IF(I119="Hidden","Hidden",IF(AND(H119&lt;&gt;"",H119&gt;TODAY()),"Scheduled",IF(IF(C119&lt;&gt;"",C119,B119)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17457,7 +17761,9 @@
       <c r="G120" s="5"/>
       <c r="H120" s="7"/>
       <c r="I120" s="5"/>
-      <c r="J120" s="8" t="str">
+      <c r="J120" s="5"/>
+      <c r="K120" s="5"/>
+      <c r="L120" s="8" t="str">
         <f aca="true">IF(A120="","",IF(I120="Hidden","Hidden",IF(AND(H120&lt;&gt;"",H120&gt;TODAY()),"Scheduled",IF(IF(C120&lt;&gt;"",C120,B120)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17472,7 +17778,9 @@
       <c r="G121" s="5"/>
       <c r="H121" s="7"/>
       <c r="I121" s="5"/>
-      <c r="J121" s="8" t="str">
+      <c r="J121" s="5"/>
+      <c r="K121" s="5"/>
+      <c r="L121" s="8" t="str">
         <f aca="true">IF(A121="","",IF(I121="Hidden","Hidden",IF(AND(H121&lt;&gt;"",H121&gt;TODAY()),"Scheduled",IF(IF(C121&lt;&gt;"",C121,B121)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17487,7 +17795,9 @@
       <c r="G122" s="5"/>
       <c r="H122" s="7"/>
       <c r="I122" s="5"/>
-      <c r="J122" s="8" t="str">
+      <c r="J122" s="5"/>
+      <c r="K122" s="5"/>
+      <c r="L122" s="8" t="str">
         <f aca="true">IF(A122="","",IF(I122="Hidden","Hidden",IF(AND(H122&lt;&gt;"",H122&gt;TODAY()),"Scheduled",IF(IF(C122&lt;&gt;"",C122,B122)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17502,7 +17812,9 @@
       <c r="G123" s="5"/>
       <c r="H123" s="7"/>
       <c r="I123" s="5"/>
-      <c r="J123" s="8" t="str">
+      <c r="J123" s="5"/>
+      <c r="K123" s="5"/>
+      <c r="L123" s="8" t="str">
         <f aca="true">IF(A123="","",IF(I123="Hidden","Hidden",IF(AND(H123&lt;&gt;"",H123&gt;TODAY()),"Scheduled",IF(IF(C123&lt;&gt;"",C123,B123)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17517,7 +17829,9 @@
       <c r="G124" s="5"/>
       <c r="H124" s="7"/>
       <c r="I124" s="5"/>
-      <c r="J124" s="8" t="str">
+      <c r="J124" s="5"/>
+      <c r="K124" s="5"/>
+      <c r="L124" s="8" t="str">
         <f aca="true">IF(A124="","",IF(I124="Hidden","Hidden",IF(AND(H124&lt;&gt;"",H124&gt;TODAY()),"Scheduled",IF(IF(C124&lt;&gt;"",C124,B124)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17532,7 +17846,9 @@
       <c r="G125" s="5"/>
       <c r="H125" s="7"/>
       <c r="I125" s="5"/>
-      <c r="J125" s="8" t="str">
+      <c r="J125" s="5"/>
+      <c r="K125" s="5"/>
+      <c r="L125" s="8" t="str">
         <f aca="true">IF(A125="","",IF(I125="Hidden","Hidden",IF(AND(H125&lt;&gt;"",H125&gt;TODAY()),"Scheduled",IF(IF(C125&lt;&gt;"",C125,B125)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17547,7 +17863,9 @@
       <c r="G126" s="5"/>
       <c r="H126" s="7"/>
       <c r="I126" s="5"/>
-      <c r="J126" s="8" t="str">
+      <c r="J126" s="5"/>
+      <c r="K126" s="5"/>
+      <c r="L126" s="8" t="str">
         <f aca="true">IF(A126="","",IF(I126="Hidden","Hidden",IF(AND(H126&lt;&gt;"",H126&gt;TODAY()),"Scheduled",IF(IF(C126&lt;&gt;"",C126,B126)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17562,7 +17880,9 @@
       <c r="G127" s="5"/>
       <c r="H127" s="7"/>
       <c r="I127" s="5"/>
-      <c r="J127" s="8" t="str">
+      <c r="J127" s="5"/>
+      <c r="K127" s="5"/>
+      <c r="L127" s="8" t="str">
         <f aca="true">IF(A127="","",IF(I127="Hidden","Hidden",IF(AND(H127&lt;&gt;"",H127&gt;TODAY()),"Scheduled",IF(IF(C127&lt;&gt;"",C127,B127)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17577,7 +17897,9 @@
       <c r="G128" s="5"/>
       <c r="H128" s="7"/>
       <c r="I128" s="5"/>
-      <c r="J128" s="8" t="str">
+      <c r="J128" s="5"/>
+      <c r="K128" s="5"/>
+      <c r="L128" s="8" t="str">
         <f aca="true">IF(A128="","",IF(I128="Hidden","Hidden",IF(AND(H128&lt;&gt;"",H128&gt;TODAY()),"Scheduled",IF(IF(C128&lt;&gt;"",C128,B128)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17592,7 +17914,9 @@
       <c r="G129" s="5"/>
       <c r="H129" s="7"/>
       <c r="I129" s="5"/>
-      <c r="J129" s="8" t="str">
+      <c r="J129" s="5"/>
+      <c r="K129" s="5"/>
+      <c r="L129" s="8" t="str">
         <f aca="true">IF(A129="","",IF(I129="Hidden","Hidden",IF(AND(H129&lt;&gt;"",H129&gt;TODAY()),"Scheduled",IF(IF(C129&lt;&gt;"",C129,B129)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17607,7 +17931,9 @@
       <c r="G130" s="5"/>
       <c r="H130" s="7"/>
       <c r="I130" s="5"/>
-      <c r="J130" s="8" t="str">
+      <c r="J130" s="5"/>
+      <c r="K130" s="5"/>
+      <c r="L130" s="8" t="str">
         <f aca="true">IF(A130="","",IF(I130="Hidden","Hidden",IF(AND(H130&lt;&gt;"",H130&gt;TODAY()),"Scheduled",IF(IF(C130&lt;&gt;"",C130,B130)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17622,7 +17948,9 @@
       <c r="G131" s="5"/>
       <c r="H131" s="7"/>
       <c r="I131" s="5"/>
-      <c r="J131" s="8" t="str">
+      <c r="J131" s="5"/>
+      <c r="K131" s="5"/>
+      <c r="L131" s="8" t="str">
         <f aca="true">IF(A131="","",IF(I131="Hidden","Hidden",IF(AND(H131&lt;&gt;"",H131&gt;TODAY()),"Scheduled",IF(IF(C131&lt;&gt;"",C131,B131)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17637,7 +17965,9 @@
       <c r="G132" s="5"/>
       <c r="H132" s="7"/>
       <c r="I132" s="5"/>
-      <c r="J132" s="8" t="str">
+      <c r="J132" s="5"/>
+      <c r="K132" s="5"/>
+      <c r="L132" s="8" t="str">
         <f aca="true">IF(A132="","",IF(I132="Hidden","Hidden",IF(AND(H132&lt;&gt;"",H132&gt;TODAY()),"Scheduled",IF(IF(C132&lt;&gt;"",C132,B132)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17652,7 +17982,9 @@
       <c r="G133" s="5"/>
       <c r="H133" s="7"/>
       <c r="I133" s="5"/>
-      <c r="J133" s="8" t="str">
+      <c r="J133" s="5"/>
+      <c r="K133" s="5"/>
+      <c r="L133" s="8" t="str">
         <f aca="true">IF(A133="","",IF(I133="Hidden","Hidden",IF(AND(H133&lt;&gt;"",H133&gt;TODAY()),"Scheduled",IF(IF(C133&lt;&gt;"",C133,B133)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17667,7 +17999,9 @@
       <c r="G134" s="5"/>
       <c r="H134" s="7"/>
       <c r="I134" s="5"/>
-      <c r="J134" s="8" t="str">
+      <c r="J134" s="5"/>
+      <c r="K134" s="5"/>
+      <c r="L134" s="8" t="str">
         <f aca="true">IF(A134="","",IF(I134="Hidden","Hidden",IF(AND(H134&lt;&gt;"",H134&gt;TODAY()),"Scheduled",IF(IF(C134&lt;&gt;"",C134,B134)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17682,7 +18016,9 @@
       <c r="G135" s="5"/>
       <c r="H135" s="7"/>
       <c r="I135" s="5"/>
-      <c r="J135" s="8" t="str">
+      <c r="J135" s="5"/>
+      <c r="K135" s="5"/>
+      <c r="L135" s="8" t="str">
         <f aca="true">IF(A135="","",IF(I135="Hidden","Hidden",IF(AND(H135&lt;&gt;"",H135&gt;TODAY()),"Scheduled",IF(IF(C135&lt;&gt;"",C135,B135)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17697,7 +18033,9 @@
       <c r="G136" s="5"/>
       <c r="H136" s="7"/>
       <c r="I136" s="5"/>
-      <c r="J136" s="8" t="str">
+      <c r="J136" s="5"/>
+      <c r="K136" s="5"/>
+      <c r="L136" s="8" t="str">
         <f aca="true">IF(A136="","",IF(I136="Hidden","Hidden",IF(AND(H136&lt;&gt;"",H136&gt;TODAY()),"Scheduled",IF(IF(C136&lt;&gt;"",C136,B136)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17712,7 +18050,9 @@
       <c r="G137" s="5"/>
       <c r="H137" s="7"/>
       <c r="I137" s="5"/>
-      <c r="J137" s="8" t="str">
+      <c r="J137" s="5"/>
+      <c r="K137" s="5"/>
+      <c r="L137" s="8" t="str">
         <f aca="true">IF(A137="","",IF(I137="Hidden","Hidden",IF(AND(H137&lt;&gt;"",H137&gt;TODAY()),"Scheduled",IF(IF(C137&lt;&gt;"",C137,B137)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17727,7 +18067,9 @@
       <c r="G138" s="5"/>
       <c r="H138" s="7"/>
       <c r="I138" s="5"/>
-      <c r="J138" s="8" t="str">
+      <c r="J138" s="5"/>
+      <c r="K138" s="5"/>
+      <c r="L138" s="8" t="str">
         <f aca="true">IF(A138="","",IF(I138="Hidden","Hidden",IF(AND(H138&lt;&gt;"",H138&gt;TODAY()),"Scheduled",IF(IF(C138&lt;&gt;"",C138,B138)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17742,7 +18084,9 @@
       <c r="G139" s="5"/>
       <c r="H139" s="7"/>
       <c r="I139" s="5"/>
-      <c r="J139" s="8" t="str">
+      <c r="J139" s="5"/>
+      <c r="K139" s="5"/>
+      <c r="L139" s="8" t="str">
         <f aca="true">IF(A139="","",IF(I139="Hidden","Hidden",IF(AND(H139&lt;&gt;"",H139&gt;TODAY()),"Scheduled",IF(IF(C139&lt;&gt;"",C139,B139)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17757,7 +18101,9 @@
       <c r="G140" s="5"/>
       <c r="H140" s="7"/>
       <c r="I140" s="5"/>
-      <c r="J140" s="8" t="str">
+      <c r="J140" s="5"/>
+      <c r="K140" s="5"/>
+      <c r="L140" s="8" t="str">
         <f aca="true">IF(A140="","",IF(I140="Hidden","Hidden",IF(AND(H140&lt;&gt;"",H140&gt;TODAY()),"Scheduled",IF(IF(C140&lt;&gt;"",C140,B140)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17772,7 +18118,9 @@
       <c r="G141" s="5"/>
       <c r="H141" s="7"/>
       <c r="I141" s="5"/>
-      <c r="J141" s="8" t="str">
+      <c r="J141" s="5"/>
+      <c r="K141" s="5"/>
+      <c r="L141" s="8" t="str">
         <f aca="true">IF(A141="","",IF(I141="Hidden","Hidden",IF(AND(H141&lt;&gt;"",H141&gt;TODAY()),"Scheduled",IF(IF(C141&lt;&gt;"",C141,B141)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17787,7 +18135,9 @@
       <c r="G142" s="5"/>
       <c r="H142" s="7"/>
       <c r="I142" s="5"/>
-      <c r="J142" s="8" t="str">
+      <c r="J142" s="5"/>
+      <c r="K142" s="5"/>
+      <c r="L142" s="8" t="str">
         <f aca="true">IF(A142="","",IF(I142="Hidden","Hidden",IF(AND(H142&lt;&gt;"",H142&gt;TODAY()),"Scheduled",IF(IF(C142&lt;&gt;"",C142,B142)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17802,7 +18152,9 @@
       <c r="G143" s="5"/>
       <c r="H143" s="7"/>
       <c r="I143" s="5"/>
-      <c r="J143" s="8" t="str">
+      <c r="J143" s="5"/>
+      <c r="K143" s="5"/>
+      <c r="L143" s="8" t="str">
         <f aca="true">IF(A143="","",IF(I143="Hidden","Hidden",IF(AND(H143&lt;&gt;"",H143&gt;TODAY()),"Scheduled",IF(IF(C143&lt;&gt;"",C143,B143)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17817,7 +18169,9 @@
       <c r="G144" s="5"/>
       <c r="H144" s="7"/>
       <c r="I144" s="5"/>
-      <c r="J144" s="8" t="str">
+      <c r="J144" s="5"/>
+      <c r="K144" s="5"/>
+      <c r="L144" s="8" t="str">
         <f aca="true">IF(A144="","",IF(I144="Hidden","Hidden",IF(AND(H144&lt;&gt;"",H144&gt;TODAY()),"Scheduled",IF(IF(C144&lt;&gt;"",C144,B144)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17832,7 +18186,9 @@
       <c r="G145" s="5"/>
       <c r="H145" s="7"/>
       <c r="I145" s="5"/>
-      <c r="J145" s="8" t="str">
+      <c r="J145" s="5"/>
+      <c r="K145" s="5"/>
+      <c r="L145" s="8" t="str">
         <f aca="true">IF(A145="","",IF(I145="Hidden","Hidden",IF(AND(H145&lt;&gt;"",H145&gt;TODAY()),"Scheduled",IF(IF(C145&lt;&gt;"",C145,B145)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17847,7 +18203,9 @@
       <c r="G146" s="5"/>
       <c r="H146" s="7"/>
       <c r="I146" s="5"/>
-      <c r="J146" s="8" t="str">
+      <c r="J146" s="5"/>
+      <c r="K146" s="5"/>
+      <c r="L146" s="8" t="str">
         <f aca="true">IF(A146="","",IF(I146="Hidden","Hidden",IF(AND(H146&lt;&gt;"",H146&gt;TODAY()),"Scheduled",IF(IF(C146&lt;&gt;"",C146,B146)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17862,7 +18220,9 @@
       <c r="G147" s="5"/>
       <c r="H147" s="7"/>
       <c r="I147" s="5"/>
-      <c r="J147" s="8" t="str">
+      <c r="J147" s="5"/>
+      <c r="K147" s="5"/>
+      <c r="L147" s="8" t="str">
         <f aca="true">IF(A147="","",IF(I147="Hidden","Hidden",IF(AND(H147&lt;&gt;"",H147&gt;TODAY()),"Scheduled",IF(IF(C147&lt;&gt;"",C147,B147)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17877,7 +18237,9 @@
       <c r="G148" s="5"/>
       <c r="H148" s="7"/>
       <c r="I148" s="5"/>
-      <c r="J148" s="8" t="str">
+      <c r="J148" s="5"/>
+      <c r="K148" s="5"/>
+      <c r="L148" s="8" t="str">
         <f aca="true">IF(A148="","",IF(I148="Hidden","Hidden",IF(AND(H148&lt;&gt;"",H148&gt;TODAY()),"Scheduled",IF(IF(C148&lt;&gt;"",C148,B148)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17892,7 +18254,9 @@
       <c r="G149" s="5"/>
       <c r="H149" s="7"/>
       <c r="I149" s="5"/>
-      <c r="J149" s="8" t="str">
+      <c r="J149" s="5"/>
+      <c r="K149" s="5"/>
+      <c r="L149" s="8" t="str">
         <f aca="true">IF(A149="","",IF(I149="Hidden","Hidden",IF(AND(H149&lt;&gt;"",H149&gt;TODAY()),"Scheduled",IF(IF(C149&lt;&gt;"",C149,B149)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17907,7 +18271,9 @@
       <c r="G150" s="5"/>
       <c r="H150" s="7"/>
       <c r="I150" s="5"/>
-      <c r="J150" s="8" t="str">
+      <c r="J150" s="5"/>
+      <c r="K150" s="5"/>
+      <c r="L150" s="8" t="str">
         <f aca="true">IF(A150="","",IF(I150="Hidden","Hidden",IF(AND(H150&lt;&gt;"",H150&gt;TODAY()),"Scheduled",IF(IF(C150&lt;&gt;"",C150,B150)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17922,7 +18288,9 @@
       <c r="G151" s="5"/>
       <c r="H151" s="7"/>
       <c r="I151" s="5"/>
-      <c r="J151" s="8" t="str">
+      <c r="J151" s="5"/>
+      <c r="K151" s="5"/>
+      <c r="L151" s="8" t="str">
         <f aca="true">IF(A151="","",IF(I151="Hidden","Hidden",IF(AND(H151&lt;&gt;"",H151&gt;TODAY()),"Scheduled",IF(IF(C151&lt;&gt;"",C151,B151)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17937,7 +18305,9 @@
       <c r="G152" s="5"/>
       <c r="H152" s="7"/>
       <c r="I152" s="5"/>
-      <c r="J152" s="8" t="str">
+      <c r="J152" s="5"/>
+      <c r="K152" s="5"/>
+      <c r="L152" s="8" t="str">
         <f aca="true">IF(A152="","",IF(I152="Hidden","Hidden",IF(AND(H152&lt;&gt;"",H152&gt;TODAY()),"Scheduled",IF(IF(C152&lt;&gt;"",C152,B152)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17952,7 +18322,9 @@
       <c r="G153" s="5"/>
       <c r="H153" s="7"/>
       <c r="I153" s="5"/>
-      <c r="J153" s="8" t="str">
+      <c r="J153" s="5"/>
+      <c r="K153" s="5"/>
+      <c r="L153" s="8" t="str">
         <f aca="true">IF(A153="","",IF(I153="Hidden","Hidden",IF(AND(H153&lt;&gt;"",H153&gt;TODAY()),"Scheduled",IF(IF(C153&lt;&gt;"",C153,B153)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17967,7 +18339,9 @@
       <c r="G154" s="5"/>
       <c r="H154" s="7"/>
       <c r="I154" s="5"/>
-      <c r="J154" s="8" t="str">
+      <c r="J154" s="5"/>
+      <c r="K154" s="5"/>
+      <c r="L154" s="8" t="str">
         <f aca="true">IF(A154="","",IF(I154="Hidden","Hidden",IF(AND(H154&lt;&gt;"",H154&gt;TODAY()),"Scheduled",IF(IF(C154&lt;&gt;"",C154,B154)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17982,7 +18356,9 @@
       <c r="G155" s="5"/>
       <c r="H155" s="7"/>
       <c r="I155" s="5"/>
-      <c r="J155" s="8" t="str">
+      <c r="J155" s="5"/>
+      <c r="K155" s="5"/>
+      <c r="L155" s="8" t="str">
         <f aca="true">IF(A155="","",IF(I155="Hidden","Hidden",IF(AND(H155&lt;&gt;"",H155&gt;TODAY()),"Scheduled",IF(IF(C155&lt;&gt;"",C155,B155)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -17997,7 +18373,9 @@
       <c r="G156" s="5"/>
       <c r="H156" s="7"/>
       <c r="I156" s="5"/>
-      <c r="J156" s="8" t="str">
+      <c r="J156" s="5"/>
+      <c r="K156" s="5"/>
+      <c r="L156" s="8" t="str">
         <f aca="true">IF(A156="","",IF(I156="Hidden","Hidden",IF(AND(H156&lt;&gt;"",H156&gt;TODAY()),"Scheduled",IF(IF(C156&lt;&gt;"",C156,B156)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18012,7 +18390,9 @@
       <c r="G157" s="5"/>
       <c r="H157" s="7"/>
       <c r="I157" s="5"/>
-      <c r="J157" s="8" t="str">
+      <c r="J157" s="5"/>
+      <c r="K157" s="5"/>
+      <c r="L157" s="8" t="str">
         <f aca="true">IF(A157="","",IF(I157="Hidden","Hidden",IF(AND(H157&lt;&gt;"",H157&gt;TODAY()),"Scheduled",IF(IF(C157&lt;&gt;"",C157,B157)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18027,7 +18407,9 @@
       <c r="G158" s="5"/>
       <c r="H158" s="7"/>
       <c r="I158" s="5"/>
-      <c r="J158" s="8" t="str">
+      <c r="J158" s="5"/>
+      <c r="K158" s="5"/>
+      <c r="L158" s="8" t="str">
         <f aca="true">IF(A158="","",IF(I158="Hidden","Hidden",IF(AND(H158&lt;&gt;"",H158&gt;TODAY()),"Scheduled",IF(IF(C158&lt;&gt;"",C158,B158)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18042,7 +18424,9 @@
       <c r="G159" s="5"/>
       <c r="H159" s="7"/>
       <c r="I159" s="5"/>
-      <c r="J159" s="8" t="str">
+      <c r="J159" s="5"/>
+      <c r="K159" s="5"/>
+      <c r="L159" s="8" t="str">
         <f aca="true">IF(A159="","",IF(I159="Hidden","Hidden",IF(AND(H159&lt;&gt;"",H159&gt;TODAY()),"Scheduled",IF(IF(C159&lt;&gt;"",C159,B159)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18057,7 +18441,9 @@
       <c r="G160" s="5"/>
       <c r="H160" s="7"/>
       <c r="I160" s="5"/>
-      <c r="J160" s="8" t="str">
+      <c r="J160" s="5"/>
+      <c r="K160" s="5"/>
+      <c r="L160" s="8" t="str">
         <f aca="true">IF(A160="","",IF(I160="Hidden","Hidden",IF(AND(H160&lt;&gt;"",H160&gt;TODAY()),"Scheduled",IF(IF(C160&lt;&gt;"",C160,B160)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18072,7 +18458,9 @@
       <c r="G161" s="5"/>
       <c r="H161" s="7"/>
       <c r="I161" s="5"/>
-      <c r="J161" s="8" t="str">
+      <c r="J161" s="5"/>
+      <c r="K161" s="5"/>
+      <c r="L161" s="8" t="str">
         <f aca="true">IF(A161="","",IF(I161="Hidden","Hidden",IF(AND(H161&lt;&gt;"",H161&gt;TODAY()),"Scheduled",IF(IF(C161&lt;&gt;"",C161,B161)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18087,7 +18475,9 @@
       <c r="G162" s="5"/>
       <c r="H162" s="7"/>
       <c r="I162" s="5"/>
-      <c r="J162" s="8" t="str">
+      <c r="J162" s="5"/>
+      <c r="K162" s="5"/>
+      <c r="L162" s="8" t="str">
         <f aca="true">IF(A162="","",IF(I162="Hidden","Hidden",IF(AND(H162&lt;&gt;"",H162&gt;TODAY()),"Scheduled",IF(IF(C162&lt;&gt;"",C162,B162)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18102,7 +18492,9 @@
       <c r="G163" s="5"/>
       <c r="H163" s="7"/>
       <c r="I163" s="5"/>
-      <c r="J163" s="8" t="str">
+      <c r="J163" s="5"/>
+      <c r="K163" s="5"/>
+      <c r="L163" s="8" t="str">
         <f aca="true">IF(A163="","",IF(I163="Hidden","Hidden",IF(AND(H163&lt;&gt;"",H163&gt;TODAY()),"Scheduled",IF(IF(C163&lt;&gt;"",C163,B163)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18117,7 +18509,9 @@
       <c r="G164" s="5"/>
       <c r="H164" s="7"/>
       <c r="I164" s="5"/>
-      <c r="J164" s="8" t="str">
+      <c r="J164" s="5"/>
+      <c r="K164" s="5"/>
+      <c r="L164" s="8" t="str">
         <f aca="true">IF(A164="","",IF(I164="Hidden","Hidden",IF(AND(H164&lt;&gt;"",H164&gt;TODAY()),"Scheduled",IF(IF(C164&lt;&gt;"",C164,B164)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18132,7 +18526,9 @@
       <c r="G165" s="5"/>
       <c r="H165" s="7"/>
       <c r="I165" s="5"/>
-      <c r="J165" s="8" t="str">
+      <c r="J165" s="5"/>
+      <c r="K165" s="5"/>
+      <c r="L165" s="8" t="str">
         <f aca="true">IF(A165="","",IF(I165="Hidden","Hidden",IF(AND(H165&lt;&gt;"",H165&gt;TODAY()),"Scheduled",IF(IF(C165&lt;&gt;"",C165,B165)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18147,7 +18543,9 @@
       <c r="G166" s="5"/>
       <c r="H166" s="7"/>
       <c r="I166" s="5"/>
-      <c r="J166" s="8" t="str">
+      <c r="J166" s="5"/>
+      <c r="K166" s="5"/>
+      <c r="L166" s="8" t="str">
         <f aca="true">IF(A166="","",IF(I166="Hidden","Hidden",IF(AND(H166&lt;&gt;"",H166&gt;TODAY()),"Scheduled",IF(IF(C166&lt;&gt;"",C166,B166)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18162,7 +18560,9 @@
       <c r="G167" s="5"/>
       <c r="H167" s="7"/>
       <c r="I167" s="5"/>
-      <c r="J167" s="8" t="str">
+      <c r="J167" s="5"/>
+      <c r="K167" s="5"/>
+      <c r="L167" s="8" t="str">
         <f aca="true">IF(A167="","",IF(I167="Hidden","Hidden",IF(AND(H167&lt;&gt;"",H167&gt;TODAY()),"Scheduled",IF(IF(C167&lt;&gt;"",C167,B167)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18177,7 +18577,9 @@
       <c r="G168" s="5"/>
       <c r="H168" s="7"/>
       <c r="I168" s="5"/>
-      <c r="J168" s="8" t="str">
+      <c r="J168" s="5"/>
+      <c r="K168" s="5"/>
+      <c r="L168" s="8" t="str">
         <f aca="true">IF(A168="","",IF(I168="Hidden","Hidden",IF(AND(H168&lt;&gt;"",H168&gt;TODAY()),"Scheduled",IF(IF(C168&lt;&gt;"",C168,B168)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18192,7 +18594,9 @@
       <c r="G169" s="5"/>
       <c r="H169" s="7"/>
       <c r="I169" s="5"/>
-      <c r="J169" s="8" t="str">
+      <c r="J169" s="5"/>
+      <c r="K169" s="5"/>
+      <c r="L169" s="8" t="str">
         <f aca="true">IF(A169="","",IF(I169="Hidden","Hidden",IF(AND(H169&lt;&gt;"",H169&gt;TODAY()),"Scheduled",IF(IF(C169&lt;&gt;"",C169,B169)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18207,7 +18611,9 @@
       <c r="G170" s="5"/>
       <c r="H170" s="7"/>
       <c r="I170" s="5"/>
-      <c r="J170" s="8" t="str">
+      <c r="J170" s="5"/>
+      <c r="K170" s="5"/>
+      <c r="L170" s="8" t="str">
         <f aca="true">IF(A170="","",IF(I170="Hidden","Hidden",IF(AND(H170&lt;&gt;"",H170&gt;TODAY()),"Scheduled",IF(IF(C170&lt;&gt;"",C170,B170)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18222,7 +18628,9 @@
       <c r="G171" s="5"/>
       <c r="H171" s="7"/>
       <c r="I171" s="5"/>
-      <c r="J171" s="8" t="str">
+      <c r="J171" s="5"/>
+      <c r="K171" s="5"/>
+      <c r="L171" s="8" t="str">
         <f aca="true">IF(A171="","",IF(I171="Hidden","Hidden",IF(AND(H171&lt;&gt;"",H171&gt;TODAY()),"Scheduled",IF(IF(C171&lt;&gt;"",C171,B171)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18237,7 +18645,9 @@
       <c r="G172" s="5"/>
       <c r="H172" s="7"/>
       <c r="I172" s="5"/>
-      <c r="J172" s="8" t="str">
+      <c r="J172" s="5"/>
+      <c r="K172" s="5"/>
+      <c r="L172" s="8" t="str">
         <f aca="true">IF(A172="","",IF(I172="Hidden","Hidden",IF(AND(H172&lt;&gt;"",H172&gt;TODAY()),"Scheduled",IF(IF(C172&lt;&gt;"",C172,B172)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18252,7 +18662,9 @@
       <c r="G173" s="5"/>
       <c r="H173" s="7"/>
       <c r="I173" s="5"/>
-      <c r="J173" s="8" t="str">
+      <c r="J173" s="5"/>
+      <c r="K173" s="5"/>
+      <c r="L173" s="8" t="str">
         <f aca="true">IF(A173="","",IF(I173="Hidden","Hidden",IF(AND(H173&lt;&gt;"",H173&gt;TODAY()),"Scheduled",IF(IF(C173&lt;&gt;"",C173,B173)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18267,7 +18679,9 @@
       <c r="G174" s="5"/>
       <c r="H174" s="7"/>
       <c r="I174" s="5"/>
-      <c r="J174" s="8" t="str">
+      <c r="J174" s="5"/>
+      <c r="K174" s="5"/>
+      <c r="L174" s="8" t="str">
         <f aca="true">IF(A174="","",IF(I174="Hidden","Hidden",IF(AND(H174&lt;&gt;"",H174&gt;TODAY()),"Scheduled",IF(IF(C174&lt;&gt;"",C174,B174)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18282,7 +18696,9 @@
       <c r="G175" s="5"/>
       <c r="H175" s="7"/>
       <c r="I175" s="5"/>
-      <c r="J175" s="8" t="str">
+      <c r="J175" s="5"/>
+      <c r="K175" s="5"/>
+      <c r="L175" s="8" t="str">
         <f aca="true">IF(A175="","",IF(I175="Hidden","Hidden",IF(AND(H175&lt;&gt;"",H175&gt;TODAY()),"Scheduled",IF(IF(C175&lt;&gt;"",C175,B175)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18297,7 +18713,9 @@
       <c r="G176" s="5"/>
       <c r="H176" s="7"/>
       <c r="I176" s="5"/>
-      <c r="J176" s="8" t="str">
+      <c r="J176" s="5"/>
+      <c r="K176" s="5"/>
+      <c r="L176" s="8" t="str">
         <f aca="true">IF(A176="","",IF(I176="Hidden","Hidden",IF(AND(H176&lt;&gt;"",H176&gt;TODAY()),"Scheduled",IF(IF(C176&lt;&gt;"",C176,B176)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18312,7 +18730,9 @@
       <c r="G177" s="5"/>
       <c r="H177" s="7"/>
       <c r="I177" s="5"/>
-      <c r="J177" s="8" t="str">
+      <c r="J177" s="5"/>
+      <c r="K177" s="5"/>
+      <c r="L177" s="8" t="str">
         <f aca="true">IF(A177="","",IF(I177="Hidden","Hidden",IF(AND(H177&lt;&gt;"",H177&gt;TODAY()),"Scheduled",IF(IF(C177&lt;&gt;"",C177,B177)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18327,7 +18747,9 @@
       <c r="G178" s="5"/>
       <c r="H178" s="7"/>
       <c r="I178" s="5"/>
-      <c r="J178" s="8" t="str">
+      <c r="J178" s="5"/>
+      <c r="K178" s="5"/>
+      <c r="L178" s="8" t="str">
         <f aca="true">IF(A178="","",IF(I178="Hidden","Hidden",IF(AND(H178&lt;&gt;"",H178&gt;TODAY()),"Scheduled",IF(IF(C178&lt;&gt;"",C178,B178)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18342,7 +18764,9 @@
       <c r="G179" s="5"/>
       <c r="H179" s="7"/>
       <c r="I179" s="5"/>
-      <c r="J179" s="8" t="str">
+      <c r="J179" s="5"/>
+      <c r="K179" s="5"/>
+      <c r="L179" s="8" t="str">
         <f aca="true">IF(A179="","",IF(I179="Hidden","Hidden",IF(AND(H179&lt;&gt;"",H179&gt;TODAY()),"Scheduled",IF(IF(C179&lt;&gt;"",C179,B179)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18357,7 +18781,9 @@
       <c r="G180" s="5"/>
       <c r="H180" s="7"/>
       <c r="I180" s="5"/>
-      <c r="J180" s="8" t="str">
+      <c r="J180" s="5"/>
+      <c r="K180" s="5"/>
+      <c r="L180" s="8" t="str">
         <f aca="true">IF(A180="","",IF(I180="Hidden","Hidden",IF(AND(H180&lt;&gt;"",H180&gt;TODAY()),"Scheduled",IF(IF(C180&lt;&gt;"",C180,B180)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18372,7 +18798,9 @@
       <c r="G181" s="5"/>
       <c r="H181" s="7"/>
       <c r="I181" s="5"/>
-      <c r="J181" s="8" t="str">
+      <c r="J181" s="5"/>
+      <c r="K181" s="5"/>
+      <c r="L181" s="8" t="str">
         <f aca="true">IF(A181="","",IF(I181="Hidden","Hidden",IF(AND(H181&lt;&gt;"",H181&gt;TODAY()),"Scheduled",IF(IF(C181&lt;&gt;"",C181,B181)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18387,7 +18815,9 @@
       <c r="G182" s="5"/>
       <c r="H182" s="7"/>
       <c r="I182" s="5"/>
-      <c r="J182" s="8" t="str">
+      <c r="J182" s="5"/>
+      <c r="K182" s="5"/>
+      <c r="L182" s="8" t="str">
         <f aca="true">IF(A182="","",IF(I182="Hidden","Hidden",IF(AND(H182&lt;&gt;"",H182&gt;TODAY()),"Scheduled",IF(IF(C182&lt;&gt;"",C182,B182)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18402,7 +18832,9 @@
       <c r="G183" s="5"/>
       <c r="H183" s="7"/>
       <c r="I183" s="5"/>
-      <c r="J183" s="8" t="str">
+      <c r="J183" s="5"/>
+      <c r="K183" s="5"/>
+      <c r="L183" s="8" t="str">
         <f aca="true">IF(A183="","",IF(I183="Hidden","Hidden",IF(AND(H183&lt;&gt;"",H183&gt;TODAY()),"Scheduled",IF(IF(C183&lt;&gt;"",C183,B183)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18417,7 +18849,9 @@
       <c r="G184" s="5"/>
       <c r="H184" s="7"/>
       <c r="I184" s="5"/>
-      <c r="J184" s="8" t="str">
+      <c r="J184" s="5"/>
+      <c r="K184" s="5"/>
+      <c r="L184" s="8" t="str">
         <f aca="true">IF(A184="","",IF(I184="Hidden","Hidden",IF(AND(H184&lt;&gt;"",H184&gt;TODAY()),"Scheduled",IF(IF(C184&lt;&gt;"",C184,B184)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18432,7 +18866,9 @@
       <c r="G185" s="5"/>
       <c r="H185" s="7"/>
       <c r="I185" s="5"/>
-      <c r="J185" s="8" t="str">
+      <c r="J185" s="5"/>
+      <c r="K185" s="5"/>
+      <c r="L185" s="8" t="str">
         <f aca="true">IF(A185="","",IF(I185="Hidden","Hidden",IF(AND(H185&lt;&gt;"",H185&gt;TODAY()),"Scheduled",IF(IF(C185&lt;&gt;"",C185,B185)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18447,7 +18883,9 @@
       <c r="G186" s="5"/>
       <c r="H186" s="7"/>
       <c r="I186" s="5"/>
-      <c r="J186" s="8" t="str">
+      <c r="J186" s="5"/>
+      <c r="K186" s="5"/>
+      <c r="L186" s="8" t="str">
         <f aca="true">IF(A186="","",IF(I186="Hidden","Hidden",IF(AND(H186&lt;&gt;"",H186&gt;TODAY()),"Scheduled",IF(IF(C186&lt;&gt;"",C186,B186)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18462,7 +18900,9 @@
       <c r="G187" s="5"/>
       <c r="H187" s="7"/>
       <c r="I187" s="5"/>
-      <c r="J187" s="8" t="str">
+      <c r="J187" s="5"/>
+      <c r="K187" s="5"/>
+      <c r="L187" s="8" t="str">
         <f aca="true">IF(A187="","",IF(I187="Hidden","Hidden",IF(AND(H187&lt;&gt;"",H187&gt;TODAY()),"Scheduled",IF(IF(C187&lt;&gt;"",C187,B187)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18477,7 +18917,9 @@
       <c r="G188" s="5"/>
       <c r="H188" s="7"/>
       <c r="I188" s="5"/>
-      <c r="J188" s="8" t="str">
+      <c r="J188" s="5"/>
+      <c r="K188" s="5"/>
+      <c r="L188" s="8" t="str">
         <f aca="true">IF(A188="","",IF(I188="Hidden","Hidden",IF(AND(H188&lt;&gt;"",H188&gt;TODAY()),"Scheduled",IF(IF(C188&lt;&gt;"",C188,B188)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18492,7 +18934,9 @@
       <c r="G189" s="5"/>
       <c r="H189" s="7"/>
       <c r="I189" s="5"/>
-      <c r="J189" s="8" t="str">
+      <c r="J189" s="5"/>
+      <c r="K189" s="5"/>
+      <c r="L189" s="8" t="str">
         <f aca="true">IF(A189="","",IF(I189="Hidden","Hidden",IF(AND(H189&lt;&gt;"",H189&gt;TODAY()),"Scheduled",IF(IF(C189&lt;&gt;"",C189,B189)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18507,7 +18951,9 @@
       <c r="G190" s="5"/>
       <c r="H190" s="7"/>
       <c r="I190" s="5"/>
-      <c r="J190" s="8" t="str">
+      <c r="J190" s="5"/>
+      <c r="K190" s="5"/>
+      <c r="L190" s="8" t="str">
         <f aca="true">IF(A190="","",IF(I190="Hidden","Hidden",IF(AND(H190&lt;&gt;"",H190&gt;TODAY()),"Scheduled",IF(IF(C190&lt;&gt;"",C190,B190)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18522,7 +18968,9 @@
       <c r="G191" s="5"/>
       <c r="H191" s="7"/>
       <c r="I191" s="5"/>
-      <c r="J191" s="8" t="str">
+      <c r="J191" s="5"/>
+      <c r="K191" s="5"/>
+      <c r="L191" s="8" t="str">
         <f aca="true">IF(A191="","",IF(I191="Hidden","Hidden",IF(AND(H191&lt;&gt;"",H191&gt;TODAY()),"Scheduled",IF(IF(C191&lt;&gt;"",C191,B191)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18537,7 +18985,9 @@
       <c r="G192" s="5"/>
       <c r="H192" s="7"/>
       <c r="I192" s="5"/>
-      <c r="J192" s="8" t="str">
+      <c r="J192" s="5"/>
+      <c r="K192" s="5"/>
+      <c r="L192" s="8" t="str">
         <f aca="true">IF(A192="","",IF(I192="Hidden","Hidden",IF(AND(H192&lt;&gt;"",H192&gt;TODAY()),"Scheduled",IF(IF(C192&lt;&gt;"",C192,B192)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18552,7 +19002,9 @@
       <c r="G193" s="5"/>
       <c r="H193" s="7"/>
       <c r="I193" s="5"/>
-      <c r="J193" s="8" t="str">
+      <c r="J193" s="5"/>
+      <c r="K193" s="5"/>
+      <c r="L193" s="8" t="str">
         <f aca="true">IF(A193="","",IF(I193="Hidden","Hidden",IF(AND(H193&lt;&gt;"",H193&gt;TODAY()),"Scheduled",IF(IF(C193&lt;&gt;"",C193,B193)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18567,7 +19019,9 @@
       <c r="G194" s="5"/>
       <c r="H194" s="7"/>
       <c r="I194" s="5"/>
-      <c r="J194" s="8" t="str">
+      <c r="J194" s="5"/>
+      <c r="K194" s="5"/>
+      <c r="L194" s="8" t="str">
         <f aca="true">IF(A194="","",IF(I194="Hidden","Hidden",IF(AND(H194&lt;&gt;"",H194&gt;TODAY()),"Scheduled",IF(IF(C194&lt;&gt;"",C194,B194)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18582,7 +19036,9 @@
       <c r="G195" s="5"/>
       <c r="H195" s="7"/>
       <c r="I195" s="5"/>
-      <c r="J195" s="8" t="str">
+      <c r="J195" s="5"/>
+      <c r="K195" s="5"/>
+      <c r="L195" s="8" t="str">
         <f aca="true">IF(A195="","",IF(I195="Hidden","Hidden",IF(AND(H195&lt;&gt;"",H195&gt;TODAY()),"Scheduled",IF(IF(C195&lt;&gt;"",C195,B195)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18597,7 +19053,9 @@
       <c r="G196" s="5"/>
       <c r="H196" s="7"/>
       <c r="I196" s="5"/>
-      <c r="J196" s="8" t="str">
+      <c r="J196" s="5"/>
+      <c r="K196" s="5"/>
+      <c r="L196" s="8" t="str">
         <f aca="true">IF(A196="","",IF(I196="Hidden","Hidden",IF(AND(H196&lt;&gt;"",H196&gt;TODAY()),"Scheduled",IF(IF(C196&lt;&gt;"",C196,B196)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18612,7 +19070,9 @@
       <c r="G197" s="5"/>
       <c r="H197" s="7"/>
       <c r="I197" s="5"/>
-      <c r="J197" s="8" t="str">
+      <c r="J197" s="5"/>
+      <c r="K197" s="5"/>
+      <c r="L197" s="8" t="str">
         <f aca="true">IF(A197="","",IF(I197="Hidden","Hidden",IF(AND(H197&lt;&gt;"",H197&gt;TODAY()),"Scheduled",IF(IF(C197&lt;&gt;"",C197,B197)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18627,7 +19087,9 @@
       <c r="G198" s="5"/>
       <c r="H198" s="7"/>
       <c r="I198" s="5"/>
-      <c r="J198" s="8" t="str">
+      <c r="J198" s="5"/>
+      <c r="K198" s="5"/>
+      <c r="L198" s="8" t="str">
         <f aca="true">IF(A198="","",IF(I198="Hidden","Hidden",IF(AND(H198&lt;&gt;"",H198&gt;TODAY()),"Scheduled",IF(IF(C198&lt;&gt;"",C198,B198)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18642,7 +19104,9 @@
       <c r="G199" s="5"/>
       <c r="H199" s="7"/>
       <c r="I199" s="5"/>
-      <c r="J199" s="8" t="str">
+      <c r="J199" s="5"/>
+      <c r="K199" s="5"/>
+      <c r="L199" s="8" t="str">
         <f aca="true">IF(A199="","",IF(I199="Hidden","Hidden",IF(AND(H199&lt;&gt;"",H199&gt;TODAY()),"Scheduled",IF(IF(C199&lt;&gt;"",C199,B199)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
@@ -18657,21 +19121,23 @@
       <c r="G200" s="5"/>
       <c r="H200" s="7"/>
       <c r="I200" s="5"/>
-      <c r="J200" s="8" t="str">
+      <c r="J200" s="5"/>
+      <c r="K200" s="5"/>
+      <c r="L200" s="8" t="str">
         <f aca="true">IF(A200="","",IF(I200="Hidden","Hidden",IF(AND(H200&lt;&gt;"",H200&gt;TODAY()),"Scheduled",IF(IF(C200&lt;&gt;"",C200,B200)&lt;TODAY(),"Expired","Showing"))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:J200">
+  <conditionalFormatting sqref="L2:L200">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>OR(J2="Showing",J2="Regular",J2="Special, in effect")</formula>
+      <formula>OR(L2="Showing",L2="Regular",L2="Special, in effect")</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>J2="Scheduled"</formula>
+      <formula>L2="Scheduled"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>OR(J2="Expired",J2="Hidden")</formula>
+      <formula>OR(L2="Expired",L2="Hidden")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -18719,22 +19185,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>193</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>84</v>
@@ -18751,35 +19217,35 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>46304</v>
+        <v>46508</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>46387</v>
+        <v>46538</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="J2" s="8" t="str">
         <f aca="true">IF(B2="","",IF(I2="Hidden","Hidden",IF(AND(G2&lt;&gt;"",G2&gt;TODAY()),"Scheduled",IF(AND(H2&lt;&gt;"",H2&lt;TODAY()),"Expired","Showing"))))</f>
-        <v>Showing</v>
+        <v>Hidden</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21807,31 +22273,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>199</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -21848,27 +22314,27 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>6.5</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -21882,10 +22348,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>2</v>
@@ -21893,14 +22359,14 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -21914,10 +22380,10 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
@@ -21927,14 +22393,14 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -21948,10 +22414,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>28.4</v>
@@ -21960,19 +22426,19 @@
         <v>2600</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -21986,10 +22452,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>20.3</v>
@@ -21998,19 +22464,19 @@
         <v>850</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>

</xml_diff>

<commit_message>
Washed-out themed backgrounds behind each event (Halloween, Christmas, NYE); remove events intro line
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="266">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -745,6 +745,9 @@
     <t xml:space="preserve">Call 01765 677198 to book your party</t>
   </si>
   <si>
+    <t xml:space="preserve">img/christmas.svg</t>
+  </si>
+  <si>
     <t xml:space="preserve">New Year's Eve BBQ</t>
   </si>
   <si>
@@ -752,6 +755,9 @@
   </si>
   <si>
     <t xml:space="preserve">Please book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img/nye.svg</t>
   </si>
   <si>
     <t xml:space="preserve">EXAMPLE: Summer BBQ in the garden</t>
@@ -15728,7 +15734,9 @@
       <c r="I3" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J3" s="5"/>
+      <c r="J3" s="5" t="s">
+        <v>212</v>
+      </c>
       <c r="K3" s="5" t="s">
         <v>92</v>
       </c>
@@ -15739,7 +15747,7 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46387</v>
@@ -15747,11 +15755,11 @@
       <c r="C4" s="7"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46304</v>
@@ -15759,7 +15767,9 @@
       <c r="I4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>216</v>
+      </c>
       <c r="K4" s="5"/>
       <c r="L4" s="8" t="str">
         <f aca="true">IF(A4="","",IF(I4="Hidden","Hidden",IF(AND(H4&lt;&gt;"",H4&gt;TODAY()),"Scheduled",IF(IF(C4&lt;&gt;"",C4,B4)&lt;TODAY(),"Expired","Showing"))))</f>
@@ -15768,21 +15778,21 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>46564</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>46508</v>
@@ -15799,23 +15809,23 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>46592</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>61</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>46553</v>
@@ -19185,22 +19195,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>193</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>84</v>
@@ -19217,22 +19227,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>46508</v>
@@ -22273,31 +22283,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>199</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>84</v>
@@ -22314,27 +22324,27 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>6.5</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -22348,10 +22358,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>2</v>
@@ -22359,14 +22369,14 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -22380,10 +22390,10 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
@@ -22393,14 +22403,14 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -22414,10 +22424,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>28.4</v>
@@ -22426,19 +22436,19 @@
         <v>2600</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -22452,10 +22462,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>20.3</v>
@@ -22464,19 +22474,19 @@
         <v>850</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>

</xml_diff>

<commit_message>
Real 555 evening menu, remove Thursday fish & chips night, flying sleigh and reindeer Christmas artwork
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvChsivB64YuL91yf74mXG
</commit_message>
<xml_diff>
--- a/Royal-Oak-content.xlsx
+++ b/Royal-Oak-content.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="279">
   <si>
     <t xml:space="preserve">The Royal Oak: website content sheet</t>
   </si>
@@ -244,7 +244,7 @@
     <t xml:space="preserve">What's on the sheet now</t>
   </si>
   <si>
-    <t xml:space="preserve">The current opening hours (with Sunday lunch on the last Sunday of each month), the current winter menu and Sunday lunch, the drinks basics from the old website, the 5-5-5 offer for 9 and 10 October 2026, and a New Year's Eve BBQ (menu feature from 9 October, banner from 1 December, both until 31 December 2026). The New Year's Eve price and times are blank because they have not been given yet. Add them in the Price and Description cells.</t>
+    <t xml:space="preserve">The current opening hours (with Sunday lunch on the last Sunday of each month), the current winter menu and Sunday lunch, the drinks basics from the old website, the 555 evening menu (five mini meals at £5), and a New Year's Eve BBQ (menu feature from 9 October, banner from 1 December, both until 31 December 2026). The New Year's Eve price and times are blank because they have not been given yet. Add them in the Price and Description cells.</t>
   </si>
   <si>
     <t xml:space="preserve">Days</t>
@@ -310,9 +310,6 @@
     <t xml:space="preserve">Food</t>
   </si>
   <si>
-    <t xml:space="preserve">Fish &amp; chips night, £9.95</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fri</t>
   </si>
   <si>
@@ -331,7 +328,7 @@
     <t xml:space="preserve">Christmas morning: drinks only, with free mince pies</t>
   </si>
   <si>
-    <t xml:space="preserve">New Year's Eve BBQ instead of fish &amp; chips. Please book.</t>
+    <t xml:space="preserve">New Year's Eve BBQ. Please book.</t>
   </si>
   <si>
     <t xml:space="preserve">EXAMPLE (hidden): Christmas Eve hours. Copy this row, change it and set Status to Live.</t>
@@ -367,19 +364,55 @@
     <t xml:space="preserve">Show until</t>
   </si>
   <si>
-    <t xml:space="preserve">Thursday: fish &amp; chips night</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fish, chips, mushy peas, bread and butter. Served 5 to 8pm.</t>
+    <t xml:space="preserve">555 evening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Five mini meals, £5 each, from 5pm.</t>
   </si>
   <si>
     <t xml:space="preserve">Board</t>
   </si>
   <si>
-    <t xml:space="preserve">The 5-5-5 menu: Friday 9 and Saturday 10 October</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fish &amp; chips. Curry. Wagyu burger. 5 bean chilli &amp; rice. Sausage &amp; mash with onion gravy.</t>
+    <t xml:space="preserve">Wagyu burger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melted cheddar, lettuce, tomato and burger sauce, topped with beer-battered onion rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beef &amp; 5 bean chilli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluffy rice and toasted pitta bread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beer-battered fish &amp; hand-cut chips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With a side of chip shop curry sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chicken Balti curry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basmati rice and garlic naan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bangers &amp; cheesy mash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With Guinness and onion gravy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extras: gourmet fries or hand-cut chips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A basket of either</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Children's meals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any of the above, or chicken nuggets and fries</t>
   </si>
   <si>
     <t xml:space="preserve">2 courses</t>
@@ -472,9 +505,6 @@
     <t xml:space="preserve">The alternative to the steak pie</t>
   </si>
   <si>
-    <t xml:space="preserve">Beer-battered fish &amp; hand-cut chips</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mushy peas, tartare sauce</t>
   </si>
   <si>
@@ -538,6 +568,15 @@
     <t xml:space="preserve">Cheeseburger &amp; fries</t>
   </si>
   <si>
+    <t xml:space="preserve">Homemade desserts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple &amp; cherry crumble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With deluxe creamy custard</t>
+  </si>
+  <si>
     <t xml:space="preserve">Slow-cooked brisket</t>
   </si>
   <si>
@@ -691,7 +730,7 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
-    <t xml:space="preserve">The 5-5-5 menu: Friday 9 and Saturday 10 October. Please reserve, we get busy.</t>
+    <t xml:space="preserve">555 evening: five mini meals at £5 each, from 5pm. Please reserve, we get busy.</t>
   </si>
   <si>
     <t xml:space="preserve">Christmas morning: we're open for drinks, with free mince pies.</t>
@@ -1776,9 +1815,7 @@
         <v>66</v>
       </c>
       <c r="H4" s="5"/>
-      <c r="I4" s="5" t="s">
-        <v>67</v>
-      </c>
+      <c r="I4" s="5"/>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
@@ -1792,7 +1829,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="n">
@@ -1823,7 +1860,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="6" t="n">
@@ -1856,7 +1893,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="6" t="n">
@@ -1883,10 +1920,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>0.5</v>
@@ -1901,7 +1938,7 @@
         <v>0.708333333333333</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -1918,7 +1955,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="6" t="n">
@@ -1932,7 +1969,7 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>46381</v>
@@ -1949,7 +1986,7 @@
         <v>Scheduled</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>65</v>
       </c>
@@ -1963,7 +2000,7 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>46387</v>
@@ -1996,7 +2033,7 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>46380</v>
@@ -2008,7 +2045,7 @@
         <v>46357</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N11" s="8" t="str">
         <f aca="true">IF(A11&amp;B11&amp;C11&amp;H11&amp;I11="","",IF(M11="Hidden","Hidden",IF(AND(J11&lt;&gt;"",J11&gt;TODAY()),"Scheduled",IF(AND(K11&lt;&gt;"",K11&lt;TODAY()),"Expired",IF(OR(J11&lt;&gt;"",K11&lt;&gt;""),"Special, in effect","Regular")))))</f>
@@ -5619,20 +5656,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:L200" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H200" type="list">
+      <formula1>"Yes"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M2:M200" type="list">
       <formula1>"Live,Hidden"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2:L200" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B200" type="list">
       <formula1>"1st,2nd,3rd,4th,Last"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H200" type="list">
-      <formula1>"Yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5665,31 +5702,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>46</v>
@@ -5702,27 +5739,23 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5" t="s">
+      <c r="A2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>9.95</v>
-      </c>
+      <c r="D2" s="9"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7" t="n">
-        <v>46386</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I2" s="7"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5" t="s">
         <v>62</v>
@@ -5732,26 +5765,26 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="B3" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>9.95</v>
+        <v>5</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>61</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="G3" s="5"/>
       <c r="H3" s="7" t="n">
-        <v>46388</v>
+        <v>46305</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" s="5"/>
@@ -5760,31 +5793,31 @@
       </c>
       <c r="L3" s="8" t="str">
         <f aca="true">IF(B3&amp;C3="","",IF(K3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(AND(I3&lt;&gt;"",I3&lt;TODAY()),"Expired","Showing"))))</f>
-        <v>Scheduled</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
+        <v>Showing</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="B4" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" s="9"/>
+        <v>91</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>61</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="G4" s="5"/>
       <c r="H4" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="I4" s="7" t="n">
         <v>46305</v>
       </c>
+      <c r="I4" s="7"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5" t="s">
         <v>62</v>
@@ -5796,26 +5829,26 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="5"/>
+        <v>92</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="D5" s="9" t="n">
-        <v>16.95</v>
+        <v>5</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I5" s="7" t="n">
-        <v>46379</v>
-      </c>
+      <c r="I5" s="7"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5" t="s">
         <v>62</v>
@@ -5827,26 +5860,26 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C6" s="5"/>
+        <v>94</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="D6" s="9" t="n">
-        <v>21.95</v>
+        <v>5</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I6" s="7" t="n">
-        <v>46379</v>
-      </c>
+      <c r="I6" s="7"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5" t="s">
         <v>62</v>
@@ -5858,26 +5891,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="5" t="s">
         <v>96</v>
       </c>
+      <c r="C7" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I7" s="7" t="n">
-        <v>46379</v>
-      </c>
+      <c r="I7" s="7"/>
       <c r="J7" s="5"/>
       <c r="K7" s="5" t="s">
         <v>62</v>
@@ -5889,28 +5922,26 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="5" t="s">
         <v>99</v>
       </c>
+      <c r="D8" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="5"/>
       <c r="F8" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I8" s="7" t="n">
-        <v>46379</v>
-      </c>
+      <c r="I8" s="7"/>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
         <v>62</v>
@@ -5922,7 +5953,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>100</v>
@@ -5930,20 +5961,18 @@
       <c r="C9" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="5" t="s">
-        <v>99</v>
-      </c>
+      <c r="D9" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="I9" s="7" t="n">
-        <v>46379</v>
-      </c>
+      <c r="I9" s="7"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5" t="s">
         <v>62</v>
@@ -5953,20 +5982,20 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D10" s="9"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="9" t="n">
+        <v>16.95</v>
+      </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="7" t="n">
@@ -5984,22 +6013,20 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="5" t="s">
-        <v>99</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="9" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E11" s="5"/>
       <c r="F11" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="7" t="n">
@@ -6019,20 +6046,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>108</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="C12" s="5"/>
       <c r="D12" s="9"/>
       <c r="E12" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="7" t="n">
@@ -6052,18 +6077,20 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D13" s="9"/>
+      <c r="E13" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="7" t="n">
@@ -6083,18 +6110,20 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="7" t="n">
@@ -6112,20 +6141,20 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>116</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="7" t="n">
@@ -6145,24 +6174,28 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>14.95</v>
-      </c>
-      <c r="E16" s="5"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="F16" s="5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
+      <c r="H16" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5" t="s">
         <v>62</v>
@@ -6174,24 +6207,28 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="9"/>
+      <c r="E17" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D17" s="9" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G17" s="5"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+      <c r="H17" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5" t="s">
         <v>62</v>
@@ -6203,24 +6240,26 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>13.95</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="D18" s="9"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
+      <c r="H18" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J18" s="5"/>
       <c r="K18" s="5" t="s">
         <v>62</v>
@@ -6232,24 +6271,26 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>13.95</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="D19" s="9"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
+      <c r="H19" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="s">
         <v>62</v>
@@ -6261,22 +6302,26 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="9" t="n">
-        <v>11.95</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="9"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G20" s="5"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
+      <c r="H20" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>46379</v>
+      </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5" t="s">
         <v>62</v>
@@ -6286,24 +6331,22 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>109</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="E21" s="5"/>
       <c r="F21" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="7"/>
@@ -6317,24 +6360,22 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>13.95</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>109</v>
-      </c>
+      <c r="E22" s="5"/>
       <c r="F22" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="7"/>
@@ -6350,16 +6391,20 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" s="5"/>
+        <v>113</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="C23" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="D23" s="9"/>
+      <c r="D23" s="9" t="n">
+        <v>13.95</v>
+      </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="7"/>
@@ -6375,18 +6420,20 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="D24" s="9" t="n">
         <v>13.95</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -6402,18 +6449,18 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="9" t="n">
-        <v>14.95</v>
+        <v>11.95</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="7"/>
@@ -6429,18 +6476,22 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" s="5"/>
+        <v>137</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="D26" s="9" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="E26" s="5"/>
+        <v>10.95</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>120</v>
+      </c>
       <c r="F26" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G26" s="5"/>
       <c r="H26" s="7"/>
@@ -6454,20 +6505,24 @@
         <v>Showing</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C27" s="5"/>
+        <v>139</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>140</v>
+      </c>
       <c r="D27" s="9" t="n">
-        <v>15.95</v>
-      </c>
-      <c r="E27" s="5"/>
+        <v>13.95</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>120</v>
+      </c>
       <c r="F27" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="7"/>
@@ -6483,20 +6538,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>137</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="B28" s="5"/>
       <c r="C28" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <v>16.95</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="D28" s="9"/>
       <c r="E28" s="5"/>
       <c r="F28" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="7"/>
@@ -6512,18 +6563,18 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="9" t="n">
-        <v>5.95</v>
+        <v>13.95</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="7"/>
@@ -6539,18 +6590,18 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="9" t="n">
-        <v>5.95</v>
+        <v>14.95</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="7"/>
@@ -6566,18 +6617,18 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="9" t="n">
-        <v>5.95</v>
+        <v>14.5</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="7"/>
@@ -6593,16 +6644,18 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>72</v>
+        <v>141</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C32" s="5"/>
-      <c r="D32" s="9"/>
+      <c r="D32" s="9" t="n">
+        <v>15.95</v>
+      </c>
       <c r="E32" s="5"/>
       <c r="F32" s="5" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="7"/>
@@ -6618,16 +6671,20 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>72</v>
+        <v>141</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="9"/>
+        <v>147</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>16.95</v>
+      </c>
       <c r="E33" s="5"/>
       <c r="F33" s="5" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="G33" s="5"/>
       <c r="H33" s="7"/>
@@ -6643,16 +6700,18 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>72</v>
+        <v>149</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C34" s="5"/>
-      <c r="D34" s="9"/>
+      <c r="D34" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E34" s="5"/>
       <c r="F34" s="5" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="7"/>
@@ -6668,18 +6727,18 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>72</v>
+        <v>149</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C35" s="5"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="5" t="s">
-        <v>109</v>
-      </c>
+      <c r="D35" s="9" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="E35" s="5"/>
       <c r="F35" s="5" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="7"/>
@@ -6694,122 +6753,192 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
+      <c r="A36" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>152</v>
+      </c>
       <c r="C36" s="5"/>
-      <c r="D36" s="9"/>
+      <c r="D36" s="9" t="n">
+        <v>5.95</v>
+      </c>
       <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
+      <c r="F36" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="G36" s="5"/>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L36" s="8" t="str">
         <f aca="true">IF(B36&amp;C36="","",IF(K36="Hidden","Hidden",IF(AND(H36&lt;&gt;"",H36&gt;TODAY()),"Scheduled",IF(AND(I36&lt;&gt;"",I36&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
+        <v>Showing</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>124</v>
+      </c>
       <c r="C37" s="5"/>
-      <c r="D37" s="9"/>
+      <c r="D37" s="9" t="n">
+        <v>6.95</v>
+      </c>
       <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
+      <c r="F37" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="G37" s="5"/>
-      <c r="H37" s="7"/>
+      <c r="H37" s="7" t="n">
+        <v>46305</v>
+      </c>
       <c r="I37" s="7"/>
       <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
+      <c r="K37" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L37" s="8" t="str">
         <f aca="true">IF(B37&amp;C37="","",IF(K37="Hidden","Hidden",IF(AND(H37&lt;&gt;"",H37&gt;TODAY()),"Scheduled",IF(AND(I37&lt;&gt;"",I37&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="9"/>
+        <v>Showing</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>6.95</v>
+      </c>
       <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
+      <c r="F38" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="G38" s="5"/>
-      <c r="H38" s="7"/>
+      <c r="H38" s="7" t="n">
+        <v>46305</v>
+      </c>
       <c r="I38" s="7"/>
       <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
+      <c r="K38" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L38" s="8" t="str">
         <f aca="true">IF(B38&amp;C38="","",IF(K38="Hidden","Hidden",IF(AND(H38&lt;&gt;"",H38&gt;TODAY()),"Scheduled",IF(AND(I38&lt;&gt;"",I38&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
+      <c r="A39" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>156</v>
+      </c>
       <c r="C39" s="5"/>
       <c r="D39" s="9"/>
       <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
+      <c r="F39" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="G39" s="5"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
+      <c r="K39" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L39" s="8" t="str">
         <f aca="true">IF(B39&amp;C39="","",IF(K39="Hidden","Hidden",IF(AND(H39&lt;&gt;"",H39&gt;TODAY()),"Scheduled",IF(AND(I39&lt;&gt;"",I39&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
+      <c r="A40" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>158</v>
+      </c>
       <c r="C40" s="5"/>
       <c r="D40" s="9"/>
       <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
+      <c r="F40" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="G40" s="5"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
       <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L40" s="8" t="str">
         <f aca="true">IF(B40&amp;C40="","",IF(K40="Hidden","Hidden",IF(AND(H40&lt;&gt;"",H40&gt;TODAY()),"Scheduled",IF(AND(I40&lt;&gt;"",I40&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>159</v>
+      </c>
       <c r="C41" s="5"/>
       <c r="D41" s="9"/>
       <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
+      <c r="F41" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="G41" s="5"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
       <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
+      <c r="K41" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L41" s="8" t="str">
         <f aca="true">IF(B41&amp;C41="","",IF(K41="Hidden","Hidden",IF(AND(H41&lt;&gt;"",H41&gt;TODAY()),"Scheduled",IF(AND(I41&lt;&gt;"",I41&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
+      <c r="A42" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="C42" s="5"/>
       <c r="D42" s="9"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
+      <c r="E42" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="G42" s="5"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
+      <c r="K42" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="L42" s="8" t="str">
         <f aca="true">IF(B42&amp;C42="","",IF(K42="Hidden","Hidden",IF(AND(H42&lt;&gt;"",H42&gt;TODAY()),"Scheduled",IF(AND(I42&lt;&gt;"",I42&lt;TODAY()),"Expired","Showing"))))</f>
-        <v/>
+        <v>Showing</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9511,20 +9640,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
+    <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K200" type="list">
+      <formula1>"Live,Sold out,Hidden"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Enter a real date, for example 31/12/2026." errorStyle="stop" errorTitle="Date" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:I200" type="date">
       <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F200" type="list">
+      <formula1>"Board,Sunday"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G200" type="list">
       <formula1>"Yes"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Choose one of the listed statuses." errorStyle="stop" errorTitle="Status" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K200" type="list">
-      <formula1>"Live,Sold out,Hidden"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F200" type="list">
-      <formula1>"Board,Sunday"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -9559,37 +9688,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>46</v>
@@ -9603,13 +9732,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -9630,13 +9759,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -9657,13 +9786,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -9684,13 +9813,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -9711,13 +9840,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -9738,10 +9867,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="9"/>
@@ -9763,13 +9892,13 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -9790,13 +9919,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -9817,13 +9946,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -9844,13 +9973,13 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -9871,13 +10000,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -9898,13 +10027,13 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -9925,13 +10054,13 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -9952,13 +10081,13 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -9979,13 +10108,13 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -10006,10 +10135,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="9"/>
@@ -10031,10 +10160,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="9"/>
@@ -10056,10 +10185,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="9"/>
@@ -13567,13 +13696,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>58</v>
@@ -13584,14 +13713,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="C2" s="7" t="n">
         <v>46305</v>
       </c>
+      <c r="C2" s="7"/>
       <c r="D2" s="5" t="s">
         <v>62</v>
       </c>
@@ -13602,7 +13729,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -15643,37 +15770,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>58</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>59</v>
@@ -15681,28 +15808,28 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46326</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="5" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="5" t="s">
         <v>62</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="K2" s="5"/>
       <c r="L2" s="8" t="str">
@@ -15712,7 +15839,7 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>46357</v>
@@ -15722,11 +15849,11 @@
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>46305</v>
@@ -15735,10 +15862,10 @@
         <v>62</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L3" s="8" t="str">
         <f aca="true">IF(A3="","",IF(I3="Hidden","Hidden",IF(AND(H3&lt;&gt;"",H3&gt;TODAY()),"Scheduled",IF(IF(C3&lt;&gt;"",C3,B3)&lt;TODAY(),"Expired","Showing"))))</f>
@@ -15747,7 +15874,7 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>46387</v>
@@ -15755,11 +15882,11 @@
       <c r="C4" s="7"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46304</v>
@@ -15768,7 +15895,7 @@
         <v>62</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="K4" s="5"/>
       <c r="L4" s="8" t="str">
@@ -15778,27 +15905,27 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>46564</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="5" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>46508</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
@@ -15809,29 +15936,29 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>46592</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="5" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>61</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>46553</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
@@ -19195,28 +19322,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>58</v>
@@ -19227,22 +19354,22 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>46508</v>
@@ -19251,7 +19378,7 @@
         <v>46538</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J2" s="8" t="str">
         <f aca="true">IF(B2="","",IF(I2="Hidden","Hidden",IF(AND(G2&lt;&gt;"",G2&gt;TODAY()),"Scheduled",IF(AND(H2&lt;&gt;"",H2&lt;TODAY()),"Expired","Showing"))))</f>
@@ -22283,37 +22410,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>58</v>
@@ -22324,27 +22451,27 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>6.5</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -22358,10 +22485,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>2</v>
@@ -22369,14 +22496,14 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -22390,10 +22517,10 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
@@ -22403,14 +22530,14 @@
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -22424,10 +22551,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>28.4</v>
@@ -22436,19 +22563,19 @@
         <v>2600</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -22462,10 +22589,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>20.3</v>
@@ -22474,19 +22601,19 @@
         <v>850</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>

</xml_diff>